<commit_message>
DM vor EM nach QB
</commit_message>
<xml_diff>
--- a/Turnierplanung.xlsx
+++ b/Turnierplanung.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="109">
   <si>
     <t>Wochenende (KW)</t>
   </si>
@@ -35,7 +35,7 @@
     <t>U15</t>
   </si>
   <si>
-    <t>U14</t>
+    <t>U13</t>
   </si>
   <si>
     <t>KW 35
@@ -66,7 +66,7 @@
   </si>
   <si>
     <t>EFC - EFC_Dublin (EFC)
-Leverkusen - QB_SEN_1 (QB)</t>
+DM - DM_Finals (DM)</t>
   </si>
   <si>
     <t>Leverkusen - CHALLENGE_U15_11 (CHALLENGE)</t>
@@ -97,7 +97,7 @@
   </si>
   <si>
     <t>EFC - EFC_Differdange (EFC)
-Reutlingen - QB_SEN_2 (QB)</t>
+Leverkusen - QB_SEN_1 (QB)</t>
   </si>
   <si>
     <t>Frankfurt - CHALLENGE_U15_14 (CHALLENGE)</t>
@@ -107,10 +107,11 @@
 2026-10-10</t>
   </si>
   <si>
-    <t>EFC - EFC_Daugavpils (EFC)</t>
-  </si>
-  <si>
-    <t>Leverkusen - QB_U17_3 (QB)</t>
+    <t>EFC - EFC_Daugavpils (EFC)
+Reutlingen - QB_SEN_2 (QB)</t>
+  </si>
+  <si>
+    <t>Waldkirch - CHALLENGE_U15_15 (CHALLENGE)</t>
   </si>
   <si>
     <t>KW 42
@@ -120,7 +121,7 @@
     <t>EFC - EFC_Zagreb (EFC)</t>
   </si>
   <si>
-    <t>Heidenheim - QB_U17_4 (QB)</t>
+    <t>Leverkusen - QB_U17_3 (QB)</t>
   </si>
   <si>
     <t>KW 43
@@ -130,7 +131,7 @@
     <t>EFC - EFC_Kamnik (EFC)</t>
   </si>
   <si>
-    <t>Leipzig - QB_U17_5 (QB)</t>
+    <t>Heidenheim - QB_U17_4 (QB)</t>
   </si>
   <si>
     <t>KW 44
@@ -140,7 +141,7 @@
     <t>FIE - FIE_SanSalvador (FIE)</t>
   </si>
   <si>
-    <t>Solingen - QB_U17_6 (QB)</t>
+    <t>Leipzig - QB_U17_5 (QB)</t>
   </si>
   <si>
     <t>KW 45
@@ -150,10 +151,7 @@
     <t>EFC - EFC_Brindisi (EFC)</t>
   </si>
   <si>
-    <t>Offenbach - QB_U20_7 (QB)</t>
-  </si>
-  <si>
-    <t>Waldkirch - CHALLENGE_U15_15 (CHALLENGE)</t>
+    <t>Solingen - QB_U17_6 (QB)</t>
   </si>
   <si>
     <t>KW 46
@@ -161,7 +159,7 @@
   </si>
   <si>
     <t>FIE - FIE_SanJose (FIE)
-Heidelberg - QB_U20_8 (QB)</t>
+Offenbach - QB_U20_7 (QB)</t>
   </si>
   <si>
     <t>Osnabrück - CHALLENGE_U15_16 (CHALLENGE)</t>
@@ -171,7 +169,7 @@
 2026-11-21</t>
   </si>
   <si>
-    <t>Leverkusen - QB_U20_9 (QB)</t>
+    <t>Heidelberg - QB_U20_8 (QB)</t>
   </si>
   <si>
     <t>KW 48
@@ -179,7 +177,7 @@
   </si>
   <si>
     <t>FIE - FIE_Hongkong (FIE)
-Osnabrück - QB_U20_10 (QB)</t>
+Leverkusen - QB_U20_9 (QB)</t>
   </si>
   <si>
     <t>KW 49
@@ -189,7 +187,7 @@
     <t>FIE - FIE_Vancouver (FIE)</t>
   </si>
   <si>
-    <t>Rüsselsheim - DM_U17_18 (DM)</t>
+    <t>Osnabrück - QB_U20_10 (QB)</t>
   </si>
   <si>
     <t>KW 50
@@ -199,7 +197,7 @@
     <t>FIE - FIE_Tashkent (FIE)</t>
   </si>
   <si>
-    <t>Leverkusen - DM_U17_19 (DM)</t>
+    <t>Rüsselsheim - DM_U17_18 (DM)</t>
   </si>
   <si>
     <t>KW 51
@@ -209,13 +207,20 @@
     <t>EFC - EFC_Lausanne (EFC)</t>
   </si>
   <si>
-    <t>Leverkusen - DM_U20_20 (DM)</t>
+    <t>Leverkusen - DM_U17_19 (DM)</t>
   </si>
   <si>
     <t>KW 52
 2026-12-26</t>
   </si>
   <si>
+    <t>Leverkusen - DM_U20_20 (DM)</t>
+  </si>
+  <si>
+    <t>KW 53
+2027-01-02</t>
+  </si>
+  <si>
     <t>Rüsselsheim - DM_U20_21 (DM)</t>
   </si>
   <si>
@@ -350,6 +355,37 @@
   </si>
   <si>
     <t>FIE - FIE_Bern (FIE)</t>
+  </si>
+  <si>
+    <t>KW 22
+2027-06-05</t>
+  </si>
+  <si>
+    <t>EFC - EFC_EM_Senioren (EFC)</t>
+  </si>
+  <si>
+    <t>KW 23
+2027-06-12</t>
+  </si>
+  <si>
+    <t>EFC - EFC_EM_U20 (EFC)</t>
+  </si>
+  <si>
+    <t>EFC - EFC_EM_U17 (EFC)</t>
+  </si>
+  <si>
+    <t>KW 24
+2027-06-19</t>
+  </si>
+  <si>
+    <t>FIE - FIE_WM_Senioren (FIE)</t>
+  </si>
+  <si>
+    <t>KW 25
+2027-06-26</t>
+  </si>
+  <si>
+    <t>FIE - FIE_WM_U20 (FIE)</t>
   </si>
 </sst>
 </file>
@@ -357,7 +393,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="39">
+  <fonts count="44">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
@@ -370,6 +406,31 @@
       <sz val="11.0"/>
       <b val="true"/>
       <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -645,7 +706,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="352">
+  <cellXfs count="397">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="true" applyFill="true" applyAlignment="true" applyBorder="true">
       <alignment horizontal="center" vertical="center"/>
@@ -983,9 +1044,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
@@ -1193,10 +1251,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1220,16 +1278,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1247,16 +1305,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1274,16 +1332,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1301,16 +1359,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1328,13 +1386,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1436,13 +1494,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1463,19 +1521,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1490,19 +1548,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1517,19 +1575,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1625,19 +1683,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1652,19 +1710,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1679,16 +1737,154 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
+      <alignment horizontal="center" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
+      <alignment horizontal="center" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
+      <alignment horizontal="center" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
+      <alignment horizontal="center" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
+      <alignment horizontal="center" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1706,7 +1902,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="25.0" customWidth="true"/>
@@ -1853,10 +2049,10 @@
       </c>
       <c r="D8" s="67"/>
       <c r="E8" s="68"/>
-      <c r="F8" t="s" s="70">
+      <c r="F8" s="69"/>
+      <c r="G8" t="s" s="71">
         <v>29</v>
       </c>
-      <c r="G8" s="71"/>
       <c r="H8" s="72"/>
     </row>
     <row r="9" ht="40.0" customHeight="true">
@@ -1916,386 +2112,456 @@
       <c r="D12" t="s" s="107">
         <v>40</v>
       </c>
-      <c r="E12" t="s" s="109">
+      <c r="E12" s="108"/>
+      <c r="F12" t="s" s="110">
         <v>41</v>
       </c>
-      <c r="F12" s="110"/>
-      <c r="G12" t="s" s="112">
+      <c r="G12" s="111"/>
+      <c r="H12" s="112"/>
+    </row>
+    <row r="13" ht="40.0" customHeight="true">
+      <c r="A13" t="s" s="113">
         <v>42</v>
       </c>
-      <c r="H12" s="113"/>
-    </row>
-    <row r="13" ht="40.0" customHeight="true">
-      <c r="A13" t="s" s="114">
+      <c r="B13" s="114"/>
+      <c r="C13" s="115"/>
+      <c r="D13" s="116"/>
+      <c r="E13" t="s" s="118">
         <v>43</v>
       </c>
-      <c r="B13" s="115"/>
-      <c r="C13" s="116"/>
-      <c r="D13" s="117"/>
-      <c r="E13" t="s" s="119">
+      <c r="F13" s="119"/>
+      <c r="G13" t="s" s="121">
         <v>44</v>
       </c>
-      <c r="F13" s="120"/>
-      <c r="G13" t="s" s="122">
+      <c r="H13" s="122"/>
+    </row>
+    <row r="14" ht="40.0" customHeight="true">
+      <c r="A14" t="s" s="123">
         <v>45</v>
       </c>
-      <c r="H13" s="123"/>
-    </row>
-    <row r="14" ht="40.0" customHeight="true">
-      <c r="A14" t="s" s="124">
+      <c r="B14" s="124"/>
+      <c r="C14" s="125"/>
+      <c r="D14" s="126"/>
+      <c r="E14" t="s" s="128">
         <v>46</v>
       </c>
-      <c r="B14" s="125"/>
-      <c r="C14" s="126"/>
-      <c r="D14" s="127"/>
-      <c r="E14" t="s" s="129">
+      <c r="F14" s="129"/>
+      <c r="G14" s="130"/>
+      <c r="H14" s="131"/>
+    </row>
+    <row r="15" ht="40.0" customHeight="true">
+      <c r="A15" t="s" s="132">
         <v>47</v>
       </c>
-      <c r="F14" s="130"/>
-      <c r="G14" s="131"/>
-      <c r="H14" s="132"/>
-    </row>
-    <row r="15" ht="40.0" customHeight="true">
-      <c r="A15" t="s" s="133">
+      <c r="B15" s="133"/>
+      <c r="C15" s="134"/>
+      <c r="D15" s="135"/>
+      <c r="E15" t="s" s="137">
         <v>48</v>
       </c>
-      <c r="B15" s="134"/>
-      <c r="C15" s="135"/>
-      <c r="D15" s="136"/>
-      <c r="E15" t="s" s="138">
+      <c r="F15" s="138"/>
+      <c r="G15" s="139"/>
+      <c r="H15" s="140"/>
+    </row>
+    <row r="16" ht="40.0" customHeight="true">
+      <c r="A16" t="s" s="141">
         <v>49</v>
       </c>
-      <c r="F15" s="139"/>
-      <c r="G15" s="140"/>
-      <c r="H15" s="141"/>
-    </row>
-    <row r="16" ht="40.0" customHeight="true">
-      <c r="A16" t="s" s="142">
+      <c r="B16" s="142"/>
+      <c r="C16" t="s" s="144">
         <v>50</v>
       </c>
-      <c r="B16" s="143"/>
-      <c r="C16" t="s" s="145">
+      <c r="D16" s="145"/>
+      <c r="E16" t="s" s="147">
         <v>51</v>
       </c>
-      <c r="D16" s="146"/>
-      <c r="E16" s="147"/>
-      <c r="F16" t="s" s="149">
+      <c r="F16" s="148"/>
+      <c r="G16" s="149"/>
+      <c r="H16" s="150"/>
+    </row>
+    <row r="17" ht="40.0" customHeight="true">
+      <c r="A17" t="s" s="151">
         <v>52</v>
       </c>
-      <c r="G16" s="150"/>
-      <c r="H16" s="151"/>
-    </row>
-    <row r="17" ht="40.0" customHeight="true">
-      <c r="A17" t="s" s="152">
+      <c r="B17" s="152"/>
+      <c r="C17" s="153"/>
+      <c r="D17" s="154"/>
+      <c r="E17" t="s" s="156">
         <v>53</v>
       </c>
-      <c r="B17" s="153"/>
-      <c r="C17" s="154"/>
-      <c r="D17" s="155"/>
-      <c r="E17" t="s" s="157">
+      <c r="F17" t="s" s="158">
         <v>54</v>
       </c>
-      <c r="F17" t="s" s="159">
+      <c r="G17" s="159"/>
+      <c r="H17" s="160"/>
+    </row>
+    <row r="18" ht="40.0" customHeight="true">
+      <c r="A18" t="s" s="161">
         <v>55</v>
       </c>
-      <c r="G17" s="160"/>
-      <c r="H17" s="161"/>
-    </row>
-    <row r="18" ht="40.0" customHeight="true">
-      <c r="A18" t="s" s="162">
+      <c r="B18" s="162"/>
+      <c r="C18" s="163"/>
+      <c r="D18" t="s" s="165">
         <v>56</v>
       </c>
-      <c r="B18" s="163"/>
-      <c r="C18" s="164"/>
-      <c r="D18" t="s" s="166">
+      <c r="E18" s="166"/>
+      <c r="F18" t="s" s="168">
         <v>57</v>
       </c>
-      <c r="E18" t="s" s="168">
+      <c r="G18" s="169"/>
+      <c r="H18" s="170"/>
+    </row>
+    <row r="19" ht="40.0" customHeight="true">
+      <c r="A19" t="s" s="171">
         <v>58</v>
       </c>
-      <c r="F18" s="169"/>
-      <c r="G18" s="170"/>
-      <c r="H18" s="171"/>
-    </row>
-    <row r="19" ht="40.0" customHeight="true">
-      <c r="A19" t="s" s="172">
+      <c r="B19" s="172"/>
+      <c r="C19" s="173"/>
+      <c r="D19" s="174"/>
+      <c r="E19" t="s" s="176">
         <v>59</v>
       </c>
-      <c r="B19" s="173"/>
-      <c r="C19" s="174"/>
-      <c r="D19" s="175"/>
-      <c r="E19" t="s" s="177">
+      <c r="F19" s="177"/>
+      <c r="G19" s="178"/>
+      <c r="H19" s="179"/>
+    </row>
+    <row r="20" ht="40.0" customHeight="true">
+      <c r="A20" t="s" s="180">
         <v>60</v>
       </c>
-      <c r="F19" s="178"/>
-      <c r="G19" s="179"/>
-      <c r="H19" s="180"/>
-    </row>
-    <row r="20" ht="40.0" customHeight="true">
-      <c r="A20" t="s" s="181">
+      <c r="B20" s="181"/>
+      <c r="C20" s="182"/>
+      <c r="D20" s="183"/>
+      <c r="E20" t="s" s="185">
         <v>61</v>
       </c>
-      <c r="B20" s="182"/>
-      <c r="C20" t="s" s="184">
+      <c r="F20" s="186"/>
+      <c r="G20" s="187"/>
+      <c r="H20" s="188"/>
+    </row>
+    <row r="21" ht="40.0" customHeight="true">
+      <c r="A21" t="s" s="189">
         <v>62</v>
       </c>
-      <c r="D20" s="185"/>
-      <c r="E20" s="186"/>
-      <c r="F20" s="187"/>
-      <c r="G20" s="188"/>
-      <c r="H20" s="189"/>
-    </row>
-    <row r="21" ht="40.0" customHeight="true">
-      <c r="A21" t="s" s="190">
+      <c r="B21" s="190"/>
+      <c r="C21" t="s" s="192">
         <v>63</v>
       </c>
-      <c r="B21" s="191"/>
-      <c r="C21" s="192"/>
       <c r="D21" s="193"/>
-      <c r="E21" t="s" s="195">
+      <c r="E21" s="194"/>
+      <c r="F21" s="195"/>
+      <c r="G21" s="196"/>
+      <c r="H21" s="197"/>
+    </row>
+    <row r="22" ht="40.0" customHeight="true">
+      <c r="A22" t="s" s="198">
         <v>64</v>
       </c>
-      <c r="F21" s="196"/>
-      <c r="G21" s="197"/>
-      <c r="H21" s="198"/>
-    </row>
-    <row r="22" ht="40.0" customHeight="true">
-      <c r="A22" t="s" s="199">
+      <c r="B22" s="199"/>
+      <c r="C22" s="200"/>
+      <c r="D22" s="201"/>
+      <c r="E22" t="s" s="203">
         <v>65</v>
       </c>
-      <c r="B22" s="200"/>
-      <c r="C22" t="s" s="202">
+      <c r="F22" s="204"/>
+      <c r="G22" s="205"/>
+      <c r="H22" s="206"/>
+    </row>
+    <row r="23" ht="40.0" customHeight="true">
+      <c r="A23" t="s" s="207">
         <v>66</v>
       </c>
-      <c r="D22" s="203"/>
-      <c r="E22" s="204"/>
-      <c r="F22" s="205"/>
-      <c r="G22" s="206"/>
-      <c r="H22" s="207"/>
-    </row>
-    <row r="23" ht="40.0" customHeight="true">
-      <c r="A23" t="s" s="208">
+      <c r="B23" s="208"/>
+      <c r="C23" t="s" s="210">
         <v>67</v>
       </c>
-      <c r="B23" s="209"/>
-      <c r="C23" s="210"/>
       <c r="D23" s="211"/>
-      <c r="E23" t="s" s="213">
+      <c r="E23" s="212"/>
+      <c r="F23" s="213"/>
+      <c r="G23" s="214"/>
+      <c r="H23" s="215"/>
+    </row>
+    <row r="24" ht="40.0" customHeight="true">
+      <c r="A24" t="s" s="216">
         <v>68</v>
       </c>
-      <c r="F23" s="214"/>
-      <c r="G23" s="215"/>
-      <c r="H23" s="216"/>
-    </row>
-    <row r="24" ht="40.0" customHeight="true">
-      <c r="A24" t="s" s="217">
+      <c r="B24" s="217"/>
+      <c r="C24" s="218"/>
+      <c r="D24" s="219"/>
+      <c r="E24" t="s" s="221">
         <v>69</v>
       </c>
-      <c r="B24" s="218"/>
-      <c r="C24" t="s" s="220">
+      <c r="F24" s="222"/>
+      <c r="G24" s="223"/>
+      <c r="H24" s="224"/>
+    </row>
+    <row r="25" ht="40.0" customHeight="true">
+      <c r="A25" t="s" s="225">
         <v>70</v>
       </c>
-      <c r="D24" s="221"/>
-      <c r="E24" s="222"/>
-      <c r="F24" s="223"/>
-      <c r="G24" s="224"/>
-      <c r="H24" s="225"/>
-    </row>
-    <row r="25" ht="40.0" customHeight="true">
-      <c r="A25" t="s" s="226">
+      <c r="B25" s="226"/>
+      <c r="C25" t="s" s="228">
         <v>71</v>
       </c>
-      <c r="B25" s="227"/>
-      <c r="C25" s="228"/>
-      <c r="D25" t="s" s="230">
+      <c r="D25" s="229"/>
+      <c r="E25" s="230"/>
+      <c r="F25" s="231"/>
+      <c r="G25" s="232"/>
+      <c r="H25" s="233"/>
+    </row>
+    <row r="26" ht="40.0" customHeight="true">
+      <c r="A26" t="s" s="234">
         <v>72</v>
       </c>
-      <c r="E25" s="231"/>
-      <c r="F25" s="232"/>
-      <c r="G25" s="233"/>
-      <c r="H25" s="234"/>
-    </row>
-    <row r="26" ht="40.0" customHeight="true">
-      <c r="A26" t="s" s="235">
+      <c r="B26" s="235"/>
+      <c r="C26" s="236"/>
+      <c r="D26" t="s" s="238">
         <v>73</v>
       </c>
-      <c r="B26" s="236"/>
-      <c r="C26" s="237"/>
-      <c r="D26" t="s" s="239">
+      <c r="E26" s="239"/>
+      <c r="F26" s="240"/>
+      <c r="G26" s="241"/>
+      <c r="H26" s="242"/>
+    </row>
+    <row r="27" ht="40.0" customHeight="true">
+      <c r="A27" t="s" s="243">
         <v>74</v>
       </c>
-      <c r="E26" s="240"/>
-      <c r="F26" s="241"/>
-      <c r="G26" s="242"/>
-      <c r="H26" s="243"/>
-    </row>
-    <row r="27" ht="40.0" customHeight="true">
-      <c r="A27" t="s" s="244">
+      <c r="B27" s="244"/>
+      <c r="C27" s="245"/>
+      <c r="D27" t="s" s="247">
         <v>75</v>
       </c>
-      <c r="B27" s="245"/>
-      <c r="C27" s="246"/>
-      <c r="D27" t="s" s="248">
+      <c r="E27" s="248"/>
+      <c r="F27" s="249"/>
+      <c r="G27" s="250"/>
+      <c r="H27" s="251"/>
+    </row>
+    <row r="28" ht="40.0" customHeight="true">
+      <c r="A28" t="s" s="252">
         <v>76</v>
       </c>
-      <c r="E27" s="249"/>
-      <c r="F27" s="250"/>
-      <c r="G27" s="251"/>
-      <c r="H27" s="252"/>
-    </row>
-    <row r="28" ht="40.0" customHeight="true">
-      <c r="A28" t="s" s="253">
+      <c r="B28" s="253"/>
+      <c r="C28" s="254"/>
+      <c r="D28" t="s" s="256">
         <v>77</v>
       </c>
-      <c r="B28" s="254"/>
-      <c r="C28" s="255"/>
-      <c r="D28" t="s" s="257">
+      <c r="E28" s="257"/>
+      <c r="F28" s="258"/>
+      <c r="G28" s="259"/>
+      <c r="H28" s="260"/>
+    </row>
+    <row r="29" ht="40.0" customHeight="true">
+      <c r="A29" t="s" s="261">
         <v>78</v>
       </c>
-      <c r="E28" s="258"/>
-      <c r="F28" s="259"/>
-      <c r="G28" s="260"/>
-      <c r="H28" s="261"/>
-    </row>
-    <row r="29" ht="40.0" customHeight="true">
-      <c r="A29" t="s" s="262">
+      <c r="B29" s="262"/>
+      <c r="C29" s="263"/>
+      <c r="D29" t="s" s="265">
         <v>79</v>
       </c>
-      <c r="B29" s="263"/>
-      <c r="C29" t="s" s="265">
+      <c r="E29" s="266"/>
+      <c r="F29" s="267"/>
+      <c r="G29" s="268"/>
+      <c r="H29" s="269"/>
+    </row>
+    <row r="30" ht="40.0" customHeight="true">
+      <c r="A30" t="s" s="270">
         <v>80</v>
       </c>
-      <c r="D29" s="266"/>
-      <c r="E29" s="267"/>
-      <c r="F29" s="268"/>
-      <c r="G29" s="269"/>
-      <c r="H29" s="270"/>
-    </row>
-    <row r="30" ht="40.0" customHeight="true">
-      <c r="A30" t="s" s="271">
+      <c r="B30" s="271"/>
+      <c r="C30" t="s" s="273">
         <v>81</v>
       </c>
-      <c r="B30" s="272"/>
-      <c r="C30" s="273"/>
       <c r="D30" s="274"/>
       <c r="E30" s="275"/>
-      <c r="F30" t="s" s="277">
+      <c r="F30" s="276"/>
+      <c r="G30" s="277"/>
+      <c r="H30" s="278"/>
+    </row>
+    <row r="31" ht="40.0" customHeight="true">
+      <c r="A31" t="s" s="279">
         <v>82</v>
       </c>
-      <c r="G30" s="278"/>
-      <c r="H30" s="279"/>
-    </row>
-    <row r="31" ht="40.0" customHeight="true">
-      <c r="A31" t="s" s="280">
+      <c r="B31" s="280"/>
+      <c r="C31" s="281"/>
+      <c r="D31" s="282"/>
+      <c r="E31" s="283"/>
+      <c r="F31" t="s" s="285">
         <v>83</v>
       </c>
-      <c r="B31" s="281"/>
-      <c r="C31" t="s" s="283">
+      <c r="G31" s="286"/>
+      <c r="H31" s="287"/>
+    </row>
+    <row r="32" ht="40.0" customHeight="true">
+      <c r="A32" t="s" s="288">
         <v>84</v>
       </c>
-      <c r="D31" s="284"/>
-      <c r="E31" s="285"/>
-      <c r="F31" s="286"/>
-      <c r="G31" s="287"/>
-      <c r="H31" s="288"/>
-    </row>
-    <row r="32" ht="40.0" customHeight="true">
-      <c r="A32" t="s" s="289">
+      <c r="B32" s="289"/>
+      <c r="C32" t="s" s="291">
         <v>85</v>
       </c>
-      <c r="B32" s="290"/>
-      <c r="C32" s="291"/>
       <c r="D32" s="292"/>
       <c r="E32" s="293"/>
-      <c r="F32" t="s" s="295">
+      <c r="F32" s="294"/>
+      <c r="G32" s="295"/>
+      <c r="H32" s="296"/>
+    </row>
+    <row r="33" ht="40.0" customHeight="true">
+      <c r="A33" t="s" s="297">
         <v>86</v>
       </c>
-      <c r="G32" s="296"/>
-      <c r="H32" s="297"/>
-    </row>
-    <row r="33" ht="40.0" customHeight="true">
-      <c r="A33" t="s" s="298">
+      <c r="B33" s="298"/>
+      <c r="C33" s="299"/>
+      <c r="D33" s="300"/>
+      <c r="E33" s="301"/>
+      <c r="F33" t="s" s="303">
         <v>87</v>
       </c>
-      <c r="B33" s="299"/>
-      <c r="C33" s="300"/>
-      <c r="D33" s="301"/>
-      <c r="E33" s="302"/>
-      <c r="F33" t="s" s="304">
+      <c r="G33" s="304"/>
+      <c r="H33" s="305"/>
+    </row>
+    <row r="34" ht="40.0" customHeight="true">
+      <c r="A34" t="s" s="306">
         <v>88</v>
       </c>
-      <c r="G33" s="305"/>
-      <c r="H33" s="306"/>
-    </row>
-    <row r="34" ht="40.0" customHeight="true">
-      <c r="A34" t="s" s="307">
+      <c r="B34" s="307"/>
+      <c r="C34" s="308"/>
+      <c r="D34" s="309"/>
+      <c r="E34" s="310"/>
+      <c r="F34" t="s" s="312">
         <v>89</v>
       </c>
-      <c r="B34" s="308"/>
-      <c r="C34" s="309"/>
-      <c r="D34" s="310"/>
-      <c r="E34" s="311"/>
-      <c r="F34" t="s" s="313">
+      <c r="G34" s="313"/>
+      <c r="H34" s="314"/>
+    </row>
+    <row r="35" ht="40.0" customHeight="true">
+      <c r="A35" t="s" s="315">
         <v>90</v>
       </c>
-      <c r="G34" s="314"/>
-      <c r="H34" s="315"/>
-    </row>
-    <row r="35" ht="40.0" customHeight="true">
-      <c r="A35" t="s" s="316">
+      <c r="B35" s="316"/>
+      <c r="C35" s="317"/>
+      <c r="D35" s="318"/>
+      <c r="E35" s="319"/>
+      <c r="F35" t="s" s="321">
         <v>91</v>
       </c>
-      <c r="B35" s="317"/>
-      <c r="C35" s="318"/>
-      <c r="D35" s="319"/>
-      <c r="E35" s="320"/>
-      <c r="F35" t="s" s="322">
+      <c r="G35" s="322"/>
+      <c r="H35" s="323"/>
+    </row>
+    <row r="36" ht="40.0" customHeight="true">
+      <c r="A36" t="s" s="324">
         <v>92</v>
       </c>
-      <c r="G35" s="323"/>
-      <c r="H35" s="324"/>
-    </row>
-    <row r="36" ht="40.0" customHeight="true">
-      <c r="A36" t="s" s="325">
+      <c r="B36" s="325"/>
+      <c r="C36" s="326"/>
+      <c r="D36" s="327"/>
+      <c r="E36" s="328"/>
+      <c r="F36" t="s" s="330">
         <v>93</v>
       </c>
-      <c r="B36" s="326"/>
-      <c r="C36" t="s" s="328">
+      <c r="G36" s="331"/>
+      <c r="H36" s="332"/>
+    </row>
+    <row r="37" ht="40.0" customHeight="true">
+      <c r="A37" t="s" s="333">
         <v>94</v>
       </c>
-      <c r="D36" s="329"/>
-      <c r="E36" s="330"/>
-      <c r="F36" s="331"/>
-      <c r="G36" s="332"/>
-      <c r="H36" s="333"/>
-    </row>
-    <row r="37" ht="40.0" customHeight="true">
-      <c r="A37" t="s" s="334">
+      <c r="B37" s="334"/>
+      <c r="C37" t="s" s="336">
         <v>95</v>
       </c>
-      <c r="B37" s="335"/>
-      <c r="C37" s="336"/>
       <c r="D37" s="337"/>
       <c r="E37" s="338"/>
-      <c r="F37" t="s" s="340">
+      <c r="F37" s="339"/>
+      <c r="G37" s="340"/>
+      <c r="H37" s="341"/>
+    </row>
+    <row r="38" ht="40.0" customHeight="true">
+      <c r="A38" t="s" s="342">
         <v>96</v>
       </c>
-      <c r="G37" s="341"/>
-      <c r="H37" s="342"/>
-    </row>
-    <row r="38" ht="40.0" customHeight="true">
-      <c r="A38" t="s" s="343">
+      <c r="B38" s="343"/>
+      <c r="C38" s="344"/>
+      <c r="D38" s="345"/>
+      <c r="E38" s="346"/>
+      <c r="F38" t="s" s="348">
         <v>97</v>
       </c>
-      <c r="B38" s="344"/>
-      <c r="C38" t="s" s="346">
+      <c r="G38" s="349"/>
+      <c r="H38" s="350"/>
+    </row>
+    <row r="39" ht="40.0" customHeight="true">
+      <c r="A39" t="s" s="351">
         <v>98</v>
       </c>
-      <c r="D38" s="347"/>
-      <c r="E38" s="348"/>
-      <c r="F38" s="349"/>
-      <c r="G38" s="350"/>
-      <c r="H38" s="351"/>
+      <c r="B39" s="352"/>
+      <c r="C39" t="s" s="354">
+        <v>99</v>
+      </c>
+      <c r="D39" s="355"/>
+      <c r="E39" s="356"/>
+      <c r="F39" s="357"/>
+      <c r="G39" s="358"/>
+      <c r="H39" s="359"/>
+    </row>
+    <row r="40" ht="40.0" customHeight="true">
+      <c r="A40" t="s" s="360">
+        <v>100</v>
+      </c>
+      <c r="B40" s="361"/>
+      <c r="C40" t="s" s="363">
+        <v>101</v>
+      </c>
+      <c r="D40" s="364"/>
+      <c r="E40" s="365"/>
+      <c r="F40" s="366"/>
+      <c r="G40" s="367"/>
+      <c r="H40" s="368"/>
+    </row>
+    <row r="41" ht="40.0" customHeight="true">
+      <c r="A41" t="s" s="369">
+        <v>102</v>
+      </c>
+      <c r="B41" s="370"/>
+      <c r="C41" s="371"/>
+      <c r="D41" s="372"/>
+      <c r="E41" t="s" s="374">
+        <v>103</v>
+      </c>
+      <c r="F41" t="s" s="376">
+        <v>104</v>
+      </c>
+      <c r="G41" s="377"/>
+      <c r="H41" s="378"/>
+    </row>
+    <row r="42" ht="40.0" customHeight="true">
+      <c r="A42" t="s" s="379">
+        <v>105</v>
+      </c>
+      <c r="B42" s="380"/>
+      <c r="C42" t="s" s="382">
+        <v>106</v>
+      </c>
+      <c r="D42" s="383"/>
+      <c r="E42" s="384"/>
+      <c r="F42" s="385"/>
+      <c r="G42" s="386"/>
+      <c r="H42" s="387"/>
+    </row>
+    <row r="43" ht="40.0" customHeight="true">
+      <c r="A43" t="s" s="388">
+        <v>107</v>
+      </c>
+      <c r="B43" s="389"/>
+      <c r="C43" s="390"/>
+      <c r="D43" s="391"/>
+      <c r="E43" t="s" s="393">
+        <v>108</v>
+      </c>
+      <c r="F43" s="394"/>
+      <c r="G43" s="395"/>
+      <c r="H43" s="396"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
KOrrektur TERMine und bugfixing
</commit_message>
<xml_diff>
--- a/Turnierplanung.xlsx
+++ b/Turnierplanung.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="116">
   <si>
     <t>Wochenende (KW)</t>
   </si>
@@ -42,86 +42,259 @@
 2026-08-29</t>
   </si>
   <si>
-    <t>Erfurt - DM_VET_17 (DM)</t>
-  </si>
-  <si>
-    <t>FIE - FIE_Basel (FIE)</t>
-  </si>
-  <si>
-    <t>EFC - EFC_Krakow (EFC)</t>
+    <t>Leverkusen - QB_SEN_1 (QB)</t>
+  </si>
+  <si>
+    <t>Leverkusen - CHALLENGE_U15_11 (CHALLENGE)</t>
   </si>
   <si>
     <t>KW 36
 2026-09-05</t>
   </si>
   <si>
-    <t>FIE - FIE_WM_Senioren (FIE)</t>
-  </si>
-  <si>
-    <t>Leverkusen - CHALLENGE_U15_11 (CHALLENGE)</t>
+    <t>Reutlingen - QB_SEN_2 (QB)</t>
+  </si>
+  <si>
+    <t>Leipzig - CHALLENGE_U15_12 (CHALLENGE)</t>
   </si>
   <si>
     <t>KW 37
 2026-09-12</t>
   </si>
   <si>
-    <t>EFC - EFC_Dublin (EFC)</t>
-  </si>
-  <si>
-    <t>FIE - FIE_WM_U20 (FIE)</t>
-  </si>
-  <si>
-    <t>Osnabrück - CHALLENGE_U15_16 (CHALLENGE)</t>
+    <t>Erfurt - DM_VET_17 (DM)</t>
+  </si>
+  <si>
+    <t>Leverkusen - QB_U17_3 (QB)</t>
   </si>
   <si>
     <t>KW 38
 2026-09-19</t>
   </si>
   <si>
-    <t>EFC - EFC_Colmar (EFC)</t>
-  </si>
-  <si>
-    <t>Bonn - CHALLENGE_U15_13 (CHALLENGE)</t>
+    <t>Heidenheim - QB_U17_4 (QB)</t>
   </si>
   <si>
     <t>KW 39
 2026-09-26</t>
   </si>
   <si>
-    <t>EFC - EFC_Berlin (EFC)</t>
-  </si>
-  <si>
-    <t>Frankfurt - CHALLENGE_U15_14 (CHALLENGE)</t>
+    <t>Leipzig - QB_U17_5 (QB)</t>
   </si>
   <si>
     <t>KW 40
 2026-10-03</t>
   </si>
   <si>
-    <t>DM - DM_Finals (DM)</t>
-  </si>
-  <si>
-    <t>EFC - EFC_Oslo (EFC)</t>
-  </si>
-  <si>
-    <t>Waldkirch - CHALLENGE_U15_15 (CHALLENGE)</t>
+    <t>Solingen - QB_U17_6 (QB)</t>
   </si>
   <si>
     <t>KW 41
 2026-10-10</t>
   </si>
   <si>
-    <t>EFC - EFC_Daugavpils (EFC)
-Leverkusen - QB_SEN_1 (QB)</t>
-  </si>
-  <si>
-    <t>Leipzig - CHALLENGE_U15_12 (CHALLENGE)</t>
+    <t>Offenbach - QB_U20_7 (QB)</t>
+  </si>
+  <si>
+    <t>Bonn - CHALLENGE_U15_13 (CHALLENGE)</t>
   </si>
   <si>
     <t>KW 42
 2026-10-17</t>
   </si>
   <si>
+    <t>EFC - EFC_Napoli (EFC)</t>
+  </si>
+  <si>
+    <t>KW 43
+2026-10-24</t>
+  </si>
+  <si>
+    <t>EFC - EFC_Dublin (EFC)</t>
+  </si>
+  <si>
+    <t>EFC - EFC_Klagenfurt (EFC)</t>
+  </si>
+  <si>
+    <t>KW 44
+2026-10-31</t>
+  </si>
+  <si>
+    <t>FIE - FIE_SanSalvador (FIE)</t>
+  </si>
+  <si>
+    <t>Frankfurt - CHALLENGE_U15_14 (CHALLENGE)</t>
+  </si>
+  <si>
+    <t>KW 45
+2026-11-07</t>
+  </si>
+  <si>
+    <t>Heidelberg - QB_U20_8 (QB)</t>
+  </si>
+  <si>
+    <t>Waldkirch - CHALLENGE_U15_15 (CHALLENGE)</t>
+  </si>
+  <si>
+    <t>KW 46
+2026-11-14</t>
+  </si>
+  <si>
+    <t>EFC - EFC_Brindisi (EFC)</t>
+  </si>
+  <si>
+    <t>FIE - FIE_SanJose (FIE)</t>
+  </si>
+  <si>
+    <t>KW 47
+2026-11-21</t>
+  </si>
+  <si>
+    <t>EFC - EFC_Lausanne (EFC)</t>
+  </si>
+  <si>
+    <t>KW 48
+2026-11-28</t>
+  </si>
+  <si>
+    <t>EFC - EFC_Grenoble (EFC)</t>
+  </si>
+  <si>
+    <t>KW 49
+2026-12-05</t>
+  </si>
+  <si>
+    <t>FIE - FIE_Vancouver (FIE)</t>
+  </si>
+  <si>
+    <t>EFC - EFC_Oslo (EFC)</t>
+  </si>
+  <si>
+    <t>KW 50
+2026-12-12</t>
+  </si>
+  <si>
+    <t>EFC - EFC_Laupheim (EFC)</t>
+  </si>
+  <si>
+    <t>Osnabrück - CHALLENGE_U15_16 (CHALLENGE)</t>
+  </si>
+  <si>
+    <t>KW 51
+2026-12-19</t>
+  </si>
+  <si>
+    <t>EFC - EFC_Thessaloniki (EFC)</t>
+  </si>
+  <si>
+    <t>KW 53
+2027-01-02</t>
+  </si>
+  <si>
+    <t>FIE - FIE_Basel (FIE)</t>
+  </si>
+  <si>
+    <t>KW 1
+2027-01-09</t>
+  </si>
+  <si>
+    <t>FIE - FIE_Fujairah (FIE)</t>
+  </si>
+  <si>
+    <t>KW 2
+2027-01-16</t>
+  </si>
+  <si>
+    <t>EFC - EFC_Bratislava (EFC)</t>
+  </si>
+  <si>
+    <t>KW 3
+2027-01-23</t>
+  </si>
+  <si>
+    <t>FIE - FIE_Doha (FIE)</t>
+  </si>
+  <si>
+    <t>KW 4
+2027-01-30</t>
+  </si>
+  <si>
+    <t>FIE - FIE_Cairo (FIE)</t>
+  </si>
+  <si>
+    <t>EFC - EFC_Belgrade (EFC)</t>
+  </si>
+  <si>
+    <t>KW 5
+2027-02-06</t>
+  </si>
+  <si>
+    <t>FIE - FIE_Heidenheim (FIE)</t>
+  </si>
+  <si>
+    <t>KW 6
+2027-02-13</t>
+  </si>
+  <si>
+    <t>EFC - EFC_Krakow (EFC)</t>
+  </si>
+  <si>
+    <t>KW 7
+2027-02-20</t>
+  </si>
+  <si>
+    <t>EFC - EFC_Sofia (EFC)</t>
+  </si>
+  <si>
+    <t>FIE - FIE_Vrsac (FIE)</t>
+  </si>
+  <si>
+    <t>KW 8
+2027-02-27</t>
+  </si>
+  <si>
+    <t>Leverkusen - QB_U20_9 (QB)</t>
+  </si>
+  <si>
+    <t>KW 9
+2027-03-06</t>
+  </si>
+  <si>
+    <t>Osnabrück - QB_U20_10 (QB)</t>
+  </si>
+  <si>
+    <t>KW 10
+2027-03-13</t>
+  </si>
+  <si>
+    <t>FIE - FIE_Budapest (FIE)
+EFC - EFC_Differdange (EFC)</t>
+  </si>
+  <si>
+    <t>KW 11
+2027-03-20</t>
+  </si>
+  <si>
+    <t>Rüsselsheim - DM_U17_18 (DM)
+Leverkusen - DM_U17_20 (DM)</t>
+  </si>
+  <si>
+    <t>Rüsselsheim - DM_U13_19 (DM)
+Leverkusen - DM_U13_21 (DM)</t>
+  </si>
+  <si>
+    <t>KW 12
+2027-03-27</t>
+  </si>
+  <si>
+    <t>FIE - FIE_Astana (FIE)
+EFC - EFC_Daugavpils (EFC)</t>
+  </si>
+  <si>
+    <t>KW 13
+2027-04-03</t>
+  </si>
+  <si>
     <t>Leverkusen - DM_U20_22 (DM)
 Rüsselsheim - DM_U20_24 (DM)</t>
   </si>
@@ -130,198 +303,18 @@
 Rüsselsheim - DM_U15_25 (DM)</t>
   </si>
   <si>
-    <t>KW 43
-2026-10-24</t>
-  </si>
-  <si>
-    <t>EFC - EFC_Kamnik (EFC)</t>
-  </si>
-  <si>
-    <t>Leverkusen - QB_U17_3 (QB)</t>
-  </si>
-  <si>
-    <t>KW 44
-2026-10-31</t>
-  </si>
-  <si>
-    <t>FIE - FIE_SanSalvador (FIE)</t>
-  </si>
-  <si>
-    <t>Heidenheim - QB_U17_4 (QB)</t>
-  </si>
-  <si>
-    <t>KW 45
-2026-11-07</t>
-  </si>
-  <si>
-    <t>EFC - EFC_Klagenfurt (EFC)</t>
-  </si>
-  <si>
-    <t>KW 46
-2026-11-14</t>
-  </si>
-  <si>
-    <t>FIE - FIE_SanJose (FIE)</t>
-  </si>
-  <si>
-    <t>Solingen - QB_U17_6 (QB)</t>
-  </si>
-  <si>
-    <t>KW 47
-2026-11-21</t>
-  </si>
-  <si>
-    <t>Offenbach - QB_U20_7 (QB)</t>
-  </si>
-  <si>
-    <t>KW 48
-2026-11-28</t>
-  </si>
-  <si>
-    <t>FIE - FIE_Hongkong (FIE)
-Heidelberg - QB_U20_8 (QB)</t>
-  </si>
-  <si>
-    <t>KW 49
-2026-12-05</t>
-  </si>
-  <si>
-    <t>FIE - FIE_Vancouver (FIE)</t>
-  </si>
-  <si>
-    <t>KW 50
-2026-12-12</t>
-  </si>
-  <si>
-    <t>FIE - FIE_Tashkent (FIE)
-Osnabrück - QB_U20_10 (QB)</t>
-  </si>
-  <si>
-    <t>KW 51
-2026-12-19</t>
-  </si>
-  <si>
-    <t>Rüsselsheim - DM_U17_18 (DM)
-Leverkusen - DM_U17_20 (DM)</t>
-  </si>
-  <si>
-    <t>Rüsselsheim - DM_U13_19 (DM)
-Leverkusen - DM_U13_21 (DM)</t>
-  </si>
-  <si>
-    <t>KW 53
-2027-01-02</t>
-  </si>
-  <si>
-    <t>EFC - EFC_Lausanne (EFC)</t>
-  </si>
-  <si>
-    <t>KW 1
-2027-01-09</t>
-  </si>
-  <si>
-    <t>FIE - FIE_Fujairah (FIE)</t>
-  </si>
-  <si>
-    <t>KW 2
-2027-01-16</t>
-  </si>
-  <si>
-    <t>FIE - FIE_Manama (FIE)</t>
-  </si>
-  <si>
-    <t>KW 3
-2027-01-23</t>
-  </si>
-  <si>
-    <t>FIE - FIE_Doha (FIE)</t>
-  </si>
-  <si>
-    <t>KW 4
-2027-01-30</t>
-  </si>
-  <si>
-    <t>FIE - FIE_Cairo (FIE)</t>
-  </si>
-  <si>
-    <t>KW 5
-2027-02-06</t>
-  </si>
-  <si>
-    <t>FIE - FIE_Heidenheim (FIE)</t>
-  </si>
-  <si>
-    <t>EFC - EFC_Brindisi (EFC)</t>
-  </si>
-  <si>
-    <t>KW 6
-2027-02-13</t>
-  </si>
-  <si>
-    <t>EFC - EFC_Differdange (EFC)</t>
-  </si>
-  <si>
-    <t>KW 7
-2027-02-20</t>
-  </si>
-  <si>
-    <t>EFC - EFC_Laupheim (EFC)</t>
-  </si>
-  <si>
-    <t>KW 8
-2027-02-27</t>
-  </si>
-  <si>
-    <t>EFC - EFC_Thessaloniki (EFC)</t>
-  </si>
-  <si>
-    <t>KW 9
-2027-03-06</t>
-  </si>
-  <si>
-    <t>EFC - EFC_Sofia (EFC)</t>
-  </si>
-  <si>
-    <t>KW 10
-2027-03-13</t>
-  </si>
-  <si>
-    <t>FIE - FIE_Budapest (FIE)</t>
-  </si>
-  <si>
-    <t>KW 11
-2027-03-20</t>
-  </si>
-  <si>
-    <t>EFC - EFC_Napoli (EFC)</t>
-  </si>
-  <si>
-    <t>KW 12
-2027-03-27</t>
-  </si>
-  <si>
-    <t>FIE - FIE_Astana (FIE)</t>
-  </si>
-  <si>
-    <t>KW 13
-2027-04-03</t>
-  </si>
-  <si>
-    <t>Leipzig - QB_U17_5 (QB)</t>
-  </si>
-  <si>
     <t>KW 14
 2027-04-10</t>
   </si>
   <si>
-    <t>EFC - EFC_Budapest (EFC)</t>
+    <t>FIE - FIE_WM_U20 (FIE)</t>
   </si>
   <si>
     <t>KW 15
 2027-04-17</t>
   </si>
   <si>
-    <t>FIE - FIE_Vrsac (FIE)</t>
+    <t>EFC - EFC_Zagreb (EFC)</t>
   </si>
   <si>
     <t>KW 16
@@ -331,43 +324,26 @@
     <t>EFC - EFC_EM_U20 (EFC)</t>
   </si>
   <si>
-    <t>KW 17
-2027-05-01</t>
-  </si>
-  <si>
-    <t>EFC - EFC_Grenoble (EFC)</t>
-  </si>
-  <si>
     <t>KW 18
 2027-05-08</t>
   </si>
   <si>
-    <t>FIE - FIE_Medellin (FIE)
-Reutlingen - QB_SEN_2 (QB)</t>
+    <t>FIE - FIE_Medellin (FIE)</t>
   </si>
   <si>
     <t>KW 19
 2027-05-15</t>
   </si>
   <si>
-    <t>EFC - EFC_Copenhagen (EFC)</t>
+    <t>EFC - EFC_Budapest (EFC)</t>
   </si>
   <si>
     <t>KW 20
 2027-05-22</t>
   </si>
   <si>
-    <t>FIE - FIE_Bern (FIE)</t>
-  </si>
-  <si>
-    <t>Leverkusen - QB_U20_9 (QB)</t>
-  </si>
-  <si>
-    <t>KW 21
-2027-05-29</t>
-  </si>
-  <si>
-    <t>EFC - EFC_Zagreb (EFC)</t>
+    <t>FIE - FIE_Bern (FIE)
+EFC - EFC_Kamnik (EFC)</t>
   </si>
   <si>
     <t>KW 22
@@ -388,14 +364,56 @@
 2027-06-19</t>
   </si>
   <si>
-    <t>EFC - EFC_Bratislava (EFC)</t>
+    <t>FIE - FIE_Manama (FIE)</t>
   </si>
   <si>
     <t>KW 25
 2027-06-26</t>
   </si>
   <si>
-    <t>EFC - EFC_Belgrade (EFC)</t>
+    <t>DM - DM_Finals (DM)</t>
+  </si>
+  <si>
+    <t>KW 28
+2027-07-17</t>
+  </si>
+  <si>
+    <t>FIE - FIE_WM_Senioren (FIE)</t>
+  </si>
+  <si>
+    <t>KW 31
+2027-08-07</t>
+  </si>
+  <si>
+    <t>EFC - EFC_Copenhagen (EFC)</t>
+  </si>
+  <si>
+    <t>KW 32
+2027-08-14</t>
+  </si>
+  <si>
+    <t>EFC - EFC_Colmar (EFC)</t>
+  </si>
+  <si>
+    <t>KW 33
+2027-08-21</t>
+  </si>
+  <si>
+    <t>FIE - FIE_Hongkong (FIE)</t>
+  </si>
+  <si>
+    <t>KW 34
+2027-08-28</t>
+  </si>
+  <si>
+    <t>FIE - FIE_Tashkent (FIE)</t>
+  </si>
+  <si>
+    <t>KW 35
+2027-09-04</t>
+  </si>
+  <si>
+    <t>EFC - EFC_Berlin (EFC)</t>
   </si>
 </sst>
 </file>
@@ -403,7 +421,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="45">
+  <fonts count="49">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
@@ -416,6 +434,26 @@
       <sz val="11.0"/>
       <b val="true"/>
       <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -672,22 +710,22 @@
     </fill>
     <fill>
       <patternFill patternType="none">
+        <fgColor rgb="0070C0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0070C0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="none">
         <fgColor rgb="C00000"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="C00000"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="none">
-        <fgColor rgb="0070C0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="0070C0"/>
       </patternFill>
     </fill>
   </fills>
@@ -721,7 +759,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="406">
+  <cellXfs count="439">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="true" applyFill="true" applyAlignment="true" applyBorder="true">
       <alignment horizontal="center" vertical="center"/>
@@ -741,16 +779,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -765,10 +800,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -795,19 +830,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -828,10 +860,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -858,10 +887,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -894,12 +920,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
@@ -921,10 +941,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -960,13 +980,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -981,22 +998,22 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1017,10 +1034,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1050,10 +1067,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1071,16 +1091,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1101,10 +1121,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1131,13 +1151,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1152,13 +1172,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1182,13 +1205,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1209,13 +1235,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1239,13 +1262,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1263,10 +1286,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1296,13 +1319,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1317,10 +1340,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1350,13 +1373,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1371,16 +1397,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1401,19 +1424,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1431,13 +1454,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1458,10 +1484,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1485,10 +1511,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1509,10 +1535,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1545,10 +1571,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1563,10 +1592,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1611,6 +1640,9 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
     <xf numFmtId="0" fontId="33" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
@@ -1623,13 +1655,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1644,16 +1676,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1677,10 +1709,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1698,19 +1730,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1725,19 +1757,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1752,19 +1784,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1800,28 +1832,25 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
     <xf numFmtId="0" fontId="40" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1836,16 +1865,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1872,10 +1901,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1890,19 +1919,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1926,10 +1955,118 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
+      <alignment horizontal="center" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
+      <alignment horizontal="center" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
+      <alignment horizontal="center" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
+      <alignment horizontal="center" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1944,7 +2081,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H48"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="25.0" customWidth="true"/>
@@ -1987,637 +2124,687 @@
       <c r="A2" t="s" s="2">
         <v>8</v>
       </c>
-      <c r="B2" t="s" s="4">
+      <c r="B2" s="3"/>
+      <c r="C2" t="s" s="5">
         <v>9</v>
       </c>
-      <c r="C2" s="5"/>
       <c r="D2" s="6"/>
-      <c r="E2" t="s" s="8">
+      <c r="E2" s="7"/>
+      <c r="F2" s="8"/>
+      <c r="G2" t="s" s="10">
         <v>10</v>
       </c>
-      <c r="F2" t="s" s="10">
+      <c r="H2" s="11"/>
+    </row>
+    <row r="3" ht="40.0" customHeight="true">
+      <c r="A3" t="s" s="12">
         <v>11</v>
       </c>
-      <c r="G2" s="11"/>
-      <c r="H2" s="12"/>
-    </row>
-    <row r="3" ht="40.0" customHeight="true">
-      <c r="A3" t="s" s="13">
+      <c r="B3" s="13"/>
+      <c r="C3" t="s" s="15">
         <v>12</v>
       </c>
-      <c r="B3" s="14"/>
-      <c r="C3" t="s" s="16">
+      <c r="D3" s="16"/>
+      <c r="E3" s="17"/>
+      <c r="F3" s="18"/>
+      <c r="G3" t="s" s="20">
         <v>13</v>
       </c>
-      <c r="D3" s="17"/>
-      <c r="E3" s="18"/>
-      <c r="F3" s="19"/>
-      <c r="G3" t="s" s="21">
+      <c r="H3" s="21"/>
+    </row>
+    <row r="4" ht="40.0" customHeight="true">
+      <c r="A4" t="s" s="22">
         <v>14</v>
       </c>
-      <c r="H3" s="22"/>
-    </row>
-    <row r="4" ht="40.0" customHeight="true">
-      <c r="A4" t="s" s="23">
+      <c r="B4" t="s" s="24">
         <v>15</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" t="s" s="26">
+      <c r="C4" s="25"/>
+      <c r="D4" s="26"/>
+      <c r="E4" s="27"/>
+      <c r="F4" t="s" s="29">
         <v>16</v>
       </c>
-      <c r="D4" s="27"/>
-      <c r="E4" t="s" s="29">
+      <c r="G4" s="30"/>
+      <c r="H4" s="31"/>
+    </row>
+    <row r="5" ht="40.0" customHeight="true">
+      <c r="A5" t="s" s="32">
         <v>17</v>
       </c>
-      <c r="F4" s="30"/>
-      <c r="G4" t="s" s="32">
+      <c r="B5" s="33"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="35"/>
+      <c r="E5" s="36"/>
+      <c r="F5" t="s" s="38">
         <v>18</v>
       </c>
-      <c r="H4" s="33"/>
-    </row>
-    <row r="5" ht="40.0" customHeight="true">
-      <c r="A5" t="s" s="34">
+      <c r="G5" s="39"/>
+      <c r="H5" s="40"/>
+    </row>
+    <row r="6" ht="40.0" customHeight="true">
+      <c r="A6" t="s" s="41">
         <v>19</v>
       </c>
-      <c r="B5" s="35"/>
-      <c r="C5" t="s" s="37">
+      <c r="B6" s="42"/>
+      <c r="C6" s="43"/>
+      <c r="D6" s="44"/>
+      <c r="E6" s="45"/>
+      <c r="F6" t="s" s="47">
         <v>20</v>
       </c>
-      <c r="D5" s="38"/>
-      <c r="E5" s="39"/>
-      <c r="F5" s="40"/>
-      <c r="G5" t="s" s="42">
+      <c r="G6" s="48"/>
+      <c r="H6" s="49"/>
+    </row>
+    <row r="7" ht="40.0" customHeight="true">
+      <c r="A7" t="s" s="50">
         <v>21</v>
       </c>
-      <c r="H5" s="43"/>
-    </row>
-    <row r="6" ht="40.0" customHeight="true">
-      <c r="A6" t="s" s="44">
+      <c r="B7" s="51"/>
+      <c r="C7" s="52"/>
+      <c r="D7" s="53"/>
+      <c r="E7" s="54"/>
+      <c r="F7" t="s" s="56">
         <v>22</v>
       </c>
-      <c r="B6" s="45"/>
-      <c r="C6" t="s" s="47">
+      <c r="G7" s="57"/>
+      <c r="H7" s="58"/>
+    </row>
+    <row r="8" ht="40.0" customHeight="true">
+      <c r="A8" t="s" s="59">
         <v>23</v>
       </c>
-      <c r="D6" s="48"/>
-      <c r="E6" s="49"/>
-      <c r="F6" s="50"/>
-      <c r="G6" t="s" s="52">
+      <c r="B8" s="60"/>
+      <c r="C8" s="61"/>
+      <c r="D8" s="62"/>
+      <c r="E8" t="s" s="64">
         <v>24</v>
       </c>
-      <c r="H6" s="53"/>
-    </row>
-    <row r="7" ht="40.0" customHeight="true">
-      <c r="A7" t="s" s="54">
+      <c r="F8" s="65"/>
+      <c r="G8" t="s" s="67">
         <v>25</v>
       </c>
-      <c r="B7" s="55"/>
-      <c r="C7" t="s" s="57">
+      <c r="H8" s="68"/>
+    </row>
+    <row r="9" ht="40.0" customHeight="true">
+      <c r="A9" t="s" s="69">
         <v>26</v>
       </c>
-      <c r="D7" t="s" s="59">
+      <c r="B9" s="70"/>
+      <c r="C9" s="71"/>
+      <c r="D9" s="72"/>
+      <c r="E9" s="73"/>
+      <c r="F9" t="s" s="75">
         <v>27</v>
       </c>
-      <c r="E7" s="60"/>
-      <c r="F7" s="61"/>
-      <c r="G7" t="s" s="63">
+      <c r="G9" s="76"/>
+      <c r="H9" s="77"/>
+    </row>
+    <row r="10" ht="40.0" customHeight="true">
+      <c r="A10" t="s" s="78">
         <v>28</v>
       </c>
-      <c r="H7" s="64"/>
-    </row>
-    <row r="8" ht="40.0" customHeight="true">
-      <c r="A8" t="s" s="65">
+      <c r="B10" s="79"/>
+      <c r="C10" t="s" s="81">
         <v>29</v>
       </c>
-      <c r="B8" s="66"/>
-      <c r="C8" t="s" s="68">
+      <c r="D10" s="82"/>
+      <c r="E10" s="83"/>
+      <c r="F10" t="s" s="85">
         <v>30</v>
       </c>
-      <c r="D8" s="69"/>
-      <c r="E8" s="70"/>
-      <c r="F8" s="71"/>
-      <c r="G8" t="s" s="73">
+      <c r="G10" s="86"/>
+      <c r="H10" s="87"/>
+    </row>
+    <row r="11" ht="40.0" customHeight="true">
+      <c r="A11" t="s" s="88">
         <v>31</v>
       </c>
-      <c r="H8" s="74"/>
-    </row>
-    <row r="9" ht="40.0" customHeight="true">
-      <c r="A9" t="s" s="75">
+      <c r="B11" s="89"/>
+      <c r="C11" s="90"/>
+      <c r="D11" s="91"/>
+      <c r="E11" t="s" s="93">
         <v>32</v>
       </c>
-      <c r="B9" s="76"/>
-      <c r="C9" s="77"/>
-      <c r="D9" s="78"/>
-      <c r="E9" t="s" s="80">
+      <c r="F11" s="94"/>
+      <c r="G11" t="s" s="96">
         <v>33</v>
       </c>
-      <c r="F9" s="81"/>
-      <c r="G9" t="s" s="83">
+      <c r="H11" s="97"/>
+    </row>
+    <row r="12" ht="40.0" customHeight="true">
+      <c r="A12" t="s" s="98">
         <v>34</v>
       </c>
-      <c r="H9" s="84"/>
-    </row>
-    <row r="10" ht="40.0" customHeight="true">
-      <c r="A10" t="s" s="85">
+      <c r="B12" s="99"/>
+      <c r="C12" s="100"/>
+      <c r="D12" s="101"/>
+      <c r="E12" t="s" s="103">
         <v>35</v>
       </c>
-      <c r="B10" s="86"/>
-      <c r="C10" t="s" s="88">
+      <c r="F12" s="104"/>
+      <c r="G12" t="s" s="106">
         <v>36</v>
       </c>
-      <c r="D10" s="89"/>
-      <c r="E10" s="90"/>
-      <c r="F10" t="s" s="92">
+      <c r="H12" s="107"/>
+    </row>
+    <row r="13" ht="40.0" customHeight="true">
+      <c r="A13" t="s" s="108">
         <v>37</v>
       </c>
-      <c r="G10" s="93"/>
-      <c r="H10" s="94"/>
-    </row>
-    <row r="11" ht="40.0" customHeight="true">
-      <c r="A11" t="s" s="95">
+      <c r="B13" s="109"/>
+      <c r="C13" s="110"/>
+      <c r="D13" t="s" s="112">
         <v>38</v>
       </c>
-      <c r="B11" s="96"/>
-      <c r="C11" s="97"/>
-      <c r="D11" s="98"/>
-      <c r="E11" t="s" s="100">
+      <c r="E13" t="s" s="114">
         <v>39</v>
       </c>
-      <c r="F11" t="s" s="102">
+      <c r="F13" s="115"/>
+      <c r="G13" s="116"/>
+      <c r="H13" s="117"/>
+    </row>
+    <row r="14" ht="40.0" customHeight="true">
+      <c r="A14" t="s" s="118">
         <v>40</v>
       </c>
-      <c r="G11" s="103"/>
-      <c r="H11" s="104"/>
-    </row>
-    <row r="12" ht="40.0" customHeight="true">
-      <c r="A12" t="s" s="105">
+      <c r="B14" s="119"/>
+      <c r="C14" s="120"/>
+      <c r="D14" t="s" s="122">
         <v>41</v>
       </c>
-      <c r="B12" s="106"/>
-      <c r="C12" s="107"/>
-      <c r="D12" s="108"/>
-      <c r="E12" s="109"/>
-      <c r="F12" t="s" s="111">
+      <c r="E14" s="123"/>
+      <c r="F14" s="124"/>
+      <c r="G14" s="125"/>
+      <c r="H14" s="126"/>
+    </row>
+    <row r="15" ht="40.0" customHeight="true">
+      <c r="A15" t="s" s="127">
         <v>42</v>
       </c>
-      <c r="G12" s="112"/>
-      <c r="H12" s="113"/>
-    </row>
-    <row r="13" ht="40.0" customHeight="true">
-      <c r="A13" t="s" s="114">
+      <c r="B15" s="128"/>
+      <c r="C15" s="129"/>
+      <c r="D15" s="130"/>
+      <c r="E15" s="131"/>
+      <c r="F15" t="s" s="133">
         <v>43</v>
       </c>
-      <c r="B13" s="115"/>
-      <c r="C13" s="116"/>
-      <c r="D13" s="117"/>
-      <c r="E13" t="s" s="119">
+      <c r="G15" s="134"/>
+      <c r="H15" s="135"/>
+    </row>
+    <row r="16" ht="40.0" customHeight="true">
+      <c r="A16" t="s" s="136">
         <v>44</v>
       </c>
-      <c r="F13" t="s" s="121">
+      <c r="B16" s="137"/>
+      <c r="C16" t="s" s="139">
         <v>45</v>
       </c>
-      <c r="G13" s="122"/>
-      <c r="H13" s="123"/>
-    </row>
-    <row r="14" ht="40.0" customHeight="true">
-      <c r="A14" t="s" s="124">
+      <c r="D16" t="s" s="141">
         <v>46</v>
       </c>
-      <c r="B14" s="125"/>
-      <c r="C14" s="126"/>
-      <c r="D14" s="127"/>
-      <c r="E14" t="s" s="129">
+      <c r="E16" s="142"/>
+      <c r="F16" s="143"/>
+      <c r="G16" s="144"/>
+      <c r="H16" s="145"/>
+    </row>
+    <row r="17" ht="40.0" customHeight="true">
+      <c r="A17" t="s" s="146">
         <v>47</v>
       </c>
-      <c r="F14" s="130"/>
-      <c r="G14" s="131"/>
-      <c r="H14" s="132"/>
-    </row>
-    <row r="15" ht="40.0" customHeight="true">
-      <c r="A15" t="s" s="133">
+      <c r="B17" s="147"/>
+      <c r="C17" s="148"/>
+      <c r="D17" t="s" s="150">
         <v>48</v>
       </c>
-      <c r="B15" s="134"/>
-      <c r="C15" s="135"/>
-      <c r="D15" s="136"/>
-      <c r="E15" t="s" s="138">
+      <c r="E17" s="151"/>
+      <c r="F17" s="152"/>
+      <c r="G17" t="s" s="154">
         <v>49</v>
       </c>
-      <c r="F15" s="139"/>
-      <c r="G15" s="140"/>
-      <c r="H15" s="141"/>
-    </row>
-    <row r="16" ht="40.0" customHeight="true">
-      <c r="A16" t="s" s="142">
+      <c r="H17" s="155"/>
+    </row>
+    <row r="18" ht="40.0" customHeight="true">
+      <c r="A18" t="s" s="156">
         <v>50</v>
       </c>
-      <c r="B16" s="143"/>
-      <c r="C16" t="s" s="145">
+      <c r="B18" s="157"/>
+      <c r="C18" s="158"/>
+      <c r="D18" t="s" s="160">
         <v>51</v>
       </c>
-      <c r="D16" s="146"/>
-      <c r="E16" s="147"/>
-      <c r="F16" s="148"/>
-      <c r="G16" s="149"/>
-      <c r="H16" s="150"/>
-    </row>
-    <row r="17" ht="40.0" customHeight="true">
-      <c r="A17" t="s" s="151">
+      <c r="E18" s="161"/>
+      <c r="F18" s="162"/>
+      <c r="G18" s="163"/>
+      <c r="H18" s="164"/>
+    </row>
+    <row r="19" ht="40.0" customHeight="true">
+      <c r="A19" t="s" s="165">
         <v>52</v>
       </c>
-      <c r="B17" s="152"/>
-      <c r="C17" s="153"/>
-      <c r="D17" s="154"/>
-      <c r="E17" t="s" s="156">
+      <c r="B19" s="166"/>
+      <c r="C19" s="167"/>
+      <c r="D19" s="168"/>
+      <c r="E19" t="s" s="170">
         <v>53</v>
       </c>
-      <c r="F17" s="157"/>
-      <c r="G17" s="158"/>
-      <c r="H17" s="159"/>
-    </row>
-    <row r="18" ht="40.0" customHeight="true">
-      <c r="A18" t="s" s="160">
+      <c r="F19" s="171"/>
+      <c r="G19" s="172"/>
+      <c r="H19" s="173"/>
+    </row>
+    <row r="20" ht="40.0" customHeight="true">
+      <c r="A20" t="s" s="174">
         <v>54</v>
       </c>
-      <c r="B18" s="161"/>
-      <c r="C18" s="162"/>
-      <c r="D18" s="163"/>
-      <c r="E18" s="164"/>
-      <c r="F18" t="s" s="166">
+      <c r="B20" s="175"/>
+      <c r="C20" t="s" s="177">
         <v>55</v>
       </c>
-      <c r="G18" s="167"/>
-      <c r="H18" t="s" s="169">
+      <c r="D20" s="178"/>
+      <c r="E20" s="179"/>
+      <c r="F20" s="180"/>
+      <c r="G20" s="181"/>
+      <c r="H20" s="182"/>
+    </row>
+    <row r="21" ht="40.0" customHeight="true">
+      <c r="A21" t="s" s="183">
         <v>56</v>
       </c>
-    </row>
-    <row r="19" ht="40.0" customHeight="true">
-      <c r="A19" t="s" s="170">
+      <c r="B21" s="184"/>
+      <c r="C21" s="185"/>
+      <c r="D21" s="186"/>
+      <c r="E21" s="187"/>
+      <c r="F21" t="s" s="189">
         <v>57</v>
       </c>
-      <c r="B19" s="171"/>
-      <c r="C19" s="172"/>
-      <c r="D19" t="s" s="174">
+      <c r="G21" s="190"/>
+      <c r="H21" s="191"/>
+    </row>
+    <row r="22" ht="40.0" customHeight="true">
+      <c r="A22" t="s" s="192">
         <v>58</v>
       </c>
-      <c r="E19" s="175"/>
-      <c r="F19" s="176"/>
-      <c r="G19" s="177"/>
-      <c r="H19" s="178"/>
-    </row>
-    <row r="20" ht="40.0" customHeight="true">
-      <c r="A20" t="s" s="179">
+      <c r="B22" s="193"/>
+      <c r="C22" t="s" s="195">
         <v>59</v>
       </c>
-      <c r="B20" s="180"/>
-      <c r="C20" t="s" s="182">
+      <c r="D22" s="196"/>
+      <c r="E22" s="197"/>
+      <c r="F22" s="198"/>
+      <c r="G22" s="199"/>
+      <c r="H22" s="200"/>
+    </row>
+    <row r="23" ht="40.0" customHeight="true">
+      <c r="A23" t="s" s="201">
         <v>60</v>
       </c>
-      <c r="D20" s="183"/>
-      <c r="E20" s="184"/>
-      <c r="F20" s="185"/>
-      <c r="G20" s="186"/>
-      <c r="H20" s="187"/>
-    </row>
-    <row r="21" ht="40.0" customHeight="true">
-      <c r="A21" t="s" s="188">
+      <c r="B23" s="202"/>
+      <c r="C23" s="203"/>
+      <c r="D23" s="204"/>
+      <c r="E23" t="s" s="206">
         <v>61</v>
       </c>
-      <c r="B21" s="189"/>
-      <c r="C21" s="190"/>
-      <c r="D21" s="191"/>
-      <c r="E21" t="s" s="193">
+      <c r="F23" t="s" s="208">
         <v>62</v>
       </c>
-      <c r="F21" s="194"/>
-      <c r="G21" s="195"/>
-      <c r="H21" s="196"/>
-    </row>
-    <row r="22" ht="40.0" customHeight="true">
-      <c r="A22" t="s" s="197">
+      <c r="G23" s="209"/>
+      <c r="H23" s="210"/>
+    </row>
+    <row r="24" ht="40.0" customHeight="true">
+      <c r="A24" t="s" s="211">
         <v>63</v>
       </c>
-      <c r="B22" s="198"/>
-      <c r="C22" t="s" s="200">
+      <c r="B24" s="212"/>
+      <c r="C24" t="s" s="214">
         <v>64</v>
       </c>
-      <c r="D22" s="201"/>
-      <c r="E22" s="202"/>
-      <c r="F22" s="203"/>
-      <c r="G22" s="204"/>
-      <c r="H22" s="205"/>
-    </row>
-    <row r="23" ht="40.0" customHeight="true">
-      <c r="A23" t="s" s="206">
+      <c r="D24" s="215"/>
+      <c r="E24" s="216"/>
+      <c r="F24" s="217"/>
+      <c r="G24" s="218"/>
+      <c r="H24" s="219"/>
+    </row>
+    <row r="25" ht="40.0" customHeight="true">
+      <c r="A25" t="s" s="220">
         <v>65</v>
       </c>
-      <c r="B23" s="207"/>
-      <c r="C23" s="208"/>
-      <c r="D23" s="209"/>
-      <c r="E23" t="s" s="211">
+      <c r="B25" s="221"/>
+      <c r="C25" s="222"/>
+      <c r="D25" s="223"/>
+      <c r="E25" s="224"/>
+      <c r="F25" t="s" s="226">
         <v>66</v>
       </c>
-      <c r="F23" s="212"/>
-      <c r="G23" s="213"/>
-      <c r="H23" s="214"/>
-    </row>
-    <row r="24" ht="40.0" customHeight="true">
-      <c r="A24" t="s" s="215">
+      <c r="G25" s="227"/>
+      <c r="H25" s="228"/>
+    </row>
+    <row r="26" ht="40.0" customHeight="true">
+      <c r="A26" t="s" s="229">
         <v>67</v>
       </c>
-      <c r="B24" s="216"/>
-      <c r="C24" t="s" s="218">
+      <c r="B26" s="230"/>
+      <c r="C26" s="231"/>
+      <c r="D26" t="s" s="233">
         <v>68</v>
       </c>
-      <c r="D24" t="s" s="220">
+      <c r="E26" t="s" s="235">
         <v>69</v>
       </c>
-      <c r="E24" s="221"/>
-      <c r="F24" s="222"/>
-      <c r="G24" s="223"/>
-      <c r="H24" s="224"/>
-    </row>
-    <row r="25" ht="40.0" customHeight="true">
-      <c r="A25" t="s" s="225">
+      <c r="F26" s="236"/>
+      <c r="G26" s="237"/>
+      <c r="H26" s="238"/>
+    </row>
+    <row r="27" ht="40.0" customHeight="true">
+      <c r="A27" t="s" s="239">
         <v>70</v>
       </c>
-      <c r="B25" s="226"/>
-      <c r="C25" t="s" s="228">
+      <c r="B27" s="240"/>
+      <c r="C27" s="241"/>
+      <c r="D27" s="242"/>
+      <c r="E27" t="s" s="244">
         <v>71</v>
       </c>
-      <c r="D25" s="229"/>
-      <c r="E25" s="230"/>
-      <c r="F25" s="231"/>
-      <c r="G25" s="232"/>
-      <c r="H25" s="233"/>
-    </row>
-    <row r="26" ht="40.0" customHeight="true">
-      <c r="A26" t="s" s="234">
+      <c r="F27" s="245"/>
+      <c r="G27" s="246"/>
+      <c r="H27" s="247"/>
+    </row>
+    <row r="28" ht="40.0" customHeight="true">
+      <c r="A28" t="s" s="248">
         <v>72</v>
       </c>
-      <c r="B26" s="235"/>
-      <c r="C26" s="236"/>
-      <c r="D26" t="s" s="238">
+      <c r="B28" s="249"/>
+      <c r="C28" s="250"/>
+      <c r="D28" s="251"/>
+      <c r="E28" t="s" s="253">
         <v>73</v>
       </c>
-      <c r="E26" s="239"/>
-      <c r="F26" s="240"/>
-      <c r="G26" s="241"/>
-      <c r="H26" s="242"/>
-    </row>
-    <row r="27" ht="40.0" customHeight="true">
-      <c r="A27" t="s" s="243">
+      <c r="F28" s="254"/>
+      <c r="G28" s="255"/>
+      <c r="H28" s="256"/>
+    </row>
+    <row r="29" ht="40.0" customHeight="true">
+      <c r="A29" t="s" s="257">
         <v>74</v>
       </c>
-      <c r="B27" s="244"/>
-      <c r="C27" s="245"/>
-      <c r="D27" t="s" s="247">
+      <c r="B29" s="258"/>
+      <c r="C29" t="s" s="260">
         <v>75</v>
       </c>
-      <c r="E27" s="248"/>
-      <c r="F27" s="249"/>
-      <c r="G27" s="250"/>
-      <c r="H27" s="251"/>
-    </row>
-    <row r="28" ht="40.0" customHeight="true">
-      <c r="A28" t="s" s="252">
+      <c r="D29" s="261"/>
+      <c r="E29" s="262"/>
+      <c r="F29" s="263"/>
+      <c r="G29" s="264"/>
+      <c r="H29" s="265"/>
+    </row>
+    <row r="30" ht="40.0" customHeight="true">
+      <c r="A30" t="s" s="266">
         <v>76</v>
       </c>
-      <c r="B28" s="253"/>
-      <c r="C28" s="254"/>
-      <c r="D28" t="s" s="256">
+      <c r="B30" s="267"/>
+      <c r="C30" s="268"/>
+      <c r="D30" s="269"/>
+      <c r="E30" s="270"/>
+      <c r="F30" t="s" s="272">
         <v>77</v>
       </c>
-      <c r="E28" s="257"/>
-      <c r="F28" s="258"/>
-      <c r="G28" s="259"/>
-      <c r="H28" s="260"/>
-    </row>
-    <row r="29" ht="40.0" customHeight="true">
-      <c r="A29" t="s" s="261">
+      <c r="G30" s="273"/>
+      <c r="H30" t="s" s="275">
         <v>78</v>
       </c>
-      <c r="B29" s="262"/>
-      <c r="C29" t="s" s="264">
+    </row>
+    <row r="31" ht="40.0" customHeight="true">
+      <c r="A31" t="s" s="276">
         <v>79</v>
       </c>
-      <c r="D29" s="265"/>
-      <c r="E29" s="266"/>
-      <c r="F29" s="267"/>
-      <c r="G29" s="268"/>
-      <c r="H29" s="269"/>
-    </row>
-    <row r="30" ht="40.0" customHeight="true">
-      <c r="A30" t="s" s="270">
+      <c r="B31" s="277"/>
+      <c r="C31" t="s" s="279">
         <v>80</v>
       </c>
-      <c r="B30" s="271"/>
-      <c r="C30" s="272"/>
-      <c r="D30" s="273"/>
-      <c r="E30" s="274"/>
-      <c r="F30" t="s" s="276">
+      <c r="D31" s="280"/>
+      <c r="E31" s="281"/>
+      <c r="F31" s="282"/>
+      <c r="G31" s="283"/>
+      <c r="H31" s="284"/>
+    </row>
+    <row r="32" ht="40.0" customHeight="true">
+      <c r="A32" t="s" s="285">
         <v>81</v>
       </c>
-      <c r="G30" s="277"/>
-      <c r="H30" s="278"/>
-    </row>
-    <row r="31" ht="40.0" customHeight="true">
-      <c r="A31" t="s" s="279">
+      <c r="B32" s="286"/>
+      <c r="C32" s="287"/>
+      <c r="D32" s="288"/>
+      <c r="E32" t="s" s="290">
         <v>82</v>
       </c>
-      <c r="B31" s="280"/>
-      <c r="C31" t="s" s="282">
+      <c r="F32" s="291"/>
+      <c r="G32" t="s" s="293">
         <v>83</v>
       </c>
-      <c r="D31" s="283"/>
-      <c r="E31" s="284"/>
-      <c r="F31" s="285"/>
-      <c r="G31" s="286"/>
-      <c r="H31" s="287"/>
-    </row>
-    <row r="32" ht="40.0" customHeight="true">
-      <c r="A32" t="s" s="288">
+      <c r="H32" s="294"/>
+    </row>
+    <row r="33" ht="40.0" customHeight="true">
+      <c r="A33" t="s" s="295">
         <v>84</v>
       </c>
-      <c r="B32" s="289"/>
-      <c r="C32" s="290"/>
-      <c r="D32" s="291"/>
-      <c r="E32" s="292"/>
-      <c r="F32" t="s" s="294">
+      <c r="B33" s="296"/>
+      <c r="C33" s="297"/>
+      <c r="D33" s="298"/>
+      <c r="E33" t="s" s="300">
         <v>85</v>
       </c>
-      <c r="G32" s="295"/>
-      <c r="H32" s="296"/>
-    </row>
-    <row r="33" ht="40.0" customHeight="true">
-      <c r="A33" t="s" s="297">
+      <c r="F33" s="301"/>
+      <c r="G33" s="302"/>
+      <c r="H33" s="303"/>
+    </row>
+    <row r="34" ht="40.0" customHeight="true">
+      <c r="A34" t="s" s="304">
         <v>86</v>
       </c>
-      <c r="B33" s="298"/>
-      <c r="C33" s="299"/>
-      <c r="D33" s="300"/>
-      <c r="E33" s="301"/>
-      <c r="F33" t="s" s="303">
+      <c r="B34" s="305"/>
+      <c r="C34" t="s" s="307">
         <v>87</v>
       </c>
-      <c r="G33" s="304"/>
-      <c r="H33" s="305"/>
-    </row>
-    <row r="34" ht="40.0" customHeight="true">
-      <c r="A34" t="s" s="306">
+      <c r="D34" s="308"/>
+      <c r="E34" s="309"/>
+      <c r="F34" s="310"/>
+      <c r="G34" s="311"/>
+      <c r="H34" s="312"/>
+    </row>
+    <row r="35" ht="40.0" customHeight="true">
+      <c r="A35" t="s" s="313">
         <v>88</v>
       </c>
-      <c r="B34" s="307"/>
-      <c r="C34" s="308"/>
-      <c r="D34" s="309"/>
-      <c r="E34" t="s" s="311">
+      <c r="B35" s="314"/>
+      <c r="C35" s="315"/>
+      <c r="D35" s="316"/>
+      <c r="E35" t="s" s="318">
         <v>89</v>
       </c>
-      <c r="F34" s="312"/>
-      <c r="G34" s="313"/>
-      <c r="H34" s="314"/>
-    </row>
-    <row r="35" ht="40.0" customHeight="true">
-      <c r="A35" t="s" s="315">
+      <c r="F35" s="319"/>
+      <c r="G35" s="320"/>
+      <c r="H35" s="321"/>
+    </row>
+    <row r="36" ht="40.0" customHeight="true">
+      <c r="A36" t="s" s="322">
         <v>90</v>
       </c>
-      <c r="B35" s="316"/>
-      <c r="C35" s="317"/>
-      <c r="D35" s="318"/>
-      <c r="E35" t="s" s="320">
+      <c r="B36" s="323"/>
+      <c r="C36" t="s" s="325">
         <v>91</v>
       </c>
-      <c r="F35" s="321"/>
-      <c r="G35" s="322"/>
-      <c r="H35" s="323"/>
-    </row>
-    <row r="36" ht="40.0" customHeight="true">
-      <c r="A36" t="s" s="324">
+      <c r="D36" s="326"/>
+      <c r="E36" s="327"/>
+      <c r="F36" s="328"/>
+      <c r="G36" s="329"/>
+      <c r="H36" s="330"/>
+    </row>
+    <row r="37" ht="40.0" customHeight="true">
+      <c r="A37" t="s" s="331">
         <v>92</v>
       </c>
-      <c r="B36" s="325"/>
-      <c r="C36" s="326"/>
-      <c r="D36" s="327"/>
-      <c r="E36" s="328"/>
-      <c r="F36" t="s" s="330">
+      <c r="B37" s="332"/>
+      <c r="C37" s="333"/>
+      <c r="D37" s="334"/>
+      <c r="E37" s="335"/>
+      <c r="F37" t="s" s="337">
         <v>93</v>
       </c>
-      <c r="G36" s="331"/>
-      <c r="H36" s="332"/>
-    </row>
-    <row r="37" ht="40.0" customHeight="true">
-      <c r="A37" t="s" s="333">
+      <c r="G37" s="338"/>
+      <c r="H37" s="339"/>
+    </row>
+    <row r="38" ht="40.0" customHeight="true">
+      <c r="A38" t="s" s="340">
         <v>94</v>
       </c>
-      <c r="B37" s="334"/>
-      <c r="C37" t="s" s="336">
+      <c r="B38" s="341"/>
+      <c r="C38" t="s" s="343">
         <v>95</v>
       </c>
-      <c r="D37" s="337"/>
-      <c r="E37" s="338"/>
-      <c r="F37" s="339"/>
-      <c r="G37" s="340"/>
-      <c r="H37" s="341"/>
-    </row>
-    <row r="38" ht="40.0" customHeight="true">
-      <c r="A38" t="s" s="342">
+      <c r="D38" s="344"/>
+      <c r="E38" s="345"/>
+      <c r="F38" s="346"/>
+      <c r="G38" s="347"/>
+      <c r="H38" s="348"/>
+    </row>
+    <row r="39" ht="40.0" customHeight="true">
+      <c r="A39" t="s" s="349">
         <v>96</v>
       </c>
-      <c r="B38" s="343"/>
-      <c r="C38" s="344"/>
-      <c r="D38" s="345"/>
-      <c r="E38" s="346"/>
-      <c r="F38" t="s" s="348">
+      <c r="B39" s="350"/>
+      <c r="C39" t="s" s="352">
         <v>97</v>
       </c>
-      <c r="G38" s="349"/>
-      <c r="H38" s="350"/>
-    </row>
-    <row r="39" ht="40.0" customHeight="true">
-      <c r="A39" t="s" s="351">
+      <c r="D39" s="353"/>
+      <c r="E39" s="354"/>
+      <c r="F39" s="355"/>
+      <c r="G39" s="356"/>
+      <c r="H39" s="357"/>
+    </row>
+    <row r="40" ht="40.0" customHeight="true">
+      <c r="A40" t="s" s="358">
         <v>98</v>
       </c>
-      <c r="B39" s="352"/>
-      <c r="C39" t="s" s="354">
+      <c r="B40" s="359"/>
+      <c r="C40" s="360"/>
+      <c r="D40" s="361"/>
+      <c r="E40" s="362"/>
+      <c r="F40" t="s" s="364">
         <v>99</v>
       </c>
-      <c r="D39" s="355"/>
-      <c r="E39" t="s" s="357">
+      <c r="G40" s="365"/>
+      <c r="H40" s="366"/>
+    </row>
+    <row r="41" ht="40.0" customHeight="true">
+      <c r="A41" t="s" s="367">
         <v>100</v>
       </c>
-      <c r="F39" s="358"/>
-      <c r="G39" s="359"/>
-      <c r="H39" s="360"/>
-    </row>
-    <row r="40" ht="40.0" customHeight="true">
-      <c r="A40" t="s" s="361">
+      <c r="B41" s="368"/>
+      <c r="C41" s="369"/>
+      <c r="D41" s="370"/>
+      <c r="E41" t="s" s="372">
         <v>101</v>
       </c>
-      <c r="B40" s="362"/>
-      <c r="C40" t="s" s="364">
+      <c r="F41" s="373"/>
+      <c r="G41" s="374"/>
+      <c r="H41" s="375"/>
+    </row>
+    <row r="42" ht="40.0" customHeight="true">
+      <c r="A42" t="s" s="376">
         <v>102</v>
       </c>
-      <c r="D40" s="365"/>
-      <c r="E40" s="366"/>
-      <c r="F40" s="367"/>
-      <c r="G40" s="368"/>
-      <c r="H40" s="369"/>
-    </row>
-    <row r="41" ht="40.0" customHeight="true">
-      <c r="A41" t="s" s="370">
+      <c r="B42" s="377"/>
+      <c r="C42" t="s" s="379">
         <v>103</v>
       </c>
-      <c r="B41" s="371"/>
-      <c r="C41" t="s" s="373">
+      <c r="D42" s="380"/>
+      <c r="E42" s="381"/>
+      <c r="F42" s="382"/>
+      <c r="G42" s="383"/>
+      <c r="H42" s="384"/>
+    </row>
+    <row r="43" ht="40.0" customHeight="true">
+      <c r="A43" t="s" s="385">
         <v>104</v>
       </c>
-      <c r="D41" s="374"/>
-      <c r="E41" s="375"/>
-      <c r="F41" s="376"/>
-      <c r="G41" s="377"/>
-      <c r="H41" s="378"/>
-    </row>
-    <row r="42" ht="40.0" customHeight="true">
-      <c r="A42" t="s" s="379">
+      <c r="B43" s="386"/>
+      <c r="C43" t="s" s="388">
         <v>105</v>
       </c>
-      <c r="B42" s="380"/>
-      <c r="C42" s="381"/>
-      <c r="D42" s="382"/>
-      <c r="E42" s="383"/>
-      <c r="F42" t="s" s="385">
+      <c r="D43" s="389"/>
+      <c r="E43" s="390"/>
+      <c r="F43" s="391"/>
+      <c r="G43" s="392"/>
+      <c r="H43" s="393"/>
+    </row>
+    <row r="44" ht="40.0" customHeight="true">
+      <c r="A44" t="s" s="394">
         <v>106</v>
       </c>
-      <c r="G42" s="386"/>
-      <c r="H42" s="387"/>
-    </row>
-    <row r="43" ht="40.0" customHeight="true">
-      <c r="A43" t="s" s="388">
+      <c r="B44" s="395"/>
+      <c r="C44" s="396"/>
+      <c r="D44" s="397"/>
+      <c r="E44" s="398"/>
+      <c r="F44" t="s" s="400">
         <v>107</v>
       </c>
-      <c r="B43" s="389"/>
-      <c r="C43" s="390"/>
-      <c r="D43" s="391"/>
-      <c r="E43" s="392"/>
-      <c r="F43" t="s" s="394">
+      <c r="G44" s="401"/>
+      <c r="H44" s="402"/>
+    </row>
+    <row r="45" ht="40.0" customHeight="true">
+      <c r="A45" t="s" s="403">
         <v>108</v>
       </c>
-      <c r="G43" s="395"/>
-      <c r="H43" s="396"/>
-    </row>
-    <row r="44" ht="40.0" customHeight="true">
-      <c r="A44" t="s" s="397">
+      <c r="B45" s="404"/>
+      <c r="C45" t="s" s="406">
         <v>109</v>
       </c>
-      <c r="B44" s="398"/>
-      <c r="C44" s="399"/>
-      <c r="D44" s="400"/>
-      <c r="E44" s="401"/>
-      <c r="F44" t="s" s="403">
+      <c r="D45" s="407"/>
+      <c r="E45" s="408"/>
+      <c r="F45" s="409"/>
+      <c r="G45" s="410"/>
+      <c r="H45" s="411"/>
+    </row>
+    <row r="46" ht="40.0" customHeight="true">
+      <c r="A46" t="s" s="412">
         <v>110</v>
       </c>
-      <c r="G44" s="404"/>
-      <c r="H44" s="405"/>
+      <c r="B46" s="413"/>
+      <c r="C46" s="414"/>
+      <c r="D46" s="415"/>
+      <c r="E46" t="s" s="417">
+        <v>111</v>
+      </c>
+      <c r="F46" s="418"/>
+      <c r="G46" s="419"/>
+      <c r="H46" s="420"/>
+    </row>
+    <row r="47" ht="40.0" customHeight="true">
+      <c r="A47" t="s" s="421">
+        <v>112</v>
+      </c>
+      <c r="B47" s="422"/>
+      <c r="C47" s="423"/>
+      <c r="D47" s="424"/>
+      <c r="E47" t="s" s="426">
+        <v>113</v>
+      </c>
+      <c r="F47" s="427"/>
+      <c r="G47" s="428"/>
+      <c r="H47" s="429"/>
+    </row>
+    <row r="48" ht="40.0" customHeight="true">
+      <c r="A48" t="s" s="430">
+        <v>114</v>
+      </c>
+      <c r="B48" s="431"/>
+      <c r="C48" t="s" s="433">
+        <v>115</v>
+      </c>
+      <c r="D48" s="434"/>
+      <c r="E48" s="435"/>
+      <c r="F48" s="436"/>
+      <c r="G48" s="437"/>
+      <c r="H48" s="438"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
Dates uodated und dann auch noch die Constarinats für fixe temrine
</commit_message>
<xml_diff>
--- a/Turnierplanung.xlsx
+++ b/Turnierplanung.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="103">
   <si>
     <t>Wochenende (KW)</t>
   </si>
@@ -45,58 +45,48 @@
     <t>Leverkusen - QB_SEN_1 (QB)</t>
   </si>
   <si>
-    <t>Leverkusen - CHALLENGE_U15_11 (CHALLENGE)</t>
+    <t>Bonn - CHALLENGE_U15_8 (CHALLENGE)</t>
   </si>
   <si>
     <t>KW 36
 2026-09-05</t>
   </si>
   <si>
-    <t>Reutlingen - QB_SEN_2 (QB)</t>
-  </si>
-  <si>
-    <t>Leipzig - CHALLENGE_U15_12 (CHALLENGE)</t>
+    <t>Erfurt - DM_VET_12 (DM)</t>
+  </si>
+  <si>
+    <t>Heidenheim - QB_U17_3 (QB)</t>
+  </si>
+  <si>
+    <t>Leverkusen - DM_U13_14 (DM)</t>
   </si>
   <si>
     <t>KW 37
 2026-09-12</t>
   </si>
   <si>
-    <t>Erfurt - DM_VET_17 (DM)</t>
-  </si>
-  <si>
-    <t>Leverkusen - QB_U17_3 (QB)</t>
+    <t>Offenbach - QB_U20_6 (QB)</t>
   </si>
   <si>
     <t>KW 38
 2026-09-19</t>
   </si>
   <si>
-    <t>Heidenheim - QB_U17_4 (QB)</t>
+    <t>Frankfurt - CHALLENGE_U15_9 (CHALLENGE)</t>
   </si>
   <si>
     <t>KW 39
 2026-09-26</t>
   </si>
   <si>
-    <t>Leipzig - QB_U17_5 (QB)</t>
-  </si>
-  <si>
-    <t>KW 40
-2026-10-03</t>
-  </si>
-  <si>
-    <t>Solingen - QB_U17_6 (QB)</t>
+    <t>Reutlingen - QB_SEN_2 (QB)</t>
   </si>
   <si>
     <t>KW 41
 2026-10-10</t>
   </si>
   <si>
-    <t>Offenbach - QB_U20_7 (QB)</t>
-  </si>
-  <si>
-    <t>Bonn - CHALLENGE_U15_13 (CHALLENGE)</t>
+    <t>Waldkirch - CHALLENGE_U15_10 (CHALLENGE)</t>
   </si>
   <si>
     <t>KW 42
@@ -120,20 +110,13 @@
 2026-10-31</t>
   </si>
   <si>
+    <t>EFC - EFC_Colmar (EFC)</t>
+  </si>
+  <si>
     <t>FIE - FIE_SanSalvador (FIE)</t>
   </si>
   <si>
-    <t>Frankfurt - CHALLENGE_U15_14 (CHALLENGE)</t>
-  </si>
-  <si>
-    <t>KW 45
-2026-11-07</t>
-  </si>
-  <si>
-    <t>Heidelberg - QB_U20_8 (QB)</t>
-  </si>
-  <si>
-    <t>Waldkirch - CHALLENGE_U15_15 (CHALLENGE)</t>
+    <t>Osnabrück - CHALLENGE_U15_11 (CHALLENGE)</t>
   </si>
   <si>
     <t>KW 46
@@ -146,6 +129,9 @@
     <t>FIE - FIE_SanJose (FIE)</t>
   </si>
   <si>
+    <t>EFC - EFC_Budapest (EFC)</t>
+  </si>
+  <si>
     <t>KW 47
 2026-11-21</t>
   </si>
@@ -157,6 +143,9 @@
 2026-11-28</t>
   </si>
   <si>
+    <t>FIE - FIE_Hongkong (FIE)</t>
+  </si>
+  <si>
     <t>EFC - EFC_Grenoble (EFC)</t>
   </si>
   <si>
@@ -170,6 +159,9 @@
     <t>EFC - EFC_Oslo (EFC)</t>
   </si>
   <si>
+    <t>EFC - EFC_Copenhagen (EFC)</t>
+  </si>
+  <si>
     <t>KW 50
 2026-12-12</t>
   </si>
@@ -177,7 +169,10 @@
     <t>EFC - EFC_Laupheim (EFC)</t>
   </si>
   <si>
-    <t>Osnabrück - CHALLENGE_U15_16 (CHALLENGE)</t>
+    <t>FIE - FIE_Tashkent (FIE)</t>
+  </si>
+  <si>
+    <t>Rüsselsheim - DM_U15_16 (DM)</t>
   </si>
   <si>
     <t>KW 51
@@ -205,6 +200,12 @@
 2027-01-16</t>
   </si>
   <si>
+    <t>EFC - EFC_Berlin (EFC)</t>
+  </si>
+  <si>
+    <t>FIE - FIE_Manama (FIE)</t>
+  </si>
+  <si>
     <t>EFC - EFC_Bratislava (EFC)</t>
   </si>
   <si>
@@ -249,18 +250,11 @@
     <t>FIE - FIE_Vrsac (FIE)</t>
   </si>
   <si>
-    <t>KW 8
-2027-02-27</t>
-  </si>
-  <si>
-    <t>Leverkusen - QB_U20_9 (QB)</t>
-  </si>
-  <si>
     <t>KW 9
 2027-03-06</t>
   </si>
   <si>
-    <t>Osnabrück - QB_U20_10 (QB)</t>
+    <t>Leipzig - QB_U17_4 (QB)</t>
   </si>
   <si>
     <t>KW 10
@@ -271,18 +265,6 @@
 EFC - EFC_Differdange (EFC)</t>
   </si>
   <si>
-    <t>KW 11
-2027-03-20</t>
-  </si>
-  <si>
-    <t>Rüsselsheim - DM_U17_18 (DM)
-Leverkusen - DM_U17_20 (DM)</t>
-  </si>
-  <si>
-    <t>Rüsselsheim - DM_U13_19 (DM)
-Leverkusen - DM_U13_21 (DM)</t>
-  </si>
-  <si>
     <t>KW 12
 2027-03-27</t>
   </si>
@@ -295,12 +277,7 @@
 2027-04-03</t>
   </si>
   <si>
-    <t>Leverkusen - DM_U20_22 (DM)
-Rüsselsheim - DM_U20_24 (DM)</t>
-  </si>
-  <si>
-    <t>Leverkusen - DM_U15_23 (DM)
-Rüsselsheim - DM_U15_25 (DM)</t>
+    <t>Solingen - QB_U17_5 (QB)</t>
   </si>
   <si>
     <t>KW 14
@@ -324,6 +301,13 @@
     <t>EFC - EFC_EM_U20 (EFC)</t>
   </si>
   <si>
+    <t>KW 17
+2027-05-01</t>
+  </si>
+  <si>
+    <t>Leverkusen - DM_U17_13 (DM)</t>
+  </si>
+  <si>
     <t>KW 18
 2027-05-08</t>
   </si>
@@ -331,13 +315,6 @@
     <t>FIE - FIE_Medellin (FIE)</t>
   </si>
   <si>
-    <t>KW 19
-2027-05-15</t>
-  </si>
-  <si>
-    <t>EFC - EFC_Budapest (EFC)</t>
-  </si>
-  <si>
     <t>KW 20
 2027-05-22</t>
   </si>
@@ -364,7 +341,7 @@
 2027-06-19</t>
   </si>
   <si>
-    <t>FIE - FIE_Manama (FIE)</t>
+    <t>Heidelberg - QB_U20_7 (QB)</t>
   </si>
   <si>
     <t>KW 25
@@ -381,39 +358,11 @@
     <t>FIE - FIE_WM_Senioren (FIE)</t>
   </si>
   <si>
-    <t>KW 31
-2027-08-07</t>
-  </si>
-  <si>
-    <t>EFC - EFC_Copenhagen (EFC)</t>
-  </si>
-  <si>
-    <t>KW 32
-2027-08-14</t>
-  </si>
-  <si>
-    <t>EFC - EFC_Colmar (EFC)</t>
-  </si>
-  <si>
-    <t>KW 33
-2027-08-21</t>
-  </si>
-  <si>
-    <t>FIE - FIE_Hongkong (FIE)</t>
-  </si>
-  <si>
-    <t>KW 34
-2027-08-28</t>
-  </si>
-  <si>
-    <t>FIE - FIE_Tashkent (FIE)</t>
-  </si>
-  <si>
-    <t>KW 35
-2027-09-04</t>
-  </si>
-  <si>
-    <t>EFC - EFC_Berlin (EFC)</t>
+    <t>KW 29
+2027-07-24</t>
+  </si>
+  <si>
+    <t>Rüsselsheim - DM_U20_15 (DM)</t>
   </si>
 </sst>
 </file>
@@ -421,7 +370,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="49">
+  <fonts count="41">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
@@ -434,46 +383,6 @@
       <sz val="11.0"/>
       <b val="true"/>
       <color indexed="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -759,7 +668,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="439">
+  <cellXfs count="370">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="true" applyFill="true" applyAlignment="true" applyBorder="true">
       <alignment horizontal="center" vertical="center"/>
@@ -824,6 +733,9 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
@@ -851,9 +763,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
@@ -950,13 +859,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -971,7 +877,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1007,13 +916,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1031,19 +943,22 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1061,13 +976,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1091,19 +1003,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1118,19 +1030,25 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1148,16 +1066,22 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1172,10 +1096,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1205,16 +1126,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1232,13 +1150,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1259,19 +1177,25 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1319,7 +1243,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1373,10 +1300,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1397,16 +1321,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1433,10 +1360,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1451,19 +1378,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1481,10 +1405,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1535,16 +1459,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1562,13 +1486,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1592,16 +1513,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1640,25 +1561,22 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
     <xf numFmtId="0" fontId="33" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1676,10 +1594,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1703,16 +1621,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1730,19 +1648,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1766,10 +1684,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1784,10 +1702,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1811,10 +1729,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1842,222 +1760,6 @@
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
-      <alignment horizontal="center" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
-      <alignment horizontal="center" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
-      <alignment horizontal="center" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
-      <alignment horizontal="center" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
-      <alignment horizontal="center" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
-      <alignment horizontal="center" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="47" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
-      <alignment horizontal="center" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
-      <alignment horizontal="center" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -2081,7 +1783,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="25.0" customWidth="true"/>
@@ -2140,31 +1842,31 @@
       <c r="A3" t="s" s="12">
         <v>11</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" t="s" s="15">
+      <c r="B3" t="s" s="14">
         <v>12</v>
       </c>
+      <c r="C3" s="15"/>
       <c r="D3" s="16"/>
       <c r="E3" s="17"/>
-      <c r="F3" s="18"/>
-      <c r="G3" t="s" s="20">
+      <c r="F3" t="s" s="19">
         <v>13</v>
       </c>
-      <c r="H3" s="21"/>
+      <c r="G3" s="20"/>
+      <c r="H3" t="s" s="22">
+        <v>14</v>
+      </c>
     </row>
     <row r="4" ht="40.0" customHeight="true">
-      <c r="A4" t="s" s="22">
-        <v>14</v>
-      </c>
-      <c r="B4" t="s" s="24">
+      <c r="A4" t="s" s="23">
         <v>15</v>
       </c>
+      <c r="B4" s="24"/>
       <c r="C4" s="25"/>
       <c r="D4" s="26"/>
-      <c r="E4" s="27"/>
-      <c r="F4" t="s" s="29">
+      <c r="E4" t="s" s="28">
         <v>16</v>
       </c>
+      <c r="F4" s="29"/>
       <c r="G4" s="30"/>
       <c r="H4" s="31"/>
     </row>
@@ -2176,10 +1878,10 @@
       <c r="C5" s="34"/>
       <c r="D5" s="35"/>
       <c r="E5" s="36"/>
-      <c r="F5" t="s" s="38">
+      <c r="F5" s="37"/>
+      <c r="G5" t="s" s="39">
         <v>18</v>
       </c>
-      <c r="G5" s="39"/>
       <c r="H5" s="40"/>
     </row>
     <row r="6" ht="40.0" customHeight="true">
@@ -2187,12 +1889,12 @@
         <v>19</v>
       </c>
       <c r="B6" s="42"/>
-      <c r="C6" s="43"/>
-      <c r="D6" s="44"/>
-      <c r="E6" s="45"/>
-      <c r="F6" t="s" s="47">
+      <c r="C6" t="s" s="44">
         <v>20</v>
       </c>
+      <c r="D6" s="45"/>
+      <c r="E6" s="46"/>
+      <c r="F6" s="47"/>
       <c r="G6" s="48"/>
       <c r="H6" s="49"/>
     </row>
@@ -2204,10 +1906,10 @@
       <c r="C7" s="52"/>
       <c r="D7" s="53"/>
       <c r="E7" s="54"/>
-      <c r="F7" t="s" s="56">
+      <c r="F7" s="55"/>
+      <c r="G7" t="s" s="57">
         <v>22</v>
       </c>
-      <c r="G7" s="57"/>
       <c r="H7" s="58"/>
     </row>
     <row r="8" ht="40.0" customHeight="true">
@@ -2217,21 +1919,21 @@
       <c r="B8" s="60"/>
       <c r="C8" s="61"/>
       <c r="D8" s="62"/>
-      <c r="E8" t="s" s="64">
+      <c r="E8" s="63"/>
+      <c r="F8" t="s" s="65">
         <v>24</v>
       </c>
-      <c r="F8" s="65"/>
-      <c r="G8" t="s" s="67">
+      <c r="G8" s="66"/>
+      <c r="H8" s="67"/>
+    </row>
+    <row r="9" ht="40.0" customHeight="true">
+      <c r="A9" t="s" s="68">
         <v>25</v>
       </c>
-      <c r="H8" s="68"/>
-    </row>
-    <row r="9" ht="40.0" customHeight="true">
-      <c r="A9" t="s" s="69">
+      <c r="B9" s="69"/>
+      <c r="C9" t="s" s="71">
         <v>26</v>
       </c>
-      <c r="B9" s="70"/>
-      <c r="C9" s="71"/>
       <c r="D9" s="72"/>
       <c r="E9" s="73"/>
       <c r="F9" t="s" s="75">
@@ -2249,562 +1951,456 @@
         <v>29</v>
       </c>
       <c r="D10" s="82"/>
-      <c r="E10" s="83"/>
-      <c r="F10" t="s" s="85">
+      <c r="E10" t="s" s="84">
         <v>30</v>
       </c>
-      <c r="G10" s="86"/>
-      <c r="H10" s="87"/>
+      <c r="F10" s="85"/>
+      <c r="G10" t="s" s="87">
+        <v>31</v>
+      </c>
+      <c r="H10" s="88"/>
     </row>
     <row r="11" ht="40.0" customHeight="true">
-      <c r="A11" t="s" s="88">
-        <v>31</v>
-      </c>
-      <c r="B11" s="89"/>
-      <c r="C11" s="90"/>
-      <c r="D11" s="91"/>
-      <c r="E11" t="s" s="93">
+      <c r="A11" t="s" s="89">
         <v>32</v>
       </c>
-      <c r="F11" s="94"/>
-      <c r="G11" t="s" s="96">
+      <c r="B11" s="90"/>
+      <c r="C11" s="91"/>
+      <c r="D11" t="s" s="93">
         <v>33</v>
       </c>
-      <c r="H11" s="97"/>
+      <c r="E11" t="s" s="95">
+        <v>34</v>
+      </c>
+      <c r="F11" t="s" s="97">
+        <v>35</v>
+      </c>
+      <c r="G11" s="98"/>
+      <c r="H11" s="99"/>
     </row>
     <row r="12" ht="40.0" customHeight="true">
-      <c r="A12" t="s" s="98">
-        <v>34</v>
-      </c>
-      <c r="B12" s="99"/>
-      <c r="C12" s="100"/>
-      <c r="D12" s="101"/>
-      <c r="E12" t="s" s="103">
-        <v>35</v>
-      </c>
-      <c r="F12" s="104"/>
-      <c r="G12" t="s" s="106">
+      <c r="A12" t="s" s="100">
         <v>36</v>
       </c>
-      <c r="H12" s="107"/>
+      <c r="B12" s="101"/>
+      <c r="C12" s="102"/>
+      <c r="D12" t="s" s="104">
+        <v>37</v>
+      </c>
+      <c r="E12" s="105"/>
+      <c r="F12" s="106"/>
+      <c r="G12" s="107"/>
+      <c r="H12" s="108"/>
     </row>
     <row r="13" ht="40.0" customHeight="true">
-      <c r="A13" t="s" s="108">
-        <v>37</v>
-      </c>
-      <c r="B13" s="109"/>
-      <c r="C13" s="110"/>
-      <c r="D13" t="s" s="112">
+      <c r="A13" t="s" s="109">
         <v>38</v>
       </c>
+      <c r="B13" s="110"/>
+      <c r="C13" s="111"/>
+      <c r="D13" s="112"/>
       <c r="E13" t="s" s="114">
         <v>39</v>
       </c>
-      <c r="F13" s="115"/>
-      <c r="G13" s="116"/>
-      <c r="H13" s="117"/>
+      <c r="F13" t="s" s="116">
+        <v>40</v>
+      </c>
+      <c r="G13" s="117"/>
+      <c r="H13" s="118"/>
     </row>
     <row r="14" ht="40.0" customHeight="true">
-      <c r="A14" t="s" s="118">
-        <v>40</v>
-      </c>
-      <c r="B14" s="119"/>
-      <c r="C14" s="120"/>
-      <c r="D14" t="s" s="122">
+      <c r="A14" t="s" s="119">
         <v>41</v>
       </c>
-      <c r="E14" s="123"/>
-      <c r="F14" s="124"/>
-      <c r="G14" s="125"/>
-      <c r="H14" s="126"/>
+      <c r="B14" s="120"/>
+      <c r="C14" t="s" s="122">
+        <v>42</v>
+      </c>
+      <c r="D14" t="s" s="124">
+        <v>43</v>
+      </c>
+      <c r="E14" s="125"/>
+      <c r="F14" t="s" s="127">
+        <v>44</v>
+      </c>
+      <c r="G14" s="128"/>
+      <c r="H14" s="129"/>
     </row>
     <row r="15" ht="40.0" customHeight="true">
-      <c r="A15" t="s" s="127">
-        <v>42</v>
-      </c>
-      <c r="B15" s="128"/>
-      <c r="C15" s="129"/>
-      <c r="D15" s="130"/>
-      <c r="E15" s="131"/>
-      <c r="F15" t="s" s="133">
-        <v>43</v>
-      </c>
-      <c r="G15" s="134"/>
-      <c r="H15" s="135"/>
+      <c r="A15" t="s" s="130">
+        <v>45</v>
+      </c>
+      <c r="B15" s="131"/>
+      <c r="C15" s="132"/>
+      <c r="D15" t="s" s="134">
+        <v>46</v>
+      </c>
+      <c r="E15" t="s" s="136">
+        <v>47</v>
+      </c>
+      <c r="F15" s="137"/>
+      <c r="G15" t="s" s="139">
+        <v>48</v>
+      </c>
+      <c r="H15" s="140"/>
     </row>
     <row r="16" ht="40.0" customHeight="true">
-      <c r="A16" t="s" s="136">
-        <v>44</v>
-      </c>
-      <c r="B16" s="137"/>
-      <c r="C16" t="s" s="139">
-        <v>45</v>
-      </c>
-      <c r="D16" t="s" s="141">
-        <v>46</v>
-      </c>
-      <c r="E16" s="142"/>
-      <c r="F16" s="143"/>
-      <c r="G16" s="144"/>
-      <c r="H16" s="145"/>
+      <c r="A16" t="s" s="141">
+        <v>49</v>
+      </c>
+      <c r="B16" s="142"/>
+      <c r="C16" s="143"/>
+      <c r="D16" t="s" s="145">
+        <v>50</v>
+      </c>
+      <c r="E16" s="146"/>
+      <c r="F16" s="147"/>
+      <c r="G16" s="148"/>
+      <c r="H16" s="149"/>
     </row>
     <row r="17" ht="40.0" customHeight="true">
-      <c r="A17" t="s" s="146">
-        <v>47</v>
-      </c>
-      <c r="B17" s="147"/>
-      <c r="C17" s="148"/>
-      <c r="D17" t="s" s="150">
-        <v>48</v>
-      </c>
-      <c r="E17" s="151"/>
-      <c r="F17" s="152"/>
-      <c r="G17" t="s" s="154">
-        <v>49</v>
-      </c>
-      <c r="H17" s="155"/>
+      <c r="A17" t="s" s="150">
+        <v>51</v>
+      </c>
+      <c r="B17" s="151"/>
+      <c r="C17" s="152"/>
+      <c r="D17" s="153"/>
+      <c r="E17" t="s" s="155">
+        <v>52</v>
+      </c>
+      <c r="F17" s="156"/>
+      <c r="G17" s="157"/>
+      <c r="H17" s="158"/>
     </row>
     <row r="18" ht="40.0" customHeight="true">
-      <c r="A18" t="s" s="156">
-        <v>50</v>
-      </c>
-      <c r="B18" s="157"/>
-      <c r="C18" s="158"/>
-      <c r="D18" t="s" s="160">
-        <v>51</v>
-      </c>
-      <c r="E18" s="161"/>
-      <c r="F18" s="162"/>
-      <c r="G18" s="163"/>
-      <c r="H18" s="164"/>
+      <c r="A18" t="s" s="159">
+        <v>53</v>
+      </c>
+      <c r="B18" s="160"/>
+      <c r="C18" t="s" s="162">
+        <v>54</v>
+      </c>
+      <c r="D18" s="163"/>
+      <c r="E18" s="164"/>
+      <c r="F18" s="165"/>
+      <c r="G18" s="166"/>
+      <c r="H18" s="167"/>
     </row>
     <row r="19" ht="40.0" customHeight="true">
-      <c r="A19" t="s" s="165">
-        <v>52</v>
-      </c>
-      <c r="B19" s="166"/>
-      <c r="C19" s="167"/>
-      <c r="D19" s="168"/>
-      <c r="E19" t="s" s="170">
-        <v>53</v>
-      </c>
-      <c r="F19" s="171"/>
-      <c r="G19" s="172"/>
-      <c r="H19" s="173"/>
+      <c r="A19" t="s" s="168">
+        <v>55</v>
+      </c>
+      <c r="B19" s="169"/>
+      <c r="C19" t="s" s="171">
+        <v>56</v>
+      </c>
+      <c r="D19" s="172"/>
+      <c r="E19" t="s" s="174">
+        <v>57</v>
+      </c>
+      <c r="F19" t="s" s="176">
+        <v>58</v>
+      </c>
+      <c r="G19" s="177"/>
+      <c r="H19" s="178"/>
     </row>
     <row r="20" ht="40.0" customHeight="true">
-      <c r="A20" t="s" s="174">
-        <v>54</v>
-      </c>
-      <c r="B20" s="175"/>
-      <c r="C20" t="s" s="177">
-        <v>55</v>
-      </c>
-      <c r="D20" s="178"/>
-      <c r="E20" s="179"/>
-      <c r="F20" s="180"/>
-      <c r="G20" s="181"/>
-      <c r="H20" s="182"/>
+      <c r="A20" t="s" s="179">
+        <v>59</v>
+      </c>
+      <c r="B20" s="180"/>
+      <c r="C20" t="s" s="182">
+        <v>60</v>
+      </c>
+      <c r="D20" s="183"/>
+      <c r="E20" s="184"/>
+      <c r="F20" s="185"/>
+      <c r="G20" s="186"/>
+      <c r="H20" s="187"/>
     </row>
     <row r="21" ht="40.0" customHeight="true">
-      <c r="A21" t="s" s="183">
-        <v>56</v>
-      </c>
-      <c r="B21" s="184"/>
-      <c r="C21" s="185"/>
-      <c r="D21" s="186"/>
-      <c r="E21" s="187"/>
-      <c r="F21" t="s" s="189">
-        <v>57</v>
-      </c>
-      <c r="G21" s="190"/>
-      <c r="H21" s="191"/>
+      <c r="A21" t="s" s="188">
+        <v>61</v>
+      </c>
+      <c r="B21" s="189"/>
+      <c r="C21" s="190"/>
+      <c r="D21" s="191"/>
+      <c r="E21" t="s" s="193">
+        <v>62</v>
+      </c>
+      <c r="F21" t="s" s="195">
+        <v>63</v>
+      </c>
+      <c r="G21" s="196"/>
+      <c r="H21" s="197"/>
     </row>
     <row r="22" ht="40.0" customHeight="true">
-      <c r="A22" t="s" s="192">
-        <v>58</v>
-      </c>
-      <c r="B22" s="193"/>
-      <c r="C22" t="s" s="195">
-        <v>59</v>
-      </c>
-      <c r="D22" s="196"/>
-      <c r="E22" s="197"/>
-      <c r="F22" s="198"/>
-      <c r="G22" s="199"/>
-      <c r="H22" s="200"/>
+      <c r="A22" t="s" s="198">
+        <v>64</v>
+      </c>
+      <c r="B22" s="199"/>
+      <c r="C22" t="s" s="201">
+        <v>65</v>
+      </c>
+      <c r="D22" s="202"/>
+      <c r="E22" s="203"/>
+      <c r="F22" s="204"/>
+      <c r="G22" s="205"/>
+      <c r="H22" s="206"/>
     </row>
     <row r="23" ht="40.0" customHeight="true">
-      <c r="A23" t="s" s="201">
-        <v>60</v>
-      </c>
-      <c r="B23" s="202"/>
-      <c r="C23" s="203"/>
-      <c r="D23" s="204"/>
-      <c r="E23" t="s" s="206">
-        <v>61</v>
-      </c>
-      <c r="F23" t="s" s="208">
-        <v>62</v>
-      </c>
-      <c r="G23" s="209"/>
-      <c r="H23" s="210"/>
+      <c r="A23" t="s" s="207">
+        <v>66</v>
+      </c>
+      <c r="B23" s="208"/>
+      <c r="C23" s="209"/>
+      <c r="D23" s="210"/>
+      <c r="E23" s="211"/>
+      <c r="F23" t="s" s="213">
+        <v>67</v>
+      </c>
+      <c r="G23" s="214"/>
+      <c r="H23" s="215"/>
     </row>
     <row r="24" ht="40.0" customHeight="true">
-      <c r="A24" t="s" s="211">
-        <v>63</v>
-      </c>
-      <c r="B24" s="212"/>
-      <c r="C24" t="s" s="214">
-        <v>64</v>
-      </c>
-      <c r="D24" s="215"/>
-      <c r="E24" s="216"/>
-      <c r="F24" s="217"/>
-      <c r="G24" s="218"/>
-      <c r="H24" s="219"/>
+      <c r="A24" t="s" s="216">
+        <v>68</v>
+      </c>
+      <c r="B24" s="217"/>
+      <c r="C24" s="218"/>
+      <c r="D24" t="s" s="220">
+        <v>69</v>
+      </c>
+      <c r="E24" t="s" s="222">
+        <v>70</v>
+      </c>
+      <c r="F24" s="223"/>
+      <c r="G24" s="224"/>
+      <c r="H24" s="225"/>
     </row>
     <row r="25" ht="40.0" customHeight="true">
-      <c r="A25" t="s" s="220">
-        <v>65</v>
-      </c>
-      <c r="B25" s="221"/>
-      <c r="C25" s="222"/>
-      <c r="D25" s="223"/>
-      <c r="E25" s="224"/>
-      <c r="F25" t="s" s="226">
-        <v>66</v>
-      </c>
-      <c r="G25" s="227"/>
-      <c r="H25" s="228"/>
+      <c r="A25" t="s" s="226">
+        <v>71</v>
+      </c>
+      <c r="B25" s="227"/>
+      <c r="C25" s="228"/>
+      <c r="D25" s="229"/>
+      <c r="E25" s="230"/>
+      <c r="F25" t="s" s="232">
+        <v>72</v>
+      </c>
+      <c r="G25" s="233"/>
+      <c r="H25" s="234"/>
     </row>
     <row r="26" ht="40.0" customHeight="true">
-      <c r="A26" t="s" s="229">
-        <v>67</v>
-      </c>
-      <c r="B26" s="230"/>
-      <c r="C26" s="231"/>
-      <c r="D26" t="s" s="233">
-        <v>68</v>
-      </c>
-      <c r="E26" t="s" s="235">
-        <v>69</v>
-      </c>
-      <c r="F26" s="236"/>
-      <c r="G26" s="237"/>
-      <c r="H26" s="238"/>
+      <c r="A26" t="s" s="235">
+        <v>73</v>
+      </c>
+      <c r="B26" s="236"/>
+      <c r="C26" t="s" s="238">
+        <v>74</v>
+      </c>
+      <c r="D26" s="239"/>
+      <c r="E26" s="240"/>
+      <c r="F26" s="241"/>
+      <c r="G26" s="242"/>
+      <c r="H26" s="243"/>
     </row>
     <row r="27" ht="40.0" customHeight="true">
-      <c r="A27" t="s" s="239">
-        <v>70</v>
-      </c>
-      <c r="B27" s="240"/>
-      <c r="C27" s="241"/>
-      <c r="D27" s="242"/>
-      <c r="E27" t="s" s="244">
-        <v>71</v>
-      </c>
-      <c r="F27" s="245"/>
-      <c r="G27" s="246"/>
-      <c r="H27" s="247"/>
+      <c r="A27" t="s" s="244">
+        <v>75</v>
+      </c>
+      <c r="B27" s="245"/>
+      <c r="C27" t="s" s="247">
+        <v>76</v>
+      </c>
+      <c r="D27" s="248"/>
+      <c r="E27" s="249"/>
+      <c r="F27" s="250"/>
+      <c r="G27" s="251"/>
+      <c r="H27" s="252"/>
     </row>
     <row r="28" ht="40.0" customHeight="true">
-      <c r="A28" t="s" s="248">
-        <v>72</v>
-      </c>
-      <c r="B28" s="249"/>
-      <c r="C28" s="250"/>
-      <c r="D28" s="251"/>
-      <c r="E28" t="s" s="253">
-        <v>73</v>
-      </c>
-      <c r="F28" s="254"/>
-      <c r="G28" s="255"/>
-      <c r="H28" s="256"/>
+      <c r="A28" t="s" s="253">
+        <v>77</v>
+      </c>
+      <c r="B28" s="254"/>
+      <c r="C28" s="255"/>
+      <c r="D28" s="256"/>
+      <c r="E28" s="257"/>
+      <c r="F28" t="s" s="259">
+        <v>78</v>
+      </c>
+      <c r="G28" s="260"/>
+      <c r="H28" s="261"/>
     </row>
     <row r="29" ht="40.0" customHeight="true">
-      <c r="A29" t="s" s="257">
-        <v>74</v>
-      </c>
-      <c r="B29" s="258"/>
-      <c r="C29" t="s" s="260">
-        <v>75</v>
-      </c>
-      <c r="D29" s="261"/>
-      <c r="E29" s="262"/>
-      <c r="F29" s="263"/>
-      <c r="G29" s="264"/>
-      <c r="H29" s="265"/>
+      <c r="A29" t="s" s="262">
+        <v>79</v>
+      </c>
+      <c r="B29" s="263"/>
+      <c r="C29" s="264"/>
+      <c r="D29" s="265"/>
+      <c r="E29" t="s" s="267">
+        <v>80</v>
+      </c>
+      <c r="F29" s="268"/>
+      <c r="G29" s="269"/>
+      <c r="H29" s="270"/>
     </row>
     <row r="30" ht="40.0" customHeight="true">
-      <c r="A30" t="s" s="266">
-        <v>76</v>
-      </c>
-      <c r="B30" s="267"/>
-      <c r="C30" s="268"/>
-      <c r="D30" s="269"/>
-      <c r="E30" s="270"/>
-      <c r="F30" t="s" s="272">
-        <v>77</v>
-      </c>
-      <c r="G30" s="273"/>
-      <c r="H30" t="s" s="275">
-        <v>78</v>
-      </c>
+      <c r="A30" t="s" s="271">
+        <v>81</v>
+      </c>
+      <c r="B30" s="272"/>
+      <c r="C30" t="s" s="274">
+        <v>82</v>
+      </c>
+      <c r="D30" s="275"/>
+      <c r="E30" s="276"/>
+      <c r="F30" s="277"/>
+      <c r="G30" s="278"/>
+      <c r="H30" s="279"/>
     </row>
     <row r="31" ht="40.0" customHeight="true">
-      <c r="A31" t="s" s="276">
-        <v>79</v>
-      </c>
-      <c r="B31" s="277"/>
-      <c r="C31" t="s" s="279">
-        <v>80</v>
-      </c>
-      <c r="D31" s="280"/>
-      <c r="E31" s="281"/>
-      <c r="F31" s="282"/>
-      <c r="G31" s="283"/>
-      <c r="H31" s="284"/>
+      <c r="A31" t="s" s="280">
+        <v>83</v>
+      </c>
+      <c r="B31" s="281"/>
+      <c r="C31" s="282"/>
+      <c r="D31" s="283"/>
+      <c r="E31" t="s" s="285">
+        <v>84</v>
+      </c>
+      <c r="F31" s="286"/>
+      <c r="G31" s="287"/>
+      <c r="H31" s="288"/>
     </row>
     <row r="32" ht="40.0" customHeight="true">
-      <c r="A32" t="s" s="285">
-        <v>81</v>
-      </c>
-      <c r="B32" s="286"/>
-      <c r="C32" s="287"/>
-      <c r="D32" s="288"/>
-      <c r="E32" t="s" s="290">
-        <v>82</v>
-      </c>
-      <c r="F32" s="291"/>
-      <c r="G32" t="s" s="293">
-        <v>83</v>
-      </c>
-      <c r="H32" s="294"/>
+      <c r="A32" t="s" s="289">
+        <v>85</v>
+      </c>
+      <c r="B32" s="290"/>
+      <c r="C32" s="291"/>
+      <c r="D32" s="292"/>
+      <c r="E32" s="293"/>
+      <c r="F32" t="s" s="295">
+        <v>86</v>
+      </c>
+      <c r="G32" s="296"/>
+      <c r="H32" s="297"/>
     </row>
     <row r="33" ht="40.0" customHeight="true">
-      <c r="A33" t="s" s="295">
-        <v>84</v>
-      </c>
-      <c r="B33" s="296"/>
-      <c r="C33" s="297"/>
-      <c r="D33" s="298"/>
-      <c r="E33" t="s" s="300">
-        <v>85</v>
-      </c>
-      <c r="F33" s="301"/>
-      <c r="G33" s="302"/>
-      <c r="H33" s="303"/>
+      <c r="A33" t="s" s="298">
+        <v>87</v>
+      </c>
+      <c r="B33" s="299"/>
+      <c r="C33" t="s" s="301">
+        <v>88</v>
+      </c>
+      <c r="D33" s="302"/>
+      <c r="E33" s="303"/>
+      <c r="F33" s="304"/>
+      <c r="G33" s="305"/>
+      <c r="H33" s="306"/>
     </row>
     <row r="34" ht="40.0" customHeight="true">
-      <c r="A34" t="s" s="304">
-        <v>86</v>
-      </c>
-      <c r="B34" s="305"/>
-      <c r="C34" t="s" s="307">
-        <v>87</v>
-      </c>
-      <c r="D34" s="308"/>
-      <c r="E34" s="309"/>
-      <c r="F34" s="310"/>
-      <c r="G34" s="311"/>
-      <c r="H34" s="312"/>
+      <c r="A34" t="s" s="307">
+        <v>89</v>
+      </c>
+      <c r="B34" s="308"/>
+      <c r="C34" t="s" s="310">
+        <v>90</v>
+      </c>
+      <c r="D34" s="311"/>
+      <c r="E34" s="312"/>
+      <c r="F34" s="313"/>
+      <c r="G34" s="314"/>
+      <c r="H34" s="315"/>
     </row>
     <row r="35" ht="40.0" customHeight="true">
-      <c r="A35" t="s" s="313">
-        <v>88</v>
-      </c>
-      <c r="B35" s="314"/>
-      <c r="C35" s="315"/>
-      <c r="D35" s="316"/>
-      <c r="E35" t="s" s="318">
-        <v>89</v>
-      </c>
-      <c r="F35" s="319"/>
-      <c r="G35" s="320"/>
-      <c r="H35" s="321"/>
+      <c r="A35" t="s" s="316">
+        <v>91</v>
+      </c>
+      <c r="B35" s="317"/>
+      <c r="C35" t="s" s="319">
+        <v>92</v>
+      </c>
+      <c r="D35" s="320"/>
+      <c r="E35" s="321"/>
+      <c r="F35" s="322"/>
+      <c r="G35" s="323"/>
+      <c r="H35" s="324"/>
     </row>
     <row r="36" ht="40.0" customHeight="true">
-      <c r="A36" t="s" s="322">
-        <v>90</v>
-      </c>
-      <c r="B36" s="323"/>
-      <c r="C36" t="s" s="325">
-        <v>91</v>
-      </c>
-      <c r="D36" s="326"/>
-      <c r="E36" s="327"/>
-      <c r="F36" s="328"/>
-      <c r="G36" s="329"/>
-      <c r="H36" s="330"/>
+      <c r="A36" t="s" s="325">
+        <v>93</v>
+      </c>
+      <c r="B36" s="326"/>
+      <c r="C36" s="327"/>
+      <c r="D36" s="328"/>
+      <c r="E36" s="329"/>
+      <c r="F36" t="s" s="331">
+        <v>94</v>
+      </c>
+      <c r="G36" s="332"/>
+      <c r="H36" s="333"/>
     </row>
     <row r="37" ht="40.0" customHeight="true">
-      <c r="A37" t="s" s="331">
-        <v>92</v>
-      </c>
-      <c r="B37" s="332"/>
-      <c r="C37" s="333"/>
-      <c r="D37" s="334"/>
-      <c r="E37" s="335"/>
-      <c r="F37" t="s" s="337">
-        <v>93</v>
-      </c>
-      <c r="G37" s="338"/>
-      <c r="H37" s="339"/>
+      <c r="A37" t="s" s="334">
+        <v>95</v>
+      </c>
+      <c r="B37" s="335"/>
+      <c r="C37" s="336"/>
+      <c r="D37" s="337"/>
+      <c r="E37" t="s" s="339">
+        <v>96</v>
+      </c>
+      <c r="F37" s="340"/>
+      <c r="G37" s="341"/>
+      <c r="H37" s="342"/>
     </row>
     <row r="38" ht="40.0" customHeight="true">
-      <c r="A38" t="s" s="340">
-        <v>94</v>
-      </c>
-      <c r="B38" s="341"/>
-      <c r="C38" t="s" s="343">
-        <v>95</v>
-      </c>
-      <c r="D38" s="344"/>
-      <c r="E38" s="345"/>
-      <c r="F38" s="346"/>
-      <c r="G38" s="347"/>
-      <c r="H38" s="348"/>
+      <c r="A38" t="s" s="343">
+        <v>97</v>
+      </c>
+      <c r="B38" s="344"/>
+      <c r="C38" t="s" s="346">
+        <v>98</v>
+      </c>
+      <c r="D38" s="347"/>
+      <c r="E38" s="348"/>
+      <c r="F38" s="349"/>
+      <c r="G38" s="350"/>
+      <c r="H38" s="351"/>
     </row>
     <row r="39" ht="40.0" customHeight="true">
-      <c r="A39" t="s" s="349">
-        <v>96</v>
-      </c>
-      <c r="B39" s="350"/>
-      <c r="C39" t="s" s="352">
-        <v>97</v>
-      </c>
-      <c r="D39" s="353"/>
-      <c r="E39" s="354"/>
-      <c r="F39" s="355"/>
-      <c r="G39" s="356"/>
-      <c r="H39" s="357"/>
+      <c r="A39" t="s" s="352">
+        <v>99</v>
+      </c>
+      <c r="B39" s="353"/>
+      <c r="C39" t="s" s="355">
+        <v>100</v>
+      </c>
+      <c r="D39" s="356"/>
+      <c r="E39" s="357"/>
+      <c r="F39" s="358"/>
+      <c r="G39" s="359"/>
+      <c r="H39" s="360"/>
     </row>
     <row r="40" ht="40.0" customHeight="true">
-      <c r="A40" t="s" s="358">
-        <v>98</v>
-      </c>
-      <c r="B40" s="359"/>
-      <c r="C40" s="360"/>
-      <c r="D40" s="361"/>
-      <c r="E40" s="362"/>
-      <c r="F40" t="s" s="364">
-        <v>99</v>
-      </c>
-      <c r="G40" s="365"/>
-      <c r="H40" s="366"/>
-    </row>
-    <row r="41" ht="40.0" customHeight="true">
-      <c r="A41" t="s" s="367">
-        <v>100</v>
-      </c>
-      <c r="B41" s="368"/>
-      <c r="C41" s="369"/>
-      <c r="D41" s="370"/>
-      <c r="E41" t="s" s="372">
+      <c r="A40" t="s" s="361">
         <v>101</v>
       </c>
-      <c r="F41" s="373"/>
-      <c r="G41" s="374"/>
-      <c r="H41" s="375"/>
-    </row>
-    <row r="42" ht="40.0" customHeight="true">
-      <c r="A42" t="s" s="376">
+      <c r="B40" s="362"/>
+      <c r="C40" s="363"/>
+      <c r="D40" s="364"/>
+      <c r="E40" t="s" s="366">
         <v>102</v>
       </c>
-      <c r="B42" s="377"/>
-      <c r="C42" t="s" s="379">
-        <v>103</v>
-      </c>
-      <c r="D42" s="380"/>
-      <c r="E42" s="381"/>
-      <c r="F42" s="382"/>
-      <c r="G42" s="383"/>
-      <c r="H42" s="384"/>
-    </row>
-    <row r="43" ht="40.0" customHeight="true">
-      <c r="A43" t="s" s="385">
-        <v>104</v>
-      </c>
-      <c r="B43" s="386"/>
-      <c r="C43" t="s" s="388">
-        <v>105</v>
-      </c>
-      <c r="D43" s="389"/>
-      <c r="E43" s="390"/>
-      <c r="F43" s="391"/>
-      <c r="G43" s="392"/>
-      <c r="H43" s="393"/>
-    </row>
-    <row r="44" ht="40.0" customHeight="true">
-      <c r="A44" t="s" s="394">
-        <v>106</v>
-      </c>
-      <c r="B44" s="395"/>
-      <c r="C44" s="396"/>
-      <c r="D44" s="397"/>
-      <c r="E44" s="398"/>
-      <c r="F44" t="s" s="400">
-        <v>107</v>
-      </c>
-      <c r="G44" s="401"/>
-      <c r="H44" s="402"/>
-    </row>
-    <row r="45" ht="40.0" customHeight="true">
-      <c r="A45" t="s" s="403">
-        <v>108</v>
-      </c>
-      <c r="B45" s="404"/>
-      <c r="C45" t="s" s="406">
-        <v>109</v>
-      </c>
-      <c r="D45" s="407"/>
-      <c r="E45" s="408"/>
-      <c r="F45" s="409"/>
-      <c r="G45" s="410"/>
-      <c r="H45" s="411"/>
-    </row>
-    <row r="46" ht="40.0" customHeight="true">
-      <c r="A46" t="s" s="412">
-        <v>110</v>
-      </c>
-      <c r="B46" s="413"/>
-      <c r="C46" s="414"/>
-      <c r="D46" s="415"/>
-      <c r="E46" t="s" s="417">
-        <v>111</v>
-      </c>
-      <c r="F46" s="418"/>
-      <c r="G46" s="419"/>
-      <c r="H46" s="420"/>
-    </row>
-    <row r="47" ht="40.0" customHeight="true">
-      <c r="A47" t="s" s="421">
-        <v>112</v>
-      </c>
-      <c r="B47" s="422"/>
-      <c r="C47" s="423"/>
-      <c r="D47" s="424"/>
-      <c r="E47" t="s" s="426">
-        <v>113</v>
-      </c>
-      <c r="F47" s="427"/>
-      <c r="G47" s="428"/>
-      <c r="H47" s="429"/>
-    </row>
-    <row r="48" ht="40.0" customHeight="true">
-      <c r="A48" t="s" s="430">
-        <v>114</v>
-      </c>
-      <c r="B48" s="431"/>
-      <c r="C48" t="s" s="433">
-        <v>115</v>
-      </c>
-      <c r="D48" s="434"/>
-      <c r="E48" s="435"/>
-      <c r="F48" s="436"/>
-      <c r="G48" s="437"/>
-      <c r="H48" s="438"/>
+      <c r="F40" s="367"/>
+      <c r="G40" s="368"/>
+      <c r="H40" s="369"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
Weitere updaes mit constraints
</commit_message>
<xml_diff>
--- a/Turnierplanung.xlsx
+++ b/Turnierplanung.xlsx
@@ -42,51 +42,52 @@
 2026-08-29</t>
   </si>
   <si>
-    <t>Leverkusen - QB_SEN_1 (QB)</t>
-  </si>
-  <si>
-    <t>Bonn - CHALLENGE_U15_8 (CHALLENGE)</t>
+    <t>Reutlingen - QB_SEN_2 (QB)</t>
+  </si>
+  <si>
+    <t>Rüsselsheim - DM_U15_16 (DM)</t>
   </si>
   <si>
     <t>KW 36
 2026-09-05</t>
   </si>
   <si>
-    <t>Erfurt - DM_VET_12 (DM)</t>
-  </si>
-  <si>
-    <t>Heidenheim - QB_U17_3 (QB)</t>
-  </si>
-  <si>
-    <t>Leverkusen - DM_U13_14 (DM)</t>
+    <t>Leipzig - QB_U17_4 (QB)</t>
   </si>
   <si>
     <t>KW 37
 2026-09-12</t>
   </si>
   <si>
-    <t>Offenbach - QB_U20_6 (QB)</t>
+    <t>Solingen - QB_U17_5 (QB)</t>
   </si>
   <si>
     <t>KW 38
 2026-09-19</t>
   </si>
   <si>
-    <t>Frankfurt - CHALLENGE_U15_9 (CHALLENGE)</t>
+    <t>Leverkusen - QB_SEN_1 (QB)</t>
   </si>
   <si>
     <t>KW 39
 2026-09-26</t>
   </si>
   <si>
-    <t>Reutlingen - QB_SEN_2 (QB)</t>
+    <t>Heidenheim - QB_U17_3 (QB)</t>
+  </si>
+  <si>
+    <t>KW 40
+2026-10-03</t>
+  </si>
+  <si>
+    <t>Leverkusen - DM_U17_13 (DM)</t>
   </si>
   <si>
     <t>KW 41
 2026-10-10</t>
   </si>
   <si>
-    <t>Waldkirch - CHALLENGE_U15_10 (CHALLENGE)</t>
+    <t>Heidelberg - QB_U20_7 (QB)</t>
   </si>
   <si>
     <t>KW 42
@@ -116,6 +117,13 @@
     <t>FIE - FIE_SanSalvador (FIE)</t>
   </si>
   <si>
+    <t>KW 45
+2026-11-07</t>
+  </si>
+  <si>
+    <t>Offenbach - QB_U20_6 (QB)</t>
+  </si>
+  <si>
     <t>Osnabrück - CHALLENGE_U15_11 (CHALLENGE)</t>
   </si>
   <si>
@@ -172,7 +180,7 @@
     <t>FIE - FIE_Tashkent (FIE)</t>
   </si>
   <si>
-    <t>Rüsselsheim - DM_U15_16 (DM)</t>
+    <t>Waldkirch - CHALLENGE_U15_10 (CHALLENGE)</t>
   </si>
   <si>
     <t>KW 51
@@ -250,11 +258,18 @@
     <t>FIE - FIE_Vrsac (FIE)</t>
   </si>
   <si>
+    <t>KW 8
+2027-02-27</t>
+  </si>
+  <si>
+    <t>Rüsselsheim - DM_U20_15 (DM)</t>
+  </si>
+  <si>
     <t>KW 9
 2027-03-06</t>
   </si>
   <si>
-    <t>Leipzig - QB_U17_4 (QB)</t>
+    <t>Leverkusen - DM_U13_14 (DM)</t>
   </si>
   <si>
     <t>KW 10
@@ -265,6 +280,9 @@
 EFC - EFC_Differdange (EFC)</t>
   </si>
   <si>
+    <t>Frankfurt - CHALLENGE_U15_9 (CHALLENGE)</t>
+  </si>
+  <si>
     <t>KW 12
 2027-03-27</t>
   </si>
@@ -273,13 +291,6 @@
 EFC - EFC_Daugavpils (EFC)</t>
   </si>
   <si>
-    <t>KW 13
-2027-04-03</t>
-  </si>
-  <si>
-    <t>Solingen - QB_U17_5 (QB)</t>
-  </si>
-  <si>
     <t>KW 14
 2027-04-10</t>
   </si>
@@ -298,6 +309,9 @@
 2027-04-24</t>
   </si>
   <si>
+    <t>Erfurt - DM_VET_12 (DM)</t>
+  </si>
+  <si>
     <t>EFC - EFC_EM_U20 (EFC)</t>
   </si>
   <si>
@@ -305,7 +319,7 @@
 2027-05-01</t>
   </si>
   <si>
-    <t>Leverkusen - DM_U17_13 (DM)</t>
+    <t>Bonn - CHALLENGE_U15_8 (CHALLENGE)</t>
   </si>
   <si>
     <t>KW 18
@@ -337,13 +351,6 @@
     <t>EFC - EFC_EM_U17 (EFC)</t>
   </si>
   <si>
-    <t>KW 24
-2027-06-19</t>
-  </si>
-  <si>
-    <t>Heidelberg - QB_U20_7 (QB)</t>
-  </si>
-  <si>
     <t>KW 25
 2027-06-26</t>
   </si>
@@ -356,13 +363,6 @@
   </si>
   <si>
     <t>FIE - FIE_WM_Senioren (FIE)</t>
-  </si>
-  <si>
-    <t>KW 29
-2027-07-24</t>
-  </si>
-  <si>
-    <t>Rüsselsheim - DM_U20_15 (DM)</t>
   </si>
 </sst>
 </file>
@@ -730,12 +730,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
@@ -859,10 +853,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -877,10 +871,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -916,16 +907,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -940,25 +928,22 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -976,10 +961,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1003,7 +991,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1030,25 +1021,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1066,22 +1051,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1096,19 +1078,25 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1126,13 +1114,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1150,13 +1144,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1177,25 +1171,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1237,7 +1225,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1300,7 +1291,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1321,19 +1315,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1360,10 +1351,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1378,16 +1369,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1405,10 +1399,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1459,16 +1453,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1486,10 +1483,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1519,10 +1516,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1540,10 +1537,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1567,16 +1564,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1594,10 +1594,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1621,10 +1621,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1648,19 +1648,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1675,10 +1675,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1711,10 +1711,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1729,10 +1729,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1756,10 +1756,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1842,464 +1842,464 @@
       <c r="A3" t="s" s="12">
         <v>11</v>
       </c>
-      <c r="B3" t="s" s="14">
+      <c r="B3" s="13"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="16"/>
+      <c r="F3" t="s" s="18">
         <v>12</v>
       </c>
-      <c r="C3" s="15"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="17"/>
-      <c r="F3" t="s" s="19">
+      <c r="G3" s="19"/>
+      <c r="H3" s="20"/>
+    </row>
+    <row r="4" ht="40.0" customHeight="true">
+      <c r="A4" t="s" s="21">
         <v>13</v>
       </c>
-      <c r="G3" s="20"/>
-      <c r="H3" t="s" s="22">
+      <c r="B4" s="22"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="25"/>
+      <c r="F4" t="s" s="27">
         <v>14</v>
       </c>
-    </row>
-    <row r="4" ht="40.0" customHeight="true">
-      <c r="A4" t="s" s="23">
+      <c r="G4" s="28"/>
+      <c r="H4" s="29"/>
+    </row>
+    <row r="5" ht="40.0" customHeight="true">
+      <c r="A5" t="s" s="30">
         <v>15</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="26"/>
-      <c r="E4" t="s" s="28">
+      <c r="B5" s="31"/>
+      <c r="C5" t="s" s="33">
         <v>16</v>
       </c>
-      <c r="F4" s="29"/>
-      <c r="G4" s="30"/>
-      <c r="H4" s="31"/>
-    </row>
-    <row r="5" ht="40.0" customHeight="true">
-      <c r="A5" t="s" s="32">
+      <c r="D5" s="34"/>
+      <c r="E5" s="35"/>
+      <c r="F5" s="36"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="38"/>
+    </row>
+    <row r="6" ht="40.0" customHeight="true">
+      <c r="A6" t="s" s="39">
         <v>17</v>
       </c>
-      <c r="B5" s="33"/>
-      <c r="C5" s="34"/>
-      <c r="D5" s="35"/>
-      <c r="E5" s="36"/>
-      <c r="F5" s="37"/>
-      <c r="G5" t="s" s="39">
+      <c r="B6" s="40"/>
+      <c r="C6" s="41"/>
+      <c r="D6" s="42"/>
+      <c r="E6" s="43"/>
+      <c r="F6" t="s" s="45">
         <v>18</v>
       </c>
-      <c r="H5" s="40"/>
-    </row>
-    <row r="6" ht="40.0" customHeight="true">
-      <c r="A6" t="s" s="41">
+      <c r="G6" s="46"/>
+      <c r="H6" s="47"/>
+    </row>
+    <row r="7" ht="40.0" customHeight="true">
+      <c r="A7" t="s" s="48">
         <v>19</v>
       </c>
-      <c r="B6" s="42"/>
-      <c r="C6" t="s" s="44">
+      <c r="B7" s="49"/>
+      <c r="C7" s="50"/>
+      <c r="D7" s="51"/>
+      <c r="E7" s="52"/>
+      <c r="F7" t="s" s="54">
         <v>20</v>
       </c>
-      <c r="D6" s="45"/>
-      <c r="E6" s="46"/>
-      <c r="F6" s="47"/>
-      <c r="G6" s="48"/>
-      <c r="H6" s="49"/>
-    </row>
-    <row r="7" ht="40.0" customHeight="true">
-      <c r="A7" t="s" s="50">
+      <c r="G7" s="55"/>
+      <c r="H7" s="56"/>
+    </row>
+    <row r="8" ht="40.0" customHeight="true">
+      <c r="A8" t="s" s="57">
         <v>21</v>
       </c>
-      <c r="B7" s="51"/>
-      <c r="C7" s="52"/>
-      <c r="D7" s="53"/>
-      <c r="E7" s="54"/>
-      <c r="F7" s="55"/>
-      <c r="G7" t="s" s="57">
+      <c r="B8" s="58"/>
+      <c r="C8" s="59"/>
+      <c r="D8" s="60"/>
+      <c r="E8" t="s" s="62">
         <v>22</v>
       </c>
-      <c r="H7" s="58"/>
-    </row>
-    <row r="8" ht="40.0" customHeight="true">
-      <c r="A8" t="s" s="59">
+      <c r="F8" s="63"/>
+      <c r="G8" s="64"/>
+      <c r="H8" s="65"/>
+    </row>
+    <row r="9" ht="40.0" customHeight="true">
+      <c r="A9" t="s" s="66">
         <v>23</v>
       </c>
-      <c r="B8" s="60"/>
-      <c r="C8" s="61"/>
-      <c r="D8" s="62"/>
-      <c r="E8" s="63"/>
-      <c r="F8" t="s" s="65">
+      <c r="B9" s="67"/>
+      <c r="C9" s="68"/>
+      <c r="D9" s="69"/>
+      <c r="E9" s="70"/>
+      <c r="F9" t="s" s="72">
         <v>24</v>
       </c>
-      <c r="G8" s="66"/>
-      <c r="H8" s="67"/>
-    </row>
-    <row r="9" ht="40.0" customHeight="true">
-      <c r="A9" t="s" s="68">
+      <c r="G9" s="73"/>
+      <c r="H9" s="74"/>
+    </row>
+    <row r="10" ht="40.0" customHeight="true">
+      <c r="A10" t="s" s="75">
         <v>25</v>
       </c>
-      <c r="B9" s="69"/>
-      <c r="C9" t="s" s="71">
+      <c r="B10" s="76"/>
+      <c r="C10" t="s" s="78">
         <v>26</v>
       </c>
-      <c r="D9" s="72"/>
-      <c r="E9" s="73"/>
-      <c r="F9" t="s" s="75">
+      <c r="D10" s="79"/>
+      <c r="E10" s="80"/>
+      <c r="F10" t="s" s="82">
         <v>27</v>
       </c>
-      <c r="G9" s="76"/>
-      <c r="H9" s="77"/>
-    </row>
-    <row r="10" ht="40.0" customHeight="true">
-      <c r="A10" t="s" s="78">
+      <c r="G10" s="83"/>
+      <c r="H10" s="84"/>
+    </row>
+    <row r="11" ht="40.0" customHeight="true">
+      <c r="A11" t="s" s="85">
         <v>28</v>
       </c>
-      <c r="B10" s="79"/>
-      <c r="C10" t="s" s="81">
+      <c r="B11" s="86"/>
+      <c r="C11" t="s" s="88">
         <v>29</v>
       </c>
-      <c r="D10" s="82"/>
-      <c r="E10" t="s" s="84">
+      <c r="D11" s="89"/>
+      <c r="E11" t="s" s="91">
         <v>30</v>
       </c>
-      <c r="F10" s="85"/>
-      <c r="G10" t="s" s="87">
+      <c r="F11" s="92"/>
+      <c r="G11" s="93"/>
+      <c r="H11" s="94"/>
+    </row>
+    <row r="12" ht="40.0" customHeight="true">
+      <c r="A12" t="s" s="95">
         <v>31</v>
       </c>
-      <c r="H10" s="88"/>
-    </row>
-    <row r="11" ht="40.0" customHeight="true">
-      <c r="A11" t="s" s="89">
+      <c r="B12" s="96"/>
+      <c r="C12" s="97"/>
+      <c r="D12" s="98"/>
+      <c r="E12" t="s" s="100">
         <v>32</v>
       </c>
-      <c r="B11" s="90"/>
-      <c r="C11" s="91"/>
-      <c r="D11" t="s" s="93">
+      <c r="F12" s="101"/>
+      <c r="G12" t="s" s="103">
         <v>33</v>
       </c>
-      <c r="E11" t="s" s="95">
+      <c r="H12" s="104"/>
+    </row>
+    <row r="13" ht="40.0" customHeight="true">
+      <c r="A13" t="s" s="105">
         <v>34</v>
       </c>
-      <c r="F11" t="s" s="97">
+      <c r="B13" s="106"/>
+      <c r="C13" s="107"/>
+      <c r="D13" t="s" s="109">
         <v>35</v>
       </c>
-      <c r="G11" s="98"/>
-      <c r="H11" s="99"/>
-    </row>
-    <row r="12" ht="40.0" customHeight="true">
-      <c r="A12" t="s" s="100">
+      <c r="E13" t="s" s="111">
         <v>36</v>
       </c>
-      <c r="B12" s="101"/>
-      <c r="C12" s="102"/>
-      <c r="D12" t="s" s="104">
+      <c r="F13" t="s" s="113">
         <v>37</v>
       </c>
-      <c r="E12" s="105"/>
-      <c r="F12" s="106"/>
-      <c r="G12" s="107"/>
-      <c r="H12" s="108"/>
-    </row>
-    <row r="13" ht="40.0" customHeight="true">
-      <c r="A13" t="s" s="109">
+      <c r="G13" s="114"/>
+      <c r="H13" s="115"/>
+    </row>
+    <row r="14" ht="40.0" customHeight="true">
+      <c r="A14" t="s" s="116">
         <v>38</v>
       </c>
-      <c r="B13" s="110"/>
-      <c r="C13" s="111"/>
-      <c r="D13" s="112"/>
-      <c r="E13" t="s" s="114">
+      <c r="B14" s="117"/>
+      <c r="C14" s="118"/>
+      <c r="D14" t="s" s="120">
         <v>39</v>
       </c>
-      <c r="F13" t="s" s="116">
+      <c r="E14" s="121"/>
+      <c r="F14" s="122"/>
+      <c r="G14" s="123"/>
+      <c r="H14" s="124"/>
+    </row>
+    <row r="15" ht="40.0" customHeight="true">
+      <c r="A15" t="s" s="125">
         <v>40</v>
       </c>
-      <c r="G13" s="117"/>
-      <c r="H13" s="118"/>
-    </row>
-    <row r="14" ht="40.0" customHeight="true">
-      <c r="A14" t="s" s="119">
+      <c r="B15" s="126"/>
+      <c r="C15" s="127"/>
+      <c r="D15" s="128"/>
+      <c r="E15" t="s" s="130">
         <v>41</v>
       </c>
-      <c r="B14" s="120"/>
-      <c r="C14" t="s" s="122">
+      <c r="F15" t="s" s="132">
         <v>42</v>
       </c>
-      <c r="D14" t="s" s="124">
+      <c r="G15" s="133"/>
+      <c r="H15" s="134"/>
+    </row>
+    <row r="16" ht="40.0" customHeight="true">
+      <c r="A16" t="s" s="135">
         <v>43</v>
       </c>
-      <c r="E14" s="125"/>
-      <c r="F14" t="s" s="127">
+      <c r="B16" s="136"/>
+      <c r="C16" t="s" s="138">
         <v>44</v>
       </c>
-      <c r="G14" s="128"/>
-      <c r="H14" s="129"/>
-    </row>
-    <row r="15" ht="40.0" customHeight="true">
-      <c r="A15" t="s" s="130">
+      <c r="D16" t="s" s="140">
         <v>45</v>
       </c>
-      <c r="B15" s="131"/>
-      <c r="C15" s="132"/>
-      <c r="D15" t="s" s="134">
+      <c r="E16" s="141"/>
+      <c r="F16" t="s" s="143">
         <v>46</v>
       </c>
-      <c r="E15" t="s" s="136">
+      <c r="G16" s="144"/>
+      <c r="H16" s="145"/>
+    </row>
+    <row r="17" ht="40.0" customHeight="true">
+      <c r="A17" t="s" s="146">
         <v>47</v>
       </c>
-      <c r="F15" s="137"/>
-      <c r="G15" t="s" s="139">
+      <c r="B17" s="147"/>
+      <c r="C17" s="148"/>
+      <c r="D17" t="s" s="150">
         <v>48</v>
       </c>
-      <c r="H15" s="140"/>
-    </row>
-    <row r="16" ht="40.0" customHeight="true">
-      <c r="A16" t="s" s="141">
+      <c r="E17" t="s" s="152">
         <v>49</v>
       </c>
-      <c r="B16" s="142"/>
-      <c r="C16" s="143"/>
-      <c r="D16" t="s" s="145">
+      <c r="F17" s="153"/>
+      <c r="G17" t="s" s="155">
         <v>50</v>
       </c>
-      <c r="E16" s="146"/>
-      <c r="F16" s="147"/>
-      <c r="G16" s="148"/>
-      <c r="H16" s="149"/>
-    </row>
-    <row r="17" ht="40.0" customHeight="true">
-      <c r="A17" t="s" s="150">
+      <c r="H17" s="156"/>
+    </row>
+    <row r="18" ht="40.0" customHeight="true">
+      <c r="A18" t="s" s="157">
         <v>51</v>
       </c>
-      <c r="B17" s="151"/>
-      <c r="C17" s="152"/>
-      <c r="D17" s="153"/>
-      <c r="E17" t="s" s="155">
+      <c r="B18" s="158"/>
+      <c r="C18" s="159"/>
+      <c r="D18" t="s" s="161">
         <v>52</v>
       </c>
-      <c r="F17" s="156"/>
-      <c r="G17" s="157"/>
-      <c r="H17" s="158"/>
-    </row>
-    <row r="18" ht="40.0" customHeight="true">
-      <c r="A18" t="s" s="159">
+      <c r="E18" s="162"/>
+      <c r="F18" s="163"/>
+      <c r="G18" s="164"/>
+      <c r="H18" s="165"/>
+    </row>
+    <row r="19" ht="40.0" customHeight="true">
+      <c r="A19" t="s" s="166">
         <v>53</v>
       </c>
-      <c r="B18" s="160"/>
-      <c r="C18" t="s" s="162">
+      <c r="B19" s="167"/>
+      <c r="C19" s="168"/>
+      <c r="D19" s="169"/>
+      <c r="E19" t="s" s="171">
         <v>54</v>
       </c>
-      <c r="D18" s="163"/>
-      <c r="E18" s="164"/>
-      <c r="F18" s="165"/>
-      <c r="G18" s="166"/>
-      <c r="H18" s="167"/>
-    </row>
-    <row r="19" ht="40.0" customHeight="true">
-      <c r="A19" t="s" s="168">
+      <c r="F19" s="172"/>
+      <c r="G19" s="173"/>
+      <c r="H19" s="174"/>
+    </row>
+    <row r="20" ht="40.0" customHeight="true">
+      <c r="A20" t="s" s="175">
         <v>55</v>
       </c>
-      <c r="B19" s="169"/>
-      <c r="C19" t="s" s="171">
+      <c r="B20" s="176"/>
+      <c r="C20" t="s" s="178">
         <v>56</v>
       </c>
-      <c r="D19" s="172"/>
-      <c r="E19" t="s" s="174">
+      <c r="D20" s="179"/>
+      <c r="E20" s="180"/>
+      <c r="F20" s="181"/>
+      <c r="G20" s="182"/>
+      <c r="H20" s="183"/>
+    </row>
+    <row r="21" ht="40.0" customHeight="true">
+      <c r="A21" t="s" s="184">
         <v>57</v>
       </c>
-      <c r="F19" t="s" s="176">
+      <c r="B21" s="185"/>
+      <c r="C21" t="s" s="187">
         <v>58</v>
       </c>
-      <c r="G19" s="177"/>
-      <c r="H19" s="178"/>
-    </row>
-    <row r="20" ht="40.0" customHeight="true">
-      <c r="A20" t="s" s="179">
+      <c r="D21" s="188"/>
+      <c r="E21" t="s" s="190">
         <v>59</v>
       </c>
-      <c r="B20" s="180"/>
-      <c r="C20" t="s" s="182">
+      <c r="F21" t="s" s="192">
         <v>60</v>
       </c>
-      <c r="D20" s="183"/>
-      <c r="E20" s="184"/>
-      <c r="F20" s="185"/>
-      <c r="G20" s="186"/>
-      <c r="H20" s="187"/>
-    </row>
-    <row r="21" ht="40.0" customHeight="true">
-      <c r="A21" t="s" s="188">
+      <c r="G21" s="193"/>
+      <c r="H21" s="194"/>
+    </row>
+    <row r="22" ht="40.0" customHeight="true">
+      <c r="A22" t="s" s="195">
         <v>61</v>
       </c>
-      <c r="B21" s="189"/>
-      <c r="C21" s="190"/>
-      <c r="D21" s="191"/>
-      <c r="E21" t="s" s="193">
+      <c r="B22" s="196"/>
+      <c r="C22" t="s" s="198">
         <v>62</v>
       </c>
-      <c r="F21" t="s" s="195">
+      <c r="D22" s="199"/>
+      <c r="E22" s="200"/>
+      <c r="F22" s="201"/>
+      <c r="G22" s="202"/>
+      <c r="H22" s="203"/>
+    </row>
+    <row r="23" ht="40.0" customHeight="true">
+      <c r="A23" t="s" s="204">
         <v>63</v>
       </c>
-      <c r="G21" s="196"/>
-      <c r="H21" s="197"/>
-    </row>
-    <row r="22" ht="40.0" customHeight="true">
-      <c r="A22" t="s" s="198">
+      <c r="B23" s="205"/>
+      <c r="C23" s="206"/>
+      <c r="D23" s="207"/>
+      <c r="E23" t="s" s="209">
         <v>64</v>
       </c>
-      <c r="B22" s="199"/>
-      <c r="C22" t="s" s="201">
+      <c r="F23" t="s" s="211">
         <v>65</v>
       </c>
-      <c r="D22" s="202"/>
-      <c r="E22" s="203"/>
-      <c r="F22" s="204"/>
-      <c r="G22" s="205"/>
-      <c r="H22" s="206"/>
-    </row>
-    <row r="23" ht="40.0" customHeight="true">
-      <c r="A23" t="s" s="207">
+      <c r="G23" s="212"/>
+      <c r="H23" s="213"/>
+    </row>
+    <row r="24" ht="40.0" customHeight="true">
+      <c r="A24" t="s" s="214">
         <v>66</v>
       </c>
-      <c r="B23" s="208"/>
-      <c r="C23" s="209"/>
-      <c r="D23" s="210"/>
-      <c r="E23" s="211"/>
-      <c r="F23" t="s" s="213">
+      <c r="B24" s="215"/>
+      <c r="C24" t="s" s="217">
         <v>67</v>
       </c>
-      <c r="G23" s="214"/>
-      <c r="H23" s="215"/>
-    </row>
-    <row r="24" ht="40.0" customHeight="true">
-      <c r="A24" t="s" s="216">
+      <c r="D24" s="218"/>
+      <c r="E24" s="219"/>
+      <c r="F24" s="220"/>
+      <c r="G24" s="221"/>
+      <c r="H24" s="222"/>
+    </row>
+    <row r="25" ht="40.0" customHeight="true">
+      <c r="A25" t="s" s="223">
         <v>68</v>
       </c>
-      <c r="B24" s="217"/>
-      <c r="C24" s="218"/>
-      <c r="D24" t="s" s="220">
+      <c r="B25" s="224"/>
+      <c r="C25" s="225"/>
+      <c r="D25" s="226"/>
+      <c r="E25" s="227"/>
+      <c r="F25" t="s" s="229">
         <v>69</v>
       </c>
-      <c r="E24" t="s" s="222">
+      <c r="G25" s="230"/>
+      <c r="H25" s="231"/>
+    </row>
+    <row r="26" ht="40.0" customHeight="true">
+      <c r="A26" t="s" s="232">
         <v>70</v>
       </c>
-      <c r="F24" s="223"/>
-      <c r="G24" s="224"/>
-      <c r="H24" s="225"/>
-    </row>
-    <row r="25" ht="40.0" customHeight="true">
-      <c r="A25" t="s" s="226">
+      <c r="B26" s="233"/>
+      <c r="C26" s="234"/>
+      <c r="D26" t="s" s="236">
         <v>71</v>
       </c>
-      <c r="B25" s="227"/>
-      <c r="C25" s="228"/>
-      <c r="D25" s="229"/>
-      <c r="E25" s="230"/>
-      <c r="F25" t="s" s="232">
+      <c r="E26" t="s" s="238">
         <v>72</v>
       </c>
-      <c r="G25" s="233"/>
-      <c r="H25" s="234"/>
-    </row>
-    <row r="26" ht="40.0" customHeight="true">
-      <c r="A26" t="s" s="235">
+      <c r="F26" s="239"/>
+      <c r="G26" s="240"/>
+      <c r="H26" s="241"/>
+    </row>
+    <row r="27" ht="40.0" customHeight="true">
+      <c r="A27" t="s" s="242">
         <v>73</v>
       </c>
-      <c r="B26" s="236"/>
-      <c r="C26" t="s" s="238">
+      <c r="B27" s="243"/>
+      <c r="C27" s="244"/>
+      <c r="D27" s="245"/>
+      <c r="E27" t="s" s="247">
         <v>74</v>
       </c>
-      <c r="D26" s="239"/>
-      <c r="E26" s="240"/>
-      <c r="F26" s="241"/>
-      <c r="G26" s="242"/>
-      <c r="H26" s="243"/>
-    </row>
-    <row r="27" ht="40.0" customHeight="true">
-      <c r="A27" t="s" s="244">
+      <c r="F27" s="248"/>
+      <c r="G27" s="249"/>
+      <c r="H27" s="250"/>
+    </row>
+    <row r="28" ht="40.0" customHeight="true">
+      <c r="A28" t="s" s="251">
         <v>75</v>
       </c>
-      <c r="B27" s="245"/>
-      <c r="C27" t="s" s="247">
+      <c r="B28" s="252"/>
+      <c r="C28" s="253"/>
+      <c r="D28" s="254"/>
+      <c r="E28" s="255"/>
+      <c r="F28" s="256"/>
+      <c r="G28" s="257"/>
+      <c r="H28" t="s" s="259">
         <v>76</v>
       </c>
-      <c r="D27" s="248"/>
-      <c r="E27" s="249"/>
-      <c r="F27" s="250"/>
-      <c r="G27" s="251"/>
-      <c r="H27" s="252"/>
-    </row>
-    <row r="28" ht="40.0" customHeight="true">
-      <c r="A28" t="s" s="253">
+    </row>
+    <row r="29" ht="40.0" customHeight="true">
+      <c r="A29" t="s" s="260">
         <v>77</v>
       </c>
-      <c r="B28" s="254"/>
-      <c r="C28" s="255"/>
-      <c r="D28" s="256"/>
-      <c r="E28" s="257"/>
-      <c r="F28" t="s" s="259">
+      <c r="B29" s="261"/>
+      <c r="C29" t="s" s="263">
         <v>78</v>
       </c>
-      <c r="G28" s="260"/>
-      <c r="H28" s="261"/>
-    </row>
-    <row r="29" ht="40.0" customHeight="true">
-      <c r="A29" t="s" s="262">
+      <c r="D29" s="264"/>
+      <c r="E29" s="265"/>
+      <c r="F29" s="266"/>
+      <c r="G29" t="s" s="268">
         <v>79</v>
       </c>
-      <c r="B29" s="263"/>
-      <c r="C29" s="264"/>
-      <c r="D29" s="265"/>
-      <c r="E29" t="s" s="267">
+      <c r="H29" s="269"/>
+    </row>
+    <row r="30" ht="40.0" customHeight="true">
+      <c r="A30" t="s" s="270">
         <v>80</v>
       </c>
-      <c r="F29" s="268"/>
-      <c r="G29" s="269"/>
-      <c r="H29" s="270"/>
-    </row>
-    <row r="30" ht="40.0" customHeight="true">
-      <c r="A30" t="s" s="271">
+      <c r="B30" s="271"/>
+      <c r="C30" t="s" s="273">
         <v>81</v>
       </c>
-      <c r="B30" s="272"/>
-      <c r="C30" t="s" s="274">
+      <c r="D30" s="274"/>
+      <c r="E30" s="275"/>
+      <c r="F30" s="276"/>
+      <c r="G30" s="277"/>
+      <c r="H30" s="278"/>
+    </row>
+    <row r="31" ht="40.0" customHeight="true">
+      <c r="A31" t="s" s="279">
         <v>82</v>
       </c>
-      <c r="D30" s="275"/>
-      <c r="E30" s="276"/>
-      <c r="F30" s="277"/>
-      <c r="G30" s="278"/>
-      <c r="H30" s="279"/>
-    </row>
-    <row r="31" ht="40.0" customHeight="true">
-      <c r="A31" t="s" s="280">
+      <c r="B31" s="280"/>
+      <c r="C31" s="281"/>
+      <c r="D31" s="282"/>
+      <c r="E31" t="s" s="284">
         <v>83</v>
       </c>
-      <c r="B31" s="281"/>
-      <c r="C31" s="282"/>
-      <c r="D31" s="283"/>
-      <c r="E31" t="s" s="285">
+      <c r="F31" s="285"/>
+      <c r="G31" s="286"/>
+      <c r="H31" s="287"/>
+    </row>
+    <row r="32" ht="40.0" customHeight="true">
+      <c r="A32" t="s" s="288">
         <v>84</v>
       </c>
-      <c r="F31" s="286"/>
-      <c r="G31" s="287"/>
-      <c r="H31" s="288"/>
-    </row>
-    <row r="32" ht="40.0" customHeight="true">
-      <c r="A32" t="s" s="289">
+      <c r="B32" s="289"/>
+      <c r="C32" t="s" s="291">
         <v>85</v>
       </c>
-      <c r="B32" s="290"/>
-      <c r="C32" s="291"/>
       <c r="D32" s="292"/>
       <c r="E32" s="293"/>
-      <c r="F32" t="s" s="295">
+      <c r="F32" s="294"/>
+      <c r="G32" s="295"/>
+      <c r="H32" s="296"/>
+    </row>
+    <row r="33" ht="40.0" customHeight="true">
+      <c r="A33" t="s" s="297">
         <v>86</v>
       </c>
-      <c r="G32" s="296"/>
-      <c r="H32" s="297"/>
-    </row>
-    <row r="33" ht="40.0" customHeight="true">
-      <c r="A33" t="s" s="298">
+      <c r="B33" t="s" s="299">
         <v>87</v>
       </c>
-      <c r="B33" s="299"/>
-      <c r="C33" t="s" s="301">
+      <c r="C33" s="300"/>
+      <c r="D33" s="301"/>
+      <c r="E33" t="s" s="303">
         <v>88</v>
       </c>
-      <c r="D33" s="302"/>
-      <c r="E33" s="303"/>
       <c r="F33" s="304"/>
       <c r="G33" s="305"/>
       <c r="H33" s="306"/>
@@ -2309,13 +2309,13 @@
         <v>89</v>
       </c>
       <c r="B34" s="308"/>
-      <c r="C34" t="s" s="310">
+      <c r="C34" s="309"/>
+      <c r="D34" s="310"/>
+      <c r="E34" s="311"/>
+      <c r="F34" s="312"/>
+      <c r="G34" t="s" s="314">
         <v>90</v>
       </c>
-      <c r="D34" s="311"/>
-      <c r="E34" s="312"/>
-      <c r="F34" s="313"/>
-      <c r="G34" s="314"/>
       <c r="H34" s="315"/>
     </row>
     <row r="35" ht="40.0" customHeight="true">
@@ -2337,12 +2337,12 @@
         <v>93</v>
       </c>
       <c r="B36" s="326"/>
-      <c r="C36" s="327"/>
-      <c r="D36" s="328"/>
-      <c r="E36" s="329"/>
-      <c r="F36" t="s" s="331">
+      <c r="C36" t="s" s="328">
         <v>94</v>
       </c>
+      <c r="D36" s="329"/>
+      <c r="E36" s="330"/>
+      <c r="F36" s="331"/>
       <c r="G36" s="332"/>
       <c r="H36" s="333"/>
     </row>
@@ -2351,11 +2351,11 @@
         <v>95</v>
       </c>
       <c r="B37" s="335"/>
-      <c r="C37" s="336"/>
-      <c r="D37" s="337"/>
-      <c r="E37" t="s" s="339">
+      <c r="C37" t="s" s="337">
         <v>96</v>
       </c>
+      <c r="D37" s="338"/>
+      <c r="E37" s="339"/>
       <c r="F37" s="340"/>
       <c r="G37" s="341"/>
       <c r="H37" s="342"/>
@@ -2365,12 +2365,12 @@
         <v>97</v>
       </c>
       <c r="B38" s="344"/>
-      <c r="C38" t="s" s="346">
+      <c r="C38" s="345"/>
+      <c r="D38" s="346"/>
+      <c r="E38" s="347"/>
+      <c r="F38" t="s" s="349">
         <v>98</v>
       </c>
-      <c r="D38" s="347"/>
-      <c r="E38" s="348"/>
-      <c r="F38" s="349"/>
       <c r="G38" s="350"/>
       <c r="H38" s="351"/>
     </row>
@@ -2393,11 +2393,11 @@
         <v>101</v>
       </c>
       <c r="B40" s="362"/>
-      <c r="C40" s="363"/>
-      <c r="D40" s="364"/>
-      <c r="E40" t="s" s="366">
+      <c r="C40" t="s" s="364">
         <v>102</v>
       </c>
+      <c r="D40" s="365"/>
+      <c r="E40" s="366"/>
       <c r="F40" s="367"/>
       <c r="G40" s="368"/>
       <c r="H40" s="369"/>

</xml_diff>

<commit_message>
Explain score, Update Venue availability
</commit_message>
<xml_diff>
--- a/Turnierplanung.xlsx
+++ b/Turnierplanung.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="104">
   <si>
     <t>Wochenende (KW)</t>
   </si>
@@ -45,35 +45,38 @@
     <t>Reutlingen - QB_SEN_2 (QB)</t>
   </si>
   <si>
-    <t>Rüsselsheim - DM_U15_16 (DM)</t>
-  </si>
-  <si>
     <t>KW 36
 2026-09-05</t>
   </si>
   <si>
-    <t>Leipzig - QB_U17_4 (QB)</t>
+    <t>Heidenheim - QB_U17_3 (QB)</t>
+  </si>
+  <si>
+    <t>Leverkusen - DM_U13_14 (DM)</t>
   </si>
   <si>
     <t>KW 37
 2026-09-12</t>
   </si>
   <si>
-    <t>Solingen - QB_U17_5 (QB)</t>
+    <t>Leverkusen - QB_SEN_1 (QB)</t>
   </si>
   <si>
     <t>KW 38
 2026-09-19</t>
   </si>
   <si>
-    <t>Leverkusen - QB_SEN_1 (QB)</t>
+    <t>Erfurt - DM_VET_12 (DM)</t>
+  </si>
+  <si>
+    <t>Leipzig - QB_U17_4 (QB)</t>
   </si>
   <si>
     <t>KW 39
 2026-09-26</t>
   </si>
   <si>
-    <t>Heidenheim - QB_U17_3 (QB)</t>
+    <t>Solingen - QB_U17_5 (QB)</t>
   </si>
   <si>
     <t>KW 40
@@ -124,9 +127,6 @@
     <t>Offenbach - QB_U20_6 (QB)</t>
   </si>
   <si>
-    <t>Osnabrück - CHALLENGE_U15_11 (CHALLENGE)</t>
-  </si>
-  <si>
     <t>KW 46
 2026-11-14</t>
   </si>
@@ -180,9 +180,6 @@
     <t>FIE - FIE_Tashkent (FIE)</t>
   </si>
   <si>
-    <t>Waldkirch - CHALLENGE_U15_10 (CHALLENGE)</t>
-  </si>
-  <si>
     <t>KW 51
 2026-12-19</t>
   </si>
@@ -190,6 +187,9 @@
     <t>EFC - EFC_Thessaloniki (EFC)</t>
   </si>
   <si>
+    <t>Rüsselsheim - DM_U15_16 (DM)</t>
+  </si>
+  <si>
     <t>KW 53
 2027-01-02</t>
   </si>
@@ -269,7 +269,7 @@
 2027-03-06</t>
   </si>
   <si>
-    <t>Leverkusen - DM_U13_14 (DM)</t>
+    <t>Osnabrück - CHALLENGE_U15_11 (CHALLENGE)</t>
   </si>
   <si>
     <t>KW 10
@@ -280,9 +280,6 @@
 EFC - EFC_Differdange (EFC)</t>
   </si>
   <si>
-    <t>Frankfurt - CHALLENGE_U15_9 (CHALLENGE)</t>
-  </si>
-  <si>
     <t>KW 12
 2027-03-27</t>
   </si>
@@ -298,6 +295,9 @@
     <t>FIE - FIE_WM_U20 (FIE)</t>
   </si>
   <si>
+    <t>Waldkirch - CHALLENGE_U15_10 (CHALLENGE)</t>
+  </si>
+  <si>
     <t>KW 15
 2027-04-17</t>
   </si>
@@ -309,17 +309,7 @@
 2027-04-24</t>
   </si>
   <si>
-    <t>Erfurt - DM_VET_12 (DM)</t>
-  </si>
-  <si>
     <t>EFC - EFC_EM_U20 (EFC)</t>
-  </si>
-  <si>
-    <t>KW 17
-2027-05-01</t>
-  </si>
-  <si>
-    <t>Bonn - CHALLENGE_U15_8 (CHALLENGE)</t>
   </si>
   <si>
     <t>KW 18
@@ -329,6 +319,13 @@
     <t>FIE - FIE_Medellin (FIE)</t>
   </si>
   <si>
+    <t>KW 19
+2027-05-15</t>
+  </si>
+  <si>
+    <t>Frankfurt - CHALLENGE_U15_9 (CHALLENGE)</t>
+  </si>
+  <si>
     <t>KW 20
 2027-05-22</t>
   </si>
@@ -363,6 +360,13 @@
   </si>
   <si>
     <t>FIE - FIE_WM_Senioren (FIE)</t>
+  </si>
+  <si>
+    <t>KW 31
+2027-08-07</t>
+  </si>
+  <si>
+    <t>Bonn - CHALLENGE_U15_8 (CHALLENGE)</t>
   </si>
 </sst>
 </file>
@@ -370,7 +374,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="41">
+  <fonts count="42">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
@@ -383,6 +387,11 @@
       <sz val="11.0"/>
       <b val="true"/>
       <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -668,7 +677,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="370">
+  <cellXfs count="378">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="true" applyFill="true" applyAlignment="true" applyBorder="true">
       <alignment horizontal="center" vertical="center"/>
@@ -700,9 +709,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
@@ -730,6 +736,9 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
@@ -784,6 +793,9 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
@@ -979,9 +991,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
@@ -1135,9 +1144,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
@@ -1165,6 +1171,9 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
     <xf numFmtId="0" fontId="19" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
@@ -1474,9 +1483,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
     <xf numFmtId="0" fontId="30" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
@@ -1531,6 +1537,9 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
     <xf numFmtId="0" fontId="32" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
@@ -1570,9 +1579,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
@@ -1594,10 +1600,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1621,10 +1627,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1760,6 +1766,33 @@
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
+      <alignment horizontal="center" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1783,7 +1816,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="25.0" customWidth="true"/>
@@ -1833,36 +1866,36 @@
       <c r="D2" s="6"/>
       <c r="E2" s="7"/>
       <c r="F2" s="8"/>
-      <c r="G2" t="s" s="10">
+      <c r="G2" s="9"/>
+      <c r="H2" s="10"/>
+    </row>
+    <row r="3" ht="40.0" customHeight="true">
+      <c r="A3" t="s" s="11">
         <v>10</v>
       </c>
-      <c r="H2" s="11"/>
-    </row>
-    <row r="3" ht="40.0" customHeight="true">
-      <c r="A3" t="s" s="12">
+      <c r="B3" s="12"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="15"/>
+      <c r="F3" t="s" s="17">
         <v>11</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="16"/>
-      <c r="F3" t="s" s="18">
+      <c r="G3" s="18"/>
+      <c r="H3" t="s" s="20">
         <v>12</v>
       </c>
-      <c r="G3" s="19"/>
-      <c r="H3" s="20"/>
     </row>
     <row r="4" ht="40.0" customHeight="true">
       <c r="A4" t="s" s="21">
         <v>13</v>
       </c>
       <c r="B4" s="22"/>
-      <c r="C4" s="23"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="25"/>
-      <c r="F4" t="s" s="27">
+      <c r="C4" t="s" s="24">
         <v>14</v>
       </c>
+      <c r="D4" s="25"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="27"/>
       <c r="G4" s="28"/>
       <c r="H4" s="29"/>
     </row>
@@ -1870,118 +1903,118 @@
       <c r="A5" t="s" s="30">
         <v>15</v>
       </c>
-      <c r="B5" s="31"/>
-      <c r="C5" t="s" s="33">
+      <c r="B5" t="s" s="32">
         <v>16</v>
       </c>
+      <c r="C5" s="33"/>
       <c r="D5" s="34"/>
       <c r="E5" s="35"/>
-      <c r="F5" s="36"/>
-      <c r="G5" s="37"/>
-      <c r="H5" s="38"/>
+      <c r="F5" t="s" s="37">
+        <v>17</v>
+      </c>
+      <c r="G5" s="38"/>
+      <c r="H5" s="39"/>
     </row>
     <row r="6" ht="40.0" customHeight="true">
-      <c r="A6" t="s" s="39">
-        <v>17</v>
-      </c>
-      <c r="B6" s="40"/>
-      <c r="C6" s="41"/>
-      <c r="D6" s="42"/>
-      <c r="E6" s="43"/>
-      <c r="F6" t="s" s="45">
+      <c r="A6" t="s" s="40">
         <v>18</v>
       </c>
-      <c r="G6" s="46"/>
-      <c r="H6" s="47"/>
+      <c r="B6" s="41"/>
+      <c r="C6" s="42"/>
+      <c r="D6" s="43"/>
+      <c r="E6" s="44"/>
+      <c r="F6" t="s" s="46">
+        <v>19</v>
+      </c>
+      <c r="G6" s="47"/>
+      <c r="H6" s="48"/>
     </row>
     <row r="7" ht="40.0" customHeight="true">
-      <c r="A7" t="s" s="48">
-        <v>19</v>
-      </c>
-      <c r="B7" s="49"/>
-      <c r="C7" s="50"/>
-      <c r="D7" s="51"/>
-      <c r="E7" s="52"/>
-      <c r="F7" t="s" s="54">
+      <c r="A7" t="s" s="49">
         <v>20</v>
       </c>
-      <c r="G7" s="55"/>
-      <c r="H7" s="56"/>
+      <c r="B7" s="50"/>
+      <c r="C7" s="51"/>
+      <c r="D7" s="52"/>
+      <c r="E7" s="53"/>
+      <c r="F7" t="s" s="55">
+        <v>21</v>
+      </c>
+      <c r="G7" s="56"/>
+      <c r="H7" s="57"/>
     </row>
     <row r="8" ht="40.0" customHeight="true">
-      <c r="A8" t="s" s="57">
-        <v>21</v>
-      </c>
-      <c r="B8" s="58"/>
-      <c r="C8" s="59"/>
-      <c r="D8" s="60"/>
-      <c r="E8" t="s" s="62">
+      <c r="A8" t="s" s="58">
         <v>22</v>
       </c>
-      <c r="F8" s="63"/>
-      <c r="G8" s="64"/>
-      <c r="H8" s="65"/>
+      <c r="B8" s="59"/>
+      <c r="C8" s="60"/>
+      <c r="D8" s="61"/>
+      <c r="E8" t="s" s="63">
+        <v>23</v>
+      </c>
+      <c r="F8" s="64"/>
+      <c r="G8" s="65"/>
+      <c r="H8" s="66"/>
     </row>
     <row r="9" ht="40.0" customHeight="true">
-      <c r="A9" t="s" s="66">
-        <v>23</v>
-      </c>
-      <c r="B9" s="67"/>
-      <c r="C9" s="68"/>
-      <c r="D9" s="69"/>
-      <c r="E9" s="70"/>
-      <c r="F9" t="s" s="72">
+      <c r="A9" t="s" s="67">
         <v>24</v>
       </c>
-      <c r="G9" s="73"/>
-      <c r="H9" s="74"/>
+      <c r="B9" s="68"/>
+      <c r="C9" s="69"/>
+      <c r="D9" s="70"/>
+      <c r="E9" s="71"/>
+      <c r="F9" t="s" s="73">
+        <v>25</v>
+      </c>
+      <c r="G9" s="74"/>
+      <c r="H9" s="75"/>
     </row>
     <row r="10" ht="40.0" customHeight="true">
-      <c r="A10" t="s" s="75">
-        <v>25</v>
-      </c>
-      <c r="B10" s="76"/>
-      <c r="C10" t="s" s="78">
+      <c r="A10" t="s" s="76">
         <v>26</v>
       </c>
-      <c r="D10" s="79"/>
-      <c r="E10" s="80"/>
-      <c r="F10" t="s" s="82">
+      <c r="B10" s="77"/>
+      <c r="C10" t="s" s="79">
         <v>27</v>
       </c>
-      <c r="G10" s="83"/>
-      <c r="H10" s="84"/>
+      <c r="D10" s="80"/>
+      <c r="E10" s="81"/>
+      <c r="F10" t="s" s="83">
+        <v>28</v>
+      </c>
+      <c r="G10" s="84"/>
+      <c r="H10" s="85"/>
     </row>
     <row r="11" ht="40.0" customHeight="true">
-      <c r="A11" t="s" s="85">
-        <v>28</v>
-      </c>
-      <c r="B11" s="86"/>
-      <c r="C11" t="s" s="88">
+      <c r="A11" t="s" s="86">
         <v>29</v>
       </c>
-      <c r="D11" s="89"/>
-      <c r="E11" t="s" s="91">
+      <c r="B11" s="87"/>
+      <c r="C11" t="s" s="89">
         <v>30</v>
       </c>
-      <c r="F11" s="92"/>
-      <c r="G11" s="93"/>
-      <c r="H11" s="94"/>
+      <c r="D11" s="90"/>
+      <c r="E11" t="s" s="92">
+        <v>31</v>
+      </c>
+      <c r="F11" s="93"/>
+      <c r="G11" s="94"/>
+      <c r="H11" s="95"/>
     </row>
     <row r="12" ht="40.0" customHeight="true">
-      <c r="A12" t="s" s="95">
-        <v>31</v>
-      </c>
-      <c r="B12" s="96"/>
-      <c r="C12" s="97"/>
-      <c r="D12" s="98"/>
-      <c r="E12" t="s" s="100">
+      <c r="A12" t="s" s="96">
         <v>32</v>
       </c>
-      <c r="F12" s="101"/>
-      <c r="G12" t="s" s="103">
+      <c r="B12" s="97"/>
+      <c r="C12" s="98"/>
+      <c r="D12" s="99"/>
+      <c r="E12" t="s" s="101">
         <v>33</v>
       </c>
+      <c r="F12" s="102"/>
+      <c r="G12" s="103"/>
       <c r="H12" s="104"/>
     </row>
     <row r="13" ht="40.0" customHeight="true">
@@ -2063,23 +2096,23 @@
         <v>49</v>
       </c>
       <c r="F17" s="153"/>
-      <c r="G17" t="s" s="155">
+      <c r="G17" s="154"/>
+      <c r="H17" s="155"/>
+    </row>
+    <row r="18" ht="40.0" customHeight="true">
+      <c r="A18" t="s" s="156">
         <v>50</v>
       </c>
-      <c r="H17" s="156"/>
-    </row>
-    <row r="18" ht="40.0" customHeight="true">
-      <c r="A18" t="s" s="157">
+      <c r="B18" s="157"/>
+      <c r="C18" s="158"/>
+      <c r="D18" t="s" s="160">
         <v>51</v>
       </c>
-      <c r="B18" s="158"/>
-      <c r="C18" s="159"/>
-      <c r="D18" t="s" s="161">
+      <c r="E18" s="161"/>
+      <c r="F18" s="162"/>
+      <c r="G18" t="s" s="164">
         <v>52</v>
       </c>
-      <c r="E18" s="162"/>
-      <c r="F18" s="163"/>
-      <c r="G18" s="164"/>
       <c r="H18" s="165"/>
     </row>
     <row r="19" ht="40.0" customHeight="true">
@@ -2225,10 +2258,10 @@
       <c r="D28" s="254"/>
       <c r="E28" s="255"/>
       <c r="F28" s="256"/>
-      <c r="G28" s="257"/>
-      <c r="H28" t="s" s="259">
+      <c r="G28" t="s" s="258">
         <v>76</v>
       </c>
+      <c r="H28" s="259"/>
     </row>
     <row r="29" ht="40.0" customHeight="true">
       <c r="A29" t="s" s="260">
@@ -2241,37 +2274,37 @@
       <c r="D29" s="264"/>
       <c r="E29" s="265"/>
       <c r="F29" s="266"/>
-      <c r="G29" t="s" s="268">
+      <c r="G29" s="267"/>
+      <c r="H29" s="268"/>
+    </row>
+    <row r="30" ht="40.0" customHeight="true">
+      <c r="A30" t="s" s="269">
         <v>79</v>
       </c>
-      <c r="H29" s="269"/>
-    </row>
-    <row r="30" ht="40.0" customHeight="true">
-      <c r="A30" t="s" s="270">
+      <c r="B30" s="270"/>
+      <c r="C30" t="s" s="272">
         <v>80</v>
       </c>
-      <c r="B30" s="271"/>
-      <c r="C30" t="s" s="273">
+      <c r="D30" s="273"/>
+      <c r="E30" s="274"/>
+      <c r="F30" s="275"/>
+      <c r="G30" s="276"/>
+      <c r="H30" s="277"/>
+    </row>
+    <row r="31" ht="40.0" customHeight="true">
+      <c r="A31" t="s" s="278">
         <v>81</v>
       </c>
-      <c r="D30" s="274"/>
-      <c r="E30" s="275"/>
-      <c r="F30" s="276"/>
-      <c r="G30" s="277"/>
-      <c r="H30" s="278"/>
-    </row>
-    <row r="31" ht="40.0" customHeight="true">
-      <c r="A31" t="s" s="279">
+      <c r="B31" s="279"/>
+      <c r="C31" s="280"/>
+      <c r="D31" s="281"/>
+      <c r="E31" t="s" s="283">
         <v>82</v>
       </c>
-      <c r="B31" s="280"/>
-      <c r="C31" s="281"/>
-      <c r="D31" s="282"/>
-      <c r="E31" t="s" s="284">
+      <c r="F31" s="284"/>
+      <c r="G31" t="s" s="286">
         <v>83</v>
       </c>
-      <c r="F31" s="285"/>
-      <c r="G31" s="286"/>
       <c r="H31" s="287"/>
     </row>
     <row r="32" ht="40.0" customHeight="true">
@@ -2292,115 +2325,127 @@
       <c r="A33" t="s" s="297">
         <v>86</v>
       </c>
-      <c r="B33" t="s" s="299">
+      <c r="B33" s="298"/>
+      <c r="C33" s="299"/>
+      <c r="D33" s="300"/>
+      <c r="E33" t="s" s="302">
         <v>87</v>
       </c>
-      <c r="C33" s="300"/>
-      <c r="D33" s="301"/>
-      <c r="E33" t="s" s="303">
+      <c r="F33" s="303"/>
+      <c r="G33" s="304"/>
+      <c r="H33" s="305"/>
+    </row>
+    <row r="34" ht="40.0" customHeight="true">
+      <c r="A34" t="s" s="306">
         <v>88</v>
       </c>
-      <c r="F33" s="304"/>
-      <c r="G33" s="305"/>
-      <c r="H33" s="306"/>
-    </row>
-    <row r="34" ht="40.0" customHeight="true">
-      <c r="A34" t="s" s="307">
+      <c r="B34" s="307"/>
+      <c r="C34" t="s" s="309">
         <v>89</v>
       </c>
-      <c r="B34" s="308"/>
-      <c r="C34" s="309"/>
       <c r="D34" s="310"/>
       <c r="E34" s="311"/>
       <c r="F34" s="312"/>
-      <c r="G34" t="s" s="314">
+      <c r="G34" s="313"/>
+      <c r="H34" s="314"/>
+    </row>
+    <row r="35" ht="40.0" customHeight="true">
+      <c r="A35" t="s" s="315">
         <v>90</v>
       </c>
-      <c r="H34" s="315"/>
-    </row>
-    <row r="35" ht="40.0" customHeight="true">
-      <c r="A35" t="s" s="316">
+      <c r="B35" s="316"/>
+      <c r="C35" s="317"/>
+      <c r="D35" s="318"/>
+      <c r="E35" s="319"/>
+      <c r="F35" s="320"/>
+      <c r="G35" t="s" s="322">
         <v>91</v>
       </c>
-      <c r="B35" s="317"/>
-      <c r="C35" t="s" s="319">
+      <c r="H35" s="323"/>
+    </row>
+    <row r="36" ht="40.0" customHeight="true">
+      <c r="A36" t="s" s="324">
         <v>92</v>
       </c>
-      <c r="D35" s="320"/>
-      <c r="E35" s="321"/>
-      <c r="F35" s="322"/>
-      <c r="G35" s="323"/>
-      <c r="H35" s="324"/>
-    </row>
-    <row r="36" ht="40.0" customHeight="true">
-      <c r="A36" t="s" s="325">
+      <c r="B36" s="325"/>
+      <c r="C36" t="s" s="327">
         <v>93</v>
       </c>
-      <c r="B36" s="326"/>
-      <c r="C36" t="s" s="328">
+      <c r="D36" s="328"/>
+      <c r="E36" s="329"/>
+      <c r="F36" s="330"/>
+      <c r="G36" s="331"/>
+      <c r="H36" s="332"/>
+    </row>
+    <row r="37" ht="40.0" customHeight="true">
+      <c r="A37" t="s" s="333">
         <v>94</v>
       </c>
-      <c r="D36" s="329"/>
-      <c r="E36" s="330"/>
-      <c r="F36" s="331"/>
-      <c r="G36" s="332"/>
-      <c r="H36" s="333"/>
-    </row>
-    <row r="37" ht="40.0" customHeight="true">
-      <c r="A37" t="s" s="334">
+      <c r="B37" s="334"/>
+      <c r="C37" t="s" s="336">
         <v>95</v>
       </c>
-      <c r="B37" s="335"/>
-      <c r="C37" t="s" s="337">
+      <c r="D37" s="337"/>
+      <c r="E37" s="338"/>
+      <c r="F37" s="339"/>
+      <c r="G37" s="340"/>
+      <c r="H37" s="341"/>
+    </row>
+    <row r="38" ht="40.0" customHeight="true">
+      <c r="A38" t="s" s="342">
         <v>96</v>
       </c>
-      <c r="D37" s="338"/>
-      <c r="E37" s="339"/>
-      <c r="F37" s="340"/>
-      <c r="G37" s="341"/>
-      <c r="H37" s="342"/>
-    </row>
-    <row r="38" ht="40.0" customHeight="true">
-      <c r="A38" t="s" s="343">
+      <c r="B38" s="343"/>
+      <c r="C38" s="344"/>
+      <c r="D38" s="345"/>
+      <c r="E38" s="346"/>
+      <c r="F38" t="s" s="348">
         <v>97</v>
       </c>
-      <c r="B38" s="344"/>
-      <c r="C38" s="345"/>
-      <c r="D38" s="346"/>
-      <c r="E38" s="347"/>
-      <c r="F38" t="s" s="349">
+      <c r="G38" s="349"/>
+      <c r="H38" s="350"/>
+    </row>
+    <row r="39" ht="40.0" customHeight="true">
+      <c r="A39" t="s" s="351">
         <v>98</v>
       </c>
-      <c r="G38" s="350"/>
-      <c r="H38" s="351"/>
-    </row>
-    <row r="39" ht="40.0" customHeight="true">
-      <c r="A39" t="s" s="352">
+      <c r="B39" s="352"/>
+      <c r="C39" t="s" s="354">
         <v>99</v>
       </c>
-      <c r="B39" s="353"/>
-      <c r="C39" t="s" s="355">
+      <c r="D39" s="355"/>
+      <c r="E39" s="356"/>
+      <c r="F39" s="357"/>
+      <c r="G39" s="358"/>
+      <c r="H39" s="359"/>
+    </row>
+    <row r="40" ht="40.0" customHeight="true">
+      <c r="A40" t="s" s="360">
         <v>100</v>
       </c>
-      <c r="D39" s="356"/>
-      <c r="E39" s="357"/>
-      <c r="F39" s="358"/>
-      <c r="G39" s="359"/>
-      <c r="H39" s="360"/>
-    </row>
-    <row r="40" ht="40.0" customHeight="true">
-      <c r="A40" t="s" s="361">
+      <c r="B40" s="361"/>
+      <c r="C40" t="s" s="363">
         <v>101</v>
       </c>
-      <c r="B40" s="362"/>
-      <c r="C40" t="s" s="364">
+      <c r="D40" s="364"/>
+      <c r="E40" s="365"/>
+      <c r="F40" s="366"/>
+      <c r="G40" s="367"/>
+      <c r="H40" s="368"/>
+    </row>
+    <row r="41" ht="40.0" customHeight="true">
+      <c r="A41" t="s" s="369">
         <v>102</v>
       </c>
-      <c r="D40" s="365"/>
-      <c r="E40" s="366"/>
-      <c r="F40" s="367"/>
-      <c r="G40" s="368"/>
-      <c r="H40" s="369"/>
+      <c r="B41" s="370"/>
+      <c r="C41" s="371"/>
+      <c r="D41" s="372"/>
+      <c r="E41" s="373"/>
+      <c r="F41" s="374"/>
+      <c r="G41" t="s" s="376">
+        <v>103</v>
+      </c>
+      <c r="H41" s="377"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
Update Fix 2.1. und beschränkungen weekends veranstalter
</commit_message>
<xml_diff>
--- a/Turnierplanung.xlsx
+++ b/Turnierplanung.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="103">
   <si>
     <t>Wochenende (KW)</t>
   </si>
@@ -36,13 +36,6 @@
   </si>
   <si>
     <t>U13</t>
-  </si>
-  <si>
-    <t>KW 35
-2026-08-29</t>
-  </si>
-  <si>
-    <t>Reutlingen - QB_SEN_2 (QB)</t>
   </si>
   <si>
     <t>KW 36
@@ -52,9 +45,6 @@
     <t>Heidenheim - QB_U17_3 (QB)</t>
   </si>
   <si>
-    <t>Leverkusen - DM_U13_14 (DM)</t>
-  </si>
-  <si>
     <t>KW 37
 2026-09-12</t>
   </si>
@@ -66,9 +56,6 @@
 2026-09-19</t>
   </si>
   <si>
-    <t>Erfurt - DM_VET_12 (DM)</t>
-  </si>
-  <si>
     <t>Leipzig - QB_U17_4 (QB)</t>
   </si>
   <si>
@@ -90,7 +77,7 @@
 2026-10-10</t>
   </si>
   <si>
-    <t>Heidelberg - QB_U20_7 (QB)</t>
+    <t>Reutlingen - QB_SEN_2 (QB)</t>
   </si>
   <si>
     <t>KW 42
@@ -124,6 +111,9 @@
 2026-11-07</t>
   </si>
   <si>
+    <t>Erfurt - DM_VET_12 (DM)</t>
+  </si>
+  <si>
     <t>Offenbach - QB_U20_6 (QB)</t>
   </si>
   <si>
@@ -187,9 +177,6 @@
     <t>EFC - EFC_Thessaloniki (EFC)</t>
   </si>
   <si>
-    <t>Rüsselsheim - DM_U15_16 (DM)</t>
-  </si>
-  <si>
     <t>KW 53
 2027-01-02</t>
   </si>
@@ -248,6 +235,9 @@
     <t>EFC - EFC_Krakow (EFC)</t>
   </si>
   <si>
+    <t>Leverkusen - DM_U13_14 (DM)</t>
+  </si>
+  <si>
     <t>KW 7
 2027-02-20</t>
   </si>
@@ -262,7 +252,7 @@
 2027-02-27</t>
   </si>
   <si>
-    <t>Rüsselsheim - DM_U20_15 (DM)</t>
+    <t>Heidelberg - QB_U20_7 (QB)</t>
   </si>
   <si>
     <t>KW 9
@@ -280,6 +270,9 @@
 EFC - EFC_Differdange (EFC)</t>
   </si>
   <si>
+    <t>Frankfurt - CHALLENGE_U15_9 (CHALLENGE)</t>
+  </si>
+  <si>
     <t>KW 12
 2027-03-27</t>
   </si>
@@ -288,6 +281,16 @@
 EFC - EFC_Daugavpils (EFC)</t>
   </si>
   <si>
+    <t>KW 13
+2027-04-03</t>
+  </si>
+  <si>
+    <t>Rüsselsheim - DM_U20_15 (DM)</t>
+  </si>
+  <si>
+    <t>Rüsselsheim - DM_U15_16 (DM)</t>
+  </si>
+  <si>
     <t>KW 14
 2027-04-10</t>
   </si>
@@ -319,13 +322,6 @@
     <t>FIE - FIE_Medellin (FIE)</t>
   </si>
   <si>
-    <t>KW 19
-2027-05-15</t>
-  </si>
-  <si>
-    <t>Frankfurt - CHALLENGE_U15_9 (CHALLENGE)</t>
-  </si>
-  <si>
     <t>KW 20
 2027-05-22</t>
   </si>
@@ -348,6 +344,13 @@
     <t>EFC - EFC_EM_U17 (EFC)</t>
   </si>
   <si>
+    <t>KW 24
+2027-06-19</t>
+  </si>
+  <si>
+    <t>Bonn - CHALLENGE_U15_8 (CHALLENGE)</t>
+  </si>
+  <si>
     <t>KW 25
 2027-06-26</t>
   </si>
@@ -360,13 +363,6 @@
   </si>
   <si>
     <t>FIE - FIE_WM_Senioren (FIE)</t>
-  </si>
-  <si>
-    <t>KW 31
-2027-08-07</t>
-  </si>
-  <si>
-    <t>Bonn - CHALLENGE_U15_8 (CHALLENGE)</t>
   </si>
 </sst>
 </file>
@@ -374,7 +370,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="42">
+  <fonts count="41">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
@@ -387,11 +383,6 @@
       <sz val="11.0"/>
       <b val="true"/>
       <color indexed="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -677,7 +668,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="378">
+  <cellXfs count="370">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="true" applyFill="true" applyAlignment="true" applyBorder="true">
       <alignment horizontal="center" vertical="center"/>
@@ -736,9 +727,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
@@ -793,9 +781,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
@@ -865,10 +850,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -883,7 +868,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -919,13 +907,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -940,19 +928,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -973,16 +961,22 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1006,16 +1000,10 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1033,16 +1021,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1057,16 +1048,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1087,25 +1081,22 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1129,10 +1120,7 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1153,16 +1141,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1180,16 +1165,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1207,19 +1192,25 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1234,25 +1225,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1267,19 +1252,22 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1294,22 +1282,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1324,16 +1309,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1354,16 +1342,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1381,16 +1372,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1435,7 +1423,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1489,10 +1480,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1627,10 +1621,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1654,10 +1648,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1681,19 +1675,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1717,10 +1711,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1766,33 +1760,6 @@
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
-      <alignment horizontal="center" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1816,7 +1783,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="25.0" customWidth="true"/>
@@ -1860,12 +1827,12 @@
         <v>8</v>
       </c>
       <c r="B2" s="3"/>
-      <c r="C2" t="s" s="5">
+      <c r="C2" s="4"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="6"/>
+      <c r="F2" t="s" s="8">
         <v>9</v>
       </c>
-      <c r="D2" s="6"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="8"/>
       <c r="G2" s="9"/>
       <c r="H2" s="10"/>
     </row>
@@ -1874,178 +1841,178 @@
         <v>10</v>
       </c>
       <c r="B3" s="12"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="15"/>
-      <c r="F3" t="s" s="17">
+      <c r="C3" t="s" s="14">
         <v>11</v>
       </c>
+      <c r="D3" s="15"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="17"/>
       <c r="G3" s="18"/>
-      <c r="H3" t="s" s="20">
+      <c r="H3" s="19"/>
+    </row>
+    <row r="4" ht="40.0" customHeight="true">
+      <c r="A4" t="s" s="20">
         <v>12</v>
       </c>
-    </row>
-    <row r="4" ht="40.0" customHeight="true">
-      <c r="A4" t="s" s="21">
+      <c r="B4" s="21"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="24"/>
+      <c r="F4" t="s" s="26">
         <v>13</v>
       </c>
-      <c r="B4" s="22"/>
-      <c r="C4" t="s" s="24">
+      <c r="G4" s="27"/>
+      <c r="H4" s="28"/>
+    </row>
+    <row r="5" ht="40.0" customHeight="true">
+      <c r="A5" t="s" s="29">
         <v>14</v>
       </c>
-      <c r="D4" s="25"/>
-      <c r="E4" s="26"/>
-      <c r="F4" s="27"/>
-      <c r="G4" s="28"/>
-      <c r="H4" s="29"/>
-    </row>
-    <row r="5" ht="40.0" customHeight="true">
-      <c r="A5" t="s" s="30">
+      <c r="B5" s="30"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="33"/>
+      <c r="F5" t="s" s="35">
         <v>15</v>
       </c>
-      <c r="B5" t="s" s="32">
+      <c r="G5" s="36"/>
+      <c r="H5" s="37"/>
+    </row>
+    <row r="6" ht="40.0" customHeight="true">
+      <c r="A6" t="s" s="38">
         <v>16</v>
       </c>
-      <c r="C5" s="33"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="35"/>
-      <c r="F5" t="s" s="37">
+      <c r="B6" s="39"/>
+      <c r="C6" s="40"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="42"/>
+      <c r="F6" t="s" s="44">
         <v>17</v>
       </c>
-      <c r="G5" s="38"/>
-      <c r="H5" s="39"/>
-    </row>
-    <row r="6" ht="40.0" customHeight="true">
-      <c r="A6" t="s" s="40">
+      <c r="G6" s="45"/>
+      <c r="H6" s="46"/>
+    </row>
+    <row r="7" ht="40.0" customHeight="true">
+      <c r="A7" t="s" s="47">
         <v>18</v>
       </c>
-      <c r="B6" s="41"/>
-      <c r="C6" s="42"/>
-      <c r="D6" s="43"/>
-      <c r="E6" s="44"/>
-      <c r="F6" t="s" s="46">
+      <c r="B7" s="48"/>
+      <c r="C7" t="s" s="50">
         <v>19</v>
       </c>
-      <c r="G6" s="47"/>
-      <c r="H6" s="48"/>
-    </row>
-    <row r="7" ht="40.0" customHeight="true">
-      <c r="A7" t="s" s="49">
+      <c r="D7" s="51"/>
+      <c r="E7" s="52"/>
+      <c r="F7" s="53"/>
+      <c r="G7" s="54"/>
+      <c r="H7" s="55"/>
+    </row>
+    <row r="8" ht="40.0" customHeight="true">
+      <c r="A8" t="s" s="56">
         <v>20</v>
       </c>
-      <c r="B7" s="50"/>
-      <c r="C7" s="51"/>
-      <c r="D7" s="52"/>
-      <c r="E7" s="53"/>
-      <c r="F7" t="s" s="55">
+      <c r="B8" s="57"/>
+      <c r="C8" s="58"/>
+      <c r="D8" s="59"/>
+      <c r="E8" s="60"/>
+      <c r="F8" t="s" s="62">
         <v>21</v>
       </c>
-      <c r="G7" s="56"/>
-      <c r="H7" s="57"/>
-    </row>
-    <row r="8" ht="40.0" customHeight="true">
-      <c r="A8" t="s" s="58">
+      <c r="G8" s="63"/>
+      <c r="H8" s="64"/>
+    </row>
+    <row r="9" ht="40.0" customHeight="true">
+      <c r="A9" t="s" s="65">
         <v>22</v>
       </c>
-      <c r="B8" s="59"/>
-      <c r="C8" s="60"/>
-      <c r="D8" s="61"/>
-      <c r="E8" t="s" s="63">
+      <c r="B9" s="66"/>
+      <c r="C9" t="s" s="68">
         <v>23</v>
       </c>
-      <c r="F8" s="64"/>
-      <c r="G8" s="65"/>
-      <c r="H8" s="66"/>
-    </row>
-    <row r="9" ht="40.0" customHeight="true">
-      <c r="A9" t="s" s="67">
+      <c r="D9" s="69"/>
+      <c r="E9" s="70"/>
+      <c r="F9" t="s" s="72">
         <v>24</v>
       </c>
-      <c r="B9" s="68"/>
-      <c r="C9" s="69"/>
-      <c r="D9" s="70"/>
-      <c r="E9" s="71"/>
-      <c r="F9" t="s" s="73">
+      <c r="G9" s="73"/>
+      <c r="H9" s="74"/>
+    </row>
+    <row r="10" ht="40.0" customHeight="true">
+      <c r="A10" t="s" s="75">
         <v>25</v>
       </c>
-      <c r="G9" s="74"/>
-      <c r="H9" s="75"/>
-    </row>
-    <row r="10" ht="40.0" customHeight="true">
-      <c r="A10" t="s" s="76">
+      <c r="B10" s="76"/>
+      <c r="C10" t="s" s="78">
         <v>26</v>
       </c>
-      <c r="B10" s="77"/>
-      <c r="C10" t="s" s="79">
+      <c r="D10" s="79"/>
+      <c r="E10" t="s" s="81">
         <v>27</v>
       </c>
-      <c r="D10" s="80"/>
-      <c r="E10" s="81"/>
-      <c r="F10" t="s" s="83">
+      <c r="F10" s="82"/>
+      <c r="G10" s="83"/>
+      <c r="H10" s="84"/>
+    </row>
+    <row r="11" ht="40.0" customHeight="true">
+      <c r="A11" t="s" s="85">
         <v>28</v>
       </c>
-      <c r="G10" s="84"/>
-      <c r="H10" s="85"/>
-    </row>
-    <row r="11" ht="40.0" customHeight="true">
-      <c r="A11" t="s" s="86">
+      <c r="B11" t="s" s="87">
         <v>29</v>
       </c>
-      <c r="B11" s="87"/>
-      <c r="C11" t="s" s="89">
+      <c r="C11" s="88"/>
+      <c r="D11" s="89"/>
+      <c r="E11" t="s" s="91">
         <v>30</v>
       </c>
-      <c r="D11" s="90"/>
-      <c r="E11" t="s" s="92">
+      <c r="F11" s="92"/>
+      <c r="G11" s="93"/>
+      <c r="H11" s="94"/>
+    </row>
+    <row r="12" ht="40.0" customHeight="true">
+      <c r="A12" t="s" s="95">
         <v>31</v>
       </c>
-      <c r="F11" s="93"/>
-      <c r="G11" s="94"/>
-      <c r="H11" s="95"/>
-    </row>
-    <row r="12" ht="40.0" customHeight="true">
-      <c r="A12" t="s" s="96">
+      <c r="B12" s="96"/>
+      <c r="C12" s="97"/>
+      <c r="D12" t="s" s="99">
         <v>32</v>
       </c>
-      <c r="B12" s="97"/>
-      <c r="C12" s="98"/>
-      <c r="D12" s="99"/>
       <c r="E12" t="s" s="101">
         <v>33</v>
       </c>
-      <c r="F12" s="102"/>
-      <c r="G12" s="103"/>
-      <c r="H12" s="104"/>
+      <c r="F12" t="s" s="103">
+        <v>34</v>
+      </c>
+      <c r="G12" s="104"/>
+      <c r="H12" s="105"/>
     </row>
     <row r="13" ht="40.0" customHeight="true">
-      <c r="A13" t="s" s="105">
-        <v>34</v>
-      </c>
-      <c r="B13" s="106"/>
-      <c r="C13" s="107"/>
-      <c r="D13" t="s" s="109">
+      <c r="A13" t="s" s="106">
         <v>35</v>
       </c>
-      <c r="E13" t="s" s="111">
+      <c r="B13" s="107"/>
+      <c r="C13" s="108"/>
+      <c r="D13" t="s" s="110">
         <v>36</v>
       </c>
-      <c r="F13" t="s" s="113">
+      <c r="E13" s="111"/>
+      <c r="F13" s="112"/>
+      <c r="G13" s="113"/>
+      <c r="H13" s="114"/>
+    </row>
+    <row r="14" ht="40.0" customHeight="true">
+      <c r="A14" t="s" s="115">
         <v>37</v>
       </c>
-      <c r="G13" s="114"/>
-      <c r="H13" s="115"/>
-    </row>
-    <row r="14" ht="40.0" customHeight="true">
-      <c r="A14" t="s" s="116">
+      <c r="B14" s="116"/>
+      <c r="C14" s="117"/>
+      <c r="D14" s="118"/>
+      <c r="E14" t="s" s="120">
         <v>38</v>
       </c>
-      <c r="B14" s="117"/>
-      <c r="C14" s="118"/>
-      <c r="D14" t="s" s="120">
+      <c r="F14" t="s" s="122">
         <v>39</v>
       </c>
-      <c r="E14" s="121"/>
-      <c r="F14" s="122"/>
       <c r="G14" s="123"/>
       <c r="H14" s="124"/>
     </row>
@@ -2054,32 +2021,32 @@
         <v>40</v>
       </c>
       <c r="B15" s="126"/>
-      <c r="C15" s="127"/>
-      <c r="D15" s="128"/>
-      <c r="E15" t="s" s="130">
+      <c r="C15" t="s" s="128">
         <v>41</v>
       </c>
-      <c r="F15" t="s" s="132">
+      <c r="D15" t="s" s="130">
         <v>42</v>
       </c>
-      <c r="G15" s="133"/>
-      <c r="H15" s="134"/>
+      <c r="E15" s="131"/>
+      <c r="F15" t="s" s="133">
+        <v>43</v>
+      </c>
+      <c r="G15" s="134"/>
+      <c r="H15" s="135"/>
     </row>
     <row r="16" ht="40.0" customHeight="true">
-      <c r="A16" t="s" s="135">
-        <v>43</v>
-      </c>
-      <c r="B16" s="136"/>
-      <c r="C16" t="s" s="138">
+      <c r="A16" t="s" s="136">
         <v>44</v>
       </c>
+      <c r="B16" s="137"/>
+      <c r="C16" s="138"/>
       <c r="D16" t="s" s="140">
         <v>45</v>
       </c>
-      <c r="E16" s="141"/>
-      <c r="F16" t="s" s="143">
+      <c r="E16" t="s" s="142">
         <v>46</v>
       </c>
+      <c r="F16" s="143"/>
       <c r="G16" s="144"/>
       <c r="H16" s="145"/>
     </row>
@@ -2092,54 +2059,54 @@
       <c r="D17" t="s" s="150">
         <v>48</v>
       </c>
-      <c r="E17" t="s" s="152">
+      <c r="E17" s="151"/>
+      <c r="F17" s="152"/>
+      <c r="G17" s="153"/>
+      <c r="H17" s="154"/>
+    </row>
+    <row r="18" ht="40.0" customHeight="true">
+      <c r="A18" t="s" s="155">
         <v>49</v>
       </c>
-      <c r="F17" s="153"/>
-      <c r="G17" s="154"/>
-      <c r="H17" s="155"/>
-    </row>
-    <row r="18" ht="40.0" customHeight="true">
-      <c r="A18" t="s" s="156">
+      <c r="B18" s="156"/>
+      <c r="C18" s="157"/>
+      <c r="D18" s="158"/>
+      <c r="E18" t="s" s="160">
         <v>50</v>
       </c>
-      <c r="B18" s="157"/>
-      <c r="C18" s="158"/>
-      <c r="D18" t="s" s="160">
+      <c r="F18" s="161"/>
+      <c r="G18" s="162"/>
+      <c r="H18" s="163"/>
+    </row>
+    <row r="19" ht="40.0" customHeight="true">
+      <c r="A19" t="s" s="164">
         <v>51</v>
       </c>
-      <c r="E18" s="161"/>
-      <c r="F18" s="162"/>
-      <c r="G18" t="s" s="164">
+      <c r="B19" s="165"/>
+      <c r="C19" t="s" s="167">
         <v>52</v>
       </c>
-      <c r="H18" s="165"/>
-    </row>
-    <row r="19" ht="40.0" customHeight="true">
-      <c r="A19" t="s" s="166">
+      <c r="D19" s="168"/>
+      <c r="E19" s="169"/>
+      <c r="F19" s="170"/>
+      <c r="G19" s="171"/>
+      <c r="H19" s="172"/>
+    </row>
+    <row r="20" ht="40.0" customHeight="true">
+      <c r="A20" t="s" s="173">
         <v>53</v>
       </c>
-      <c r="B19" s="167"/>
-      <c r="C19" s="168"/>
-      <c r="D19" s="169"/>
-      <c r="E19" t="s" s="171">
+      <c r="B20" s="174"/>
+      <c r="C20" t="s" s="176">
         <v>54</v>
       </c>
-      <c r="F19" s="172"/>
-      <c r="G19" s="173"/>
-      <c r="H19" s="174"/>
-    </row>
-    <row r="20" ht="40.0" customHeight="true">
-      <c r="A20" t="s" s="175">
+      <c r="D20" s="177"/>
+      <c r="E20" t="s" s="179">
         <v>55</v>
       </c>
-      <c r="B20" s="176"/>
-      <c r="C20" t="s" s="178">
+      <c r="F20" t="s" s="181">
         <v>56</v>
       </c>
-      <c r="D20" s="179"/>
-      <c r="E20" s="180"/>
-      <c r="F20" s="181"/>
       <c r="G20" s="182"/>
       <c r="H20" s="183"/>
     </row>
@@ -2152,70 +2119,70 @@
         <v>58</v>
       </c>
       <c r="D21" s="188"/>
-      <c r="E21" t="s" s="190">
+      <c r="E21" s="189"/>
+      <c r="F21" s="190"/>
+      <c r="G21" s="191"/>
+      <c r="H21" s="192"/>
+    </row>
+    <row r="22" ht="40.0" customHeight="true">
+      <c r="A22" t="s" s="193">
         <v>59</v>
       </c>
-      <c r="F21" t="s" s="192">
+      <c r="B22" s="194"/>
+      <c r="C22" s="195"/>
+      <c r="D22" s="196"/>
+      <c r="E22" t="s" s="198">
         <v>60</v>
       </c>
-      <c r="G21" s="193"/>
-      <c r="H21" s="194"/>
-    </row>
-    <row r="22" ht="40.0" customHeight="true">
-      <c r="A22" t="s" s="195">
+      <c r="F22" t="s" s="200">
         <v>61</v>
       </c>
-      <c r="B22" s="196"/>
-      <c r="C22" t="s" s="198">
+      <c r="G22" s="201"/>
+      <c r="H22" s="202"/>
+    </row>
+    <row r="23" ht="40.0" customHeight="true">
+      <c r="A23" t="s" s="203">
         <v>62</v>
       </c>
-      <c r="D22" s="199"/>
-      <c r="E22" s="200"/>
-      <c r="F22" s="201"/>
-      <c r="G22" s="202"/>
-      <c r="H22" s="203"/>
-    </row>
-    <row r="23" ht="40.0" customHeight="true">
-      <c r="A23" t="s" s="204">
+      <c r="B23" s="204"/>
+      <c r="C23" t="s" s="206">
         <v>63</v>
       </c>
-      <c r="B23" s="205"/>
-      <c r="C23" s="206"/>
       <c r="D23" s="207"/>
-      <c r="E23" t="s" s="209">
+      <c r="E23" s="208"/>
+      <c r="F23" s="209"/>
+      <c r="G23" s="210"/>
+      <c r="H23" s="211"/>
+    </row>
+    <row r="24" ht="40.0" customHeight="true">
+      <c r="A24" t="s" s="212">
         <v>64</v>
       </c>
-      <c r="F23" t="s" s="211">
+      <c r="B24" s="213"/>
+      <c r="C24" s="214"/>
+      <c r="D24" s="215"/>
+      <c r="E24" s="216"/>
+      <c r="F24" t="s" s="218">
         <v>65</v>
       </c>
-      <c r="G23" s="212"/>
-      <c r="H23" s="213"/>
-    </row>
-    <row r="24" ht="40.0" customHeight="true">
-      <c r="A24" t="s" s="214">
+      <c r="G24" s="219"/>
+      <c r="H24" t="s" s="221">
         <v>66</v>
       </c>
-      <c r="B24" s="215"/>
-      <c r="C24" t="s" s="217">
+    </row>
+    <row r="25" ht="40.0" customHeight="true">
+      <c r="A25" t="s" s="222">
         <v>67</v>
       </c>
-      <c r="D24" s="218"/>
-      <c r="E24" s="219"/>
-      <c r="F24" s="220"/>
-      <c r="G24" s="221"/>
-      <c r="H24" s="222"/>
-    </row>
-    <row r="25" ht="40.0" customHeight="true">
-      <c r="A25" t="s" s="223">
+      <c r="B25" s="223"/>
+      <c r="C25" s="224"/>
+      <c r="D25" t="s" s="226">
         <v>68</v>
       </c>
-      <c r="B25" s="224"/>
-      <c r="C25" s="225"/>
-      <c r="D25" s="226"/>
-      <c r="E25" s="227"/>
-      <c r="F25" t="s" s="229">
+      <c r="E25" t="s" s="228">
         <v>69</v>
       </c>
+      <c r="F25" s="229"/>
       <c r="G25" s="230"/>
       <c r="H25" s="231"/>
     </row>
@@ -2225,36 +2192,36 @@
       </c>
       <c r="B26" s="233"/>
       <c r="C26" s="234"/>
-      <c r="D26" t="s" s="236">
+      <c r="D26" s="235"/>
+      <c r="E26" t="s" s="237">
         <v>71</v>
       </c>
-      <c r="E26" t="s" s="238">
+      <c r="F26" s="238"/>
+      <c r="G26" s="239"/>
+      <c r="H26" s="240"/>
+    </row>
+    <row r="27" ht="40.0" customHeight="true">
+      <c r="A27" t="s" s="241">
         <v>72</v>
       </c>
-      <c r="F26" s="239"/>
-      <c r="G26" s="240"/>
-      <c r="H26" s="241"/>
-    </row>
-    <row r="27" ht="40.0" customHeight="true">
-      <c r="A27" t="s" s="242">
+      <c r="B27" s="242"/>
+      <c r="C27" s="243"/>
+      <c r="D27" s="244"/>
+      <c r="E27" s="245"/>
+      <c r="F27" s="246"/>
+      <c r="G27" t="s" s="248">
         <v>73</v>
       </c>
-      <c r="B27" s="243"/>
-      <c r="C27" s="244"/>
-      <c r="D27" s="245"/>
-      <c r="E27" t="s" s="247">
+      <c r="H27" s="249"/>
+    </row>
+    <row r="28" ht="40.0" customHeight="true">
+      <c r="A28" t="s" s="250">
         <v>74</v>
       </c>
-      <c r="F27" s="248"/>
-      <c r="G27" s="249"/>
-      <c r="H27" s="250"/>
-    </row>
-    <row r="28" ht="40.0" customHeight="true">
-      <c r="A28" t="s" s="251">
+      <c r="B28" s="251"/>
+      <c r="C28" t="s" s="253">
         <v>75</v>
       </c>
-      <c r="B28" s="252"/>
-      <c r="C28" s="253"/>
       <c r="D28" s="254"/>
       <c r="E28" s="255"/>
       <c r="F28" s="256"/>
@@ -2282,170 +2249,158 @@
         <v>79</v>
       </c>
       <c r="B30" s="270"/>
-      <c r="C30" t="s" s="272">
+      <c r="C30" s="271"/>
+      <c r="D30" s="272"/>
+      <c r="E30" t="s" s="274">
         <v>80</v>
       </c>
-      <c r="D30" s="273"/>
-      <c r="E30" s="274"/>
       <c r="F30" s="275"/>
-      <c r="G30" s="276"/>
-      <c r="H30" s="277"/>
+      <c r="G30" t="s" s="277">
+        <v>81</v>
+      </c>
+      <c r="H30" s="278"/>
     </row>
     <row r="31" ht="40.0" customHeight="true">
-      <c r="A31" t="s" s="278">
-        <v>81</v>
-      </c>
-      <c r="B31" s="279"/>
-      <c r="C31" s="280"/>
-      <c r="D31" s="281"/>
-      <c r="E31" t="s" s="283">
+      <c r="A31" t="s" s="279">
         <v>82</v>
       </c>
-      <c r="F31" s="284"/>
-      <c r="G31" t="s" s="286">
+      <c r="B31" s="280"/>
+      <c r="C31" s="281"/>
+      <c r="D31" s="282"/>
+      <c r="E31" t="s" s="284">
         <v>83</v>
       </c>
-      <c r="H31" s="287"/>
+      <c r="F31" s="285"/>
+      <c r="G31" t="s" s="287">
+        <v>84</v>
+      </c>
+      <c r="H31" s="288"/>
     </row>
     <row r="32" ht="40.0" customHeight="true">
-      <c r="A32" t="s" s="288">
-        <v>84</v>
-      </c>
-      <c r="B32" s="289"/>
-      <c r="C32" t="s" s="291">
+      <c r="A32" t="s" s="289">
         <v>85</v>
       </c>
-      <c r="D32" s="292"/>
-      <c r="E32" s="293"/>
-      <c r="F32" s="294"/>
-      <c r="G32" s="295"/>
-      <c r="H32" s="296"/>
+      <c r="B32" s="290"/>
+      <c r="C32" t="s" s="292">
+        <v>86</v>
+      </c>
+      <c r="D32" s="293"/>
+      <c r="E32" s="294"/>
+      <c r="F32" s="295"/>
+      <c r="G32" s="296"/>
+      <c r="H32" s="297"/>
     </row>
     <row r="33" ht="40.0" customHeight="true">
-      <c r="A33" t="s" s="297">
-        <v>86</v>
-      </c>
-      <c r="B33" s="298"/>
-      <c r="C33" s="299"/>
-      <c r="D33" s="300"/>
-      <c r="E33" t="s" s="302">
+      <c r="A33" t="s" s="298">
         <v>87</v>
       </c>
-      <c r="F33" s="303"/>
-      <c r="G33" s="304"/>
-      <c r="H33" s="305"/>
+      <c r="B33" s="299"/>
+      <c r="C33" s="300"/>
+      <c r="D33" s="301"/>
+      <c r="E33" t="s" s="303">
+        <v>88</v>
+      </c>
+      <c r="F33" s="304"/>
+      <c r="G33" s="305"/>
+      <c r="H33" s="306"/>
     </row>
     <row r="34" ht="40.0" customHeight="true">
-      <c r="A34" t="s" s="306">
-        <v>88</v>
-      </c>
-      <c r="B34" s="307"/>
-      <c r="C34" t="s" s="309">
+      <c r="A34" t="s" s="307">
         <v>89</v>
       </c>
-      <c r="D34" s="310"/>
-      <c r="E34" s="311"/>
-      <c r="F34" s="312"/>
-      <c r="G34" s="313"/>
-      <c r="H34" s="314"/>
+      <c r="B34" s="308"/>
+      <c r="C34" t="s" s="310">
+        <v>90</v>
+      </c>
+      <c r="D34" s="311"/>
+      <c r="E34" s="312"/>
+      <c r="F34" s="313"/>
+      <c r="G34" s="314"/>
+      <c r="H34" s="315"/>
     </row>
     <row r="35" ht="40.0" customHeight="true">
-      <c r="A35" t="s" s="315">
-        <v>90</v>
-      </c>
-      <c r="B35" s="316"/>
-      <c r="C35" s="317"/>
-      <c r="D35" s="318"/>
-      <c r="E35" s="319"/>
-      <c r="F35" s="320"/>
-      <c r="G35" t="s" s="322">
+      <c r="A35" t="s" s="316">
         <v>91</v>
       </c>
-      <c r="H35" s="323"/>
+      <c r="B35" s="317"/>
+      <c r="C35" t="s" s="319">
+        <v>92</v>
+      </c>
+      <c r="D35" s="320"/>
+      <c r="E35" s="321"/>
+      <c r="F35" s="322"/>
+      <c r="G35" s="323"/>
+      <c r="H35" s="324"/>
     </row>
     <row r="36" ht="40.0" customHeight="true">
-      <c r="A36" t="s" s="324">
-        <v>92</v>
-      </c>
-      <c r="B36" s="325"/>
-      <c r="C36" t="s" s="327">
+      <c r="A36" t="s" s="325">
         <v>93</v>
       </c>
-      <c r="D36" s="328"/>
-      <c r="E36" s="329"/>
-      <c r="F36" s="330"/>
-      <c r="G36" s="331"/>
-      <c r="H36" s="332"/>
+      <c r="B36" s="326"/>
+      <c r="C36" t="s" s="328">
+        <v>94</v>
+      </c>
+      <c r="D36" s="329"/>
+      <c r="E36" s="330"/>
+      <c r="F36" s="331"/>
+      <c r="G36" s="332"/>
+      <c r="H36" s="333"/>
     </row>
     <row r="37" ht="40.0" customHeight="true">
-      <c r="A37" t="s" s="333">
-        <v>94</v>
-      </c>
-      <c r="B37" s="334"/>
-      <c r="C37" t="s" s="336">
+      <c r="A37" t="s" s="334">
         <v>95</v>
       </c>
+      <c r="B37" s="335"/>
+      <c r="C37" s="336"/>
       <c r="D37" s="337"/>
       <c r="E37" s="338"/>
-      <c r="F37" s="339"/>
-      <c r="G37" s="340"/>
-      <c r="H37" s="341"/>
+      <c r="F37" t="s" s="340">
+        <v>96</v>
+      </c>
+      <c r="G37" s="341"/>
+      <c r="H37" s="342"/>
     </row>
     <row r="38" ht="40.0" customHeight="true">
-      <c r="A38" t="s" s="342">
-        <v>96</v>
-      </c>
-      <c r="B38" s="343"/>
-      <c r="C38" s="344"/>
-      <c r="D38" s="345"/>
-      <c r="E38" s="346"/>
-      <c r="F38" t="s" s="348">
+      <c r="A38" t="s" s="343">
         <v>97</v>
       </c>
-      <c r="G38" s="349"/>
-      <c r="H38" s="350"/>
+      <c r="B38" s="344"/>
+      <c r="C38" s="345"/>
+      <c r="D38" s="346"/>
+      <c r="E38" s="347"/>
+      <c r="F38" s="348"/>
+      <c r="G38" t="s" s="350">
+        <v>98</v>
+      </c>
+      <c r="H38" s="351"/>
     </row>
     <row r="39" ht="40.0" customHeight="true">
-      <c r="A39" t="s" s="351">
-        <v>98</v>
-      </c>
-      <c r="B39" s="352"/>
-      <c r="C39" t="s" s="354">
+      <c r="A39" t="s" s="352">
         <v>99</v>
       </c>
-      <c r="D39" s="355"/>
-      <c r="E39" s="356"/>
-      <c r="F39" s="357"/>
-      <c r="G39" s="358"/>
-      <c r="H39" s="359"/>
+      <c r="B39" s="353"/>
+      <c r="C39" t="s" s="355">
+        <v>100</v>
+      </c>
+      <c r="D39" s="356"/>
+      <c r="E39" s="357"/>
+      <c r="F39" s="358"/>
+      <c r="G39" s="359"/>
+      <c r="H39" s="360"/>
     </row>
     <row r="40" ht="40.0" customHeight="true">
-      <c r="A40" t="s" s="360">
-        <v>100</v>
-      </c>
-      <c r="B40" s="361"/>
-      <c r="C40" t="s" s="363">
+      <c r="A40" t="s" s="361">
         <v>101</v>
       </c>
-      <c r="D40" s="364"/>
-      <c r="E40" s="365"/>
-      <c r="F40" s="366"/>
-      <c r="G40" s="367"/>
-      <c r="H40" s="368"/>
-    </row>
-    <row r="41" ht="40.0" customHeight="true">
-      <c r="A41" t="s" s="369">
+      <c r="B40" s="362"/>
+      <c r="C40" t="s" s="364">
         <v>102</v>
       </c>
-      <c r="B41" s="370"/>
-      <c r="C41" s="371"/>
-      <c r="D41" s="372"/>
-      <c r="E41" s="373"/>
-      <c r="F41" s="374"/>
-      <c r="G41" t="s" s="376">
-        <v>103</v>
-      </c>
-      <c r="H41" s="377"/>
+      <c r="D40" s="365"/>
+      <c r="E40" s="366"/>
+      <c r="F40" s="367"/>
+      <c r="G40" s="368"/>
+      <c r="H40" s="369"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
Daten und DM fix.
</commit_message>
<xml_diff>
--- a/Turnierplanung.xlsx
+++ b/Turnierplanung.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="102">
   <si>
     <t>Wochenende (KW)</t>
   </si>
@@ -42,14 +42,14 @@
 2026-09-05</t>
   </si>
   <si>
-    <t>Heidenheim - QB_U17_3 (QB)</t>
+    <t>Leverkusen - QB_SEN_1 (QB)</t>
   </si>
   <si>
     <t>KW 37
 2026-09-12</t>
   </si>
   <si>
-    <t>Leverkusen - QB_SEN_1 (QB)</t>
+    <t>Heidenheim - QB_U17_3 (QB)</t>
   </si>
   <si>
     <t>KW 38
@@ -70,14 +70,14 @@
 2026-10-03</t>
   </si>
   <si>
-    <t>Leverkusen - DM_U17_13 (DM)</t>
+    <t>Reutlingen - QB_SEN_2 (QB)</t>
   </si>
   <si>
     <t>KW 41
 2026-10-10</t>
   </si>
   <si>
-    <t>Reutlingen - QB_SEN_2 (QB)</t>
+    <t>Heidelberg - QB_U20_7 (QB)</t>
   </si>
   <si>
     <t>KW 42
@@ -235,9 +235,6 @@
     <t>EFC - EFC_Krakow (EFC)</t>
   </si>
   <si>
-    <t>Leverkusen - DM_U13_14 (DM)</t>
-  </si>
-  <si>
     <t>KW 7
 2027-02-20</t>
   </si>
@@ -248,13 +245,6 @@
     <t>FIE - FIE_Vrsac (FIE)</t>
   </si>
   <si>
-    <t>KW 8
-2027-02-27</t>
-  </si>
-  <si>
-    <t>Heidelberg - QB_U20_7 (QB)</t>
-  </si>
-  <si>
     <t>KW 9
 2027-03-06</t>
   </si>
@@ -315,6 +305,16 @@
     <t>EFC - EFC_EM_U20 (EFC)</t>
   </si>
   <si>
+    <t>KW 17
+2027-05-01</t>
+  </si>
+  <si>
+    <t>Leverkusen - DM_U17_13 (DM)</t>
+  </si>
+  <si>
+    <t>Leverkusen - DM_U13_14 (DM)</t>
+  </si>
+  <si>
     <t>KW 18
 2027-05-08</t>
   </si>
@@ -337,18 +337,14 @@
     <t>EFC - EFC_EM_Senioren (EFC)</t>
   </si>
   <si>
+    <t>Bonn - CHALLENGE_U15_8 (CHALLENGE)</t>
+  </si>
+  <si>
     <t>KW 23
 2027-06-12</t>
   </si>
   <si>
     <t>EFC - EFC_EM_U17 (EFC)</t>
-  </si>
-  <si>
-    <t>KW 24
-2027-06-19</t>
-  </si>
-  <si>
-    <t>Bonn - CHALLENGE_U15_8 (CHALLENGE)</t>
   </si>
   <si>
     <t>KW 25
@@ -370,7 +366,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="41">
+  <fonts count="40">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
@@ -383,11 +379,6 @@
       <sz val="11.0"/>
       <b val="true"/>
       <color indexed="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -668,7 +659,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="370">
+  <cellXfs count="362">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="true" applyFill="true" applyAlignment="true" applyBorder="true">
       <alignment horizontal="center" vertical="center"/>
@@ -1330,9 +1321,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
@@ -1396,7 +1384,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1444,19 +1435,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
     <xf numFmtId="0" fontId="29" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1486,10 +1477,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1510,16 +1501,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1540,16 +1528,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1573,10 +1561,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1669,6 +1660,9 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
     <xf numFmtId="0" fontId="37" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
@@ -1724,33 +1718,6 @@
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
-      <alignment horizontal="center" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1783,7 +1750,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H39"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="25.0" customWidth="true"/>
@@ -1827,12 +1794,12 @@
         <v>8</v>
       </c>
       <c r="B2" s="3"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="6"/>
-      <c r="F2" t="s" s="8">
+      <c r="C2" t="s" s="5">
         <v>9</v>
       </c>
+      <c r="D2" s="6"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="8"/>
       <c r="G2" s="9"/>
       <c r="H2" s="10"/>
     </row>
@@ -1841,12 +1808,12 @@
         <v>10</v>
       </c>
       <c r="B3" s="12"/>
-      <c r="C3" t="s" s="14">
+      <c r="C3" s="13"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="15"/>
+      <c r="F3" t="s" s="17">
         <v>11</v>
       </c>
-      <c r="D3" s="15"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="17"/>
       <c r="G3" s="18"/>
       <c r="H3" s="19"/>
     </row>
@@ -1883,12 +1850,12 @@
         <v>16</v>
       </c>
       <c r="B6" s="39"/>
-      <c r="C6" s="40"/>
-      <c r="D6" s="41"/>
-      <c r="E6" s="42"/>
-      <c r="F6" t="s" s="44">
+      <c r="C6" t="s" s="41">
         <v>17</v>
       </c>
+      <c r="D6" s="42"/>
+      <c r="E6" s="43"/>
+      <c r="F6" s="44"/>
       <c r="G6" s="45"/>
       <c r="H6" s="46"/>
     </row>
@@ -1897,11 +1864,11 @@
         <v>18</v>
       </c>
       <c r="B7" s="48"/>
-      <c r="C7" t="s" s="50">
+      <c r="C7" s="49"/>
+      <c r="D7" s="50"/>
+      <c r="E7" t="s" s="52">
         <v>19</v>
       </c>
-      <c r="D7" s="51"/>
-      <c r="E7" s="52"/>
       <c r="F7" s="53"/>
       <c r="G7" s="54"/>
       <c r="H7" s="55"/>
@@ -2166,46 +2133,46 @@
         <v>65</v>
       </c>
       <c r="G24" s="219"/>
-      <c r="H24" t="s" s="221">
+      <c r="H24" s="220"/>
+    </row>
+    <row r="25" ht="40.0" customHeight="true">
+      <c r="A25" t="s" s="221">
         <v>66</v>
       </c>
-    </row>
-    <row r="25" ht="40.0" customHeight="true">
-      <c r="A25" t="s" s="222">
+      <c r="B25" s="222"/>
+      <c r="C25" s="223"/>
+      <c r="D25" t="s" s="225">
         <v>67</v>
       </c>
-      <c r="B25" s="223"/>
-      <c r="C25" s="224"/>
-      <c r="D25" t="s" s="226">
+      <c r="E25" t="s" s="227">
         <v>68</v>
       </c>
-      <c r="E25" t="s" s="228">
+      <c r="F25" s="228"/>
+      <c r="G25" s="229"/>
+      <c r="H25" s="230"/>
+    </row>
+    <row r="26" ht="40.0" customHeight="true">
+      <c r="A26" t="s" s="231">
         <v>69</v>
       </c>
-      <c r="F25" s="229"/>
-      <c r="G25" s="230"/>
-      <c r="H25" s="231"/>
-    </row>
-    <row r="26" ht="40.0" customHeight="true">
-      <c r="A26" t="s" s="232">
+      <c r="B26" s="232"/>
+      <c r="C26" s="233"/>
+      <c r="D26" s="234"/>
+      <c r="E26" s="235"/>
+      <c r="F26" s="236"/>
+      <c r="G26" t="s" s="238">
         <v>70</v>
       </c>
-      <c r="B26" s="233"/>
-      <c r="C26" s="234"/>
-      <c r="D26" s="235"/>
-      <c r="E26" t="s" s="237">
+      <c r="H26" s="239"/>
+    </row>
+    <row r="27" ht="40.0" customHeight="true">
+      <c r="A27" t="s" s="240">
         <v>71</v>
       </c>
-      <c r="F26" s="238"/>
-      <c r="G26" s="239"/>
-      <c r="H26" s="240"/>
-    </row>
-    <row r="27" ht="40.0" customHeight="true">
-      <c r="A27" t="s" s="241">
+      <c r="B27" s="241"/>
+      <c r="C27" t="s" s="243">
         <v>72</v>
       </c>
-      <c r="B27" s="242"/>
-      <c r="C27" s="243"/>
       <c r="D27" s="244"/>
       <c r="E27" s="245"/>
       <c r="F27" s="246"/>
@@ -2225,23 +2192,23 @@
       <c r="D28" s="254"/>
       <c r="E28" s="255"/>
       <c r="F28" s="256"/>
-      <c r="G28" t="s" s="258">
+      <c r="G28" s="257"/>
+      <c r="H28" s="258"/>
+    </row>
+    <row r="29" ht="40.0" customHeight="true">
+      <c r="A29" t="s" s="259">
         <v>76</v>
       </c>
-      <c r="H28" s="259"/>
-    </row>
-    <row r="29" ht="40.0" customHeight="true">
-      <c r="A29" t="s" s="260">
+      <c r="B29" s="260"/>
+      <c r="C29" s="261"/>
+      <c r="D29" s="262"/>
+      <c r="E29" t="s" s="264">
         <v>77</v>
       </c>
-      <c r="B29" s="261"/>
-      <c r="C29" t="s" s="263">
+      <c r="F29" s="265"/>
+      <c r="G29" t="s" s="267">
         <v>78</v>
       </c>
-      <c r="D29" s="264"/>
-      <c r="E29" s="265"/>
-      <c r="F29" s="266"/>
-      <c r="G29" s="267"/>
       <c r="H29" s="268"/>
     </row>
     <row r="30" ht="40.0" customHeight="true">
@@ -2265,44 +2232,44 @@
         <v>82</v>
       </c>
       <c r="B31" s="280"/>
-      <c r="C31" s="281"/>
-      <c r="D31" s="282"/>
-      <c r="E31" t="s" s="284">
+      <c r="C31" t="s" s="282">
         <v>83</v>
       </c>
+      <c r="D31" s="283"/>
+      <c r="E31" s="284"/>
       <c r="F31" s="285"/>
-      <c r="G31" t="s" s="287">
+      <c r="G31" s="286"/>
+      <c r="H31" s="287"/>
+    </row>
+    <row r="32" ht="40.0" customHeight="true">
+      <c r="A32" t="s" s="288">
         <v>84</v>
       </c>
-      <c r="H31" s="288"/>
-    </row>
-    <row r="32" ht="40.0" customHeight="true">
-      <c r="A32" t="s" s="289">
+      <c r="B32" s="289"/>
+      <c r="C32" s="290"/>
+      <c r="D32" s="291"/>
+      <c r="E32" t="s" s="293">
         <v>85</v>
       </c>
-      <c r="B32" s="290"/>
-      <c r="C32" t="s" s="292">
+      <c r="F32" s="294"/>
+      <c r="G32" s="295"/>
+      <c r="H32" s="296"/>
+    </row>
+    <row r="33" ht="40.0" customHeight="true">
+      <c r="A33" t="s" s="297">
         <v>86</v>
       </c>
-      <c r="D32" s="293"/>
-      <c r="E32" s="294"/>
-      <c r="F32" s="295"/>
-      <c r="G32" s="296"/>
-      <c r="H32" s="297"/>
-    </row>
-    <row r="33" ht="40.0" customHeight="true">
-      <c r="A33" t="s" s="298">
+      <c r="B33" s="298"/>
+      <c r="C33" s="299"/>
+      <c r="D33" s="300"/>
+      <c r="E33" s="301"/>
+      <c r="F33" t="s" s="303">
         <v>87</v>
       </c>
-      <c r="B33" s="299"/>
-      <c r="C33" s="300"/>
-      <c r="D33" s="301"/>
-      <c r="E33" t="s" s="303">
+      <c r="G33" s="304"/>
+      <c r="H33" t="s" s="306">
         <v>88</v>
       </c>
-      <c r="F33" s="304"/>
-      <c r="G33" s="305"/>
-      <c r="H33" s="306"/>
     </row>
     <row r="34" ht="40.0" customHeight="true">
       <c r="A34" t="s" s="307">
@@ -2343,64 +2310,52 @@
       <c r="D36" s="329"/>
       <c r="E36" s="330"/>
       <c r="F36" s="331"/>
-      <c r="G36" s="332"/>
-      <c r="H36" s="333"/>
+      <c r="G36" t="s" s="333">
+        <v>95</v>
+      </c>
+      <c r="H36" s="334"/>
     </row>
     <row r="37" ht="40.0" customHeight="true">
-      <c r="A37" t="s" s="334">
-        <v>95</v>
-      </c>
-      <c r="B37" s="335"/>
-      <c r="C37" s="336"/>
-      <c r="D37" s="337"/>
-      <c r="E37" s="338"/>
-      <c r="F37" t="s" s="340">
+      <c r="A37" t="s" s="335">
         <v>96</v>
       </c>
-      <c r="G37" s="341"/>
-      <c r="H37" s="342"/>
+      <c r="B37" s="336"/>
+      <c r="C37" s="337"/>
+      <c r="D37" s="338"/>
+      <c r="E37" s="339"/>
+      <c r="F37" t="s" s="341">
+        <v>97</v>
+      </c>
+      <c r="G37" s="342"/>
+      <c r="H37" s="343"/>
     </row>
     <row r="38" ht="40.0" customHeight="true">
-      <c r="A38" t="s" s="343">
-        <v>97</v>
-      </c>
-      <c r="B38" s="344"/>
-      <c r="C38" s="345"/>
-      <c r="D38" s="346"/>
-      <c r="E38" s="347"/>
-      <c r="F38" s="348"/>
-      <c r="G38" t="s" s="350">
+      <c r="A38" t="s" s="344">
         <v>98</v>
       </c>
-      <c r="H38" s="351"/>
+      <c r="B38" s="345"/>
+      <c r="C38" t="s" s="347">
+        <v>99</v>
+      </c>
+      <c r="D38" s="348"/>
+      <c r="E38" s="349"/>
+      <c r="F38" s="350"/>
+      <c r="G38" s="351"/>
+      <c r="H38" s="352"/>
     </row>
     <row r="39" ht="40.0" customHeight="true">
-      <c r="A39" t="s" s="352">
-        <v>99</v>
-      </c>
-      <c r="B39" s="353"/>
-      <c r="C39" t="s" s="355">
+      <c r="A39" t="s" s="353">
         <v>100</v>
       </c>
-      <c r="D39" s="356"/>
-      <c r="E39" s="357"/>
-      <c r="F39" s="358"/>
-      <c r="G39" s="359"/>
-      <c r="H39" s="360"/>
-    </row>
-    <row r="40" ht="40.0" customHeight="true">
-      <c r="A40" t="s" s="361">
+      <c r="B39" s="354"/>
+      <c r="C39" t="s" s="356">
         <v>101</v>
       </c>
-      <c r="B40" s="362"/>
-      <c r="C40" t="s" s="364">
-        <v>102</v>
-      </c>
-      <c r="D40" s="365"/>
-      <c r="E40" s="366"/>
-      <c r="F40" s="367"/>
-      <c r="G40" s="368"/>
-      <c r="H40" s="369"/>
+      <c r="D39" s="357"/>
+      <c r="E39" s="358"/>
+      <c r="F39" s="359"/>
+      <c r="G39" s="360"/>
+      <c r="H39" s="361"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>

<commit_message>
DM constraints und Abstandsoptimierung
</commit_message>
<xml_diff>
--- a/Turnierplanung.xlsx
+++ b/Turnierplanung.xlsx
@@ -42,14 +42,14 @@
 2026-09-05</t>
   </si>
   <si>
-    <t>Leverkusen - QB_SEN_1 (QB)</t>
+    <t>Heidenheim - QB_U17_3 (QB)</t>
   </si>
   <si>
     <t>KW 37
 2026-09-12</t>
   </si>
   <si>
-    <t>Heidenheim - QB_U17_3 (QB)</t>
+    <t>Leverkusen - QB_SEN_1 (QB)</t>
   </si>
   <si>
     <t>KW 38
@@ -228,6 +228,9 @@
     <t>FIE - FIE_Heidenheim (FIE)</t>
   </si>
   <si>
+    <t>Waldkirch - CHALLENGE_U15_10 (CHALLENGE)</t>
+  </si>
+  <si>
     <t>KW 6
 2027-02-13</t>
   </si>
@@ -245,8 +248,8 @@
     <t>FIE - FIE_Vrsac (FIE)</t>
   </si>
   <si>
-    <t>KW 9
-2027-03-06</t>
+    <t>KW 8
+2027-02-27</t>
   </si>
   <si>
     <t>Osnabrück - CHALLENGE_U15_11 (CHALLENGE)</t>
@@ -288,9 +291,6 @@
     <t>FIE - FIE_WM_U20 (FIE)</t>
   </si>
   <si>
-    <t>Waldkirch - CHALLENGE_U15_10 (CHALLENGE)</t>
-  </si>
-  <si>
     <t>KW 15
 2027-04-17</t>
   </si>
@@ -305,6 +305,9 @@
     <t>EFC - EFC_EM_U20 (EFC)</t>
   </si>
   <si>
+    <t>Bonn - CHALLENGE_U15_8 (CHALLENGE)</t>
+  </si>
+  <si>
     <t>KW 17
 2027-05-01</t>
   </si>
@@ -335,9 +338,6 @@
   </si>
   <si>
     <t>EFC - EFC_EM_Senioren (EFC)</t>
-  </si>
-  <si>
-    <t>Bonn - CHALLENGE_U15_8 (CHALLENGE)</t>
   </si>
   <si>
     <t>KW 23
@@ -1294,6 +1294,9 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
@@ -1492,9 +1495,6 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
     <xf numFmtId="0" fontId="31" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
@@ -1549,6 +1549,9 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
     <xf numFmtId="0" fontId="33" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
@@ -1643,9 +1646,6 @@
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1794,12 +1794,12 @@
         <v>8</v>
       </c>
       <c r="B2" s="3"/>
-      <c r="C2" t="s" s="5">
+      <c r="C2" s="4"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="6"/>
+      <c r="F2" t="s" s="8">
         <v>9</v>
       </c>
-      <c r="D2" s="6"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="8"/>
       <c r="G2" s="9"/>
       <c r="H2" s="10"/>
     </row>
@@ -1808,12 +1808,12 @@
         <v>10</v>
       </c>
       <c r="B3" s="12"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="15"/>
-      <c r="F3" t="s" s="17">
+      <c r="C3" t="s" s="14">
         <v>11</v>
       </c>
+      <c r="D3" s="15"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="17"/>
       <c r="G3" s="18"/>
       <c r="H3" s="19"/>
     </row>
@@ -2118,113 +2118,113 @@
       <c r="D23" s="207"/>
       <c r="E23" s="208"/>
       <c r="F23" s="209"/>
-      <c r="G23" s="210"/>
-      <c r="H23" s="211"/>
+      <c r="G23" t="s" s="211">
+        <v>64</v>
+      </c>
+      <c r="H23" s="212"/>
     </row>
     <row r="24" ht="40.0" customHeight="true">
-      <c r="A24" t="s" s="212">
-        <v>64</v>
-      </c>
-      <c r="B24" s="213"/>
-      <c r="C24" s="214"/>
-      <c r="D24" s="215"/>
-      <c r="E24" s="216"/>
-      <c r="F24" t="s" s="218">
+      <c r="A24" t="s" s="213">
         <v>65</v>
       </c>
-      <c r="G24" s="219"/>
-      <c r="H24" s="220"/>
+      <c r="B24" s="214"/>
+      <c r="C24" s="215"/>
+      <c r="D24" s="216"/>
+      <c r="E24" s="217"/>
+      <c r="F24" t="s" s="219">
+        <v>66</v>
+      </c>
+      <c r="G24" s="220"/>
+      <c r="H24" s="221"/>
     </row>
     <row r="25" ht="40.0" customHeight="true">
-      <c r="A25" t="s" s="221">
-        <v>66</v>
-      </c>
-      <c r="B25" s="222"/>
-      <c r="C25" s="223"/>
-      <c r="D25" t="s" s="225">
+      <c r="A25" t="s" s="222">
         <v>67</v>
       </c>
-      <c r="E25" t="s" s="227">
+      <c r="B25" s="223"/>
+      <c r="C25" s="224"/>
+      <c r="D25" t="s" s="226">
         <v>68</v>
       </c>
-      <c r="F25" s="228"/>
-      <c r="G25" s="229"/>
-      <c r="H25" s="230"/>
+      <c r="E25" t="s" s="228">
+        <v>69</v>
+      </c>
+      <c r="F25" s="229"/>
+      <c r="G25" s="230"/>
+      <c r="H25" s="231"/>
     </row>
     <row r="26" ht="40.0" customHeight="true">
-      <c r="A26" t="s" s="231">
-        <v>69</v>
-      </c>
-      <c r="B26" s="232"/>
-      <c r="C26" s="233"/>
-      <c r="D26" s="234"/>
-      <c r="E26" s="235"/>
-      <c r="F26" s="236"/>
-      <c r="G26" t="s" s="238">
+      <c r="A26" t="s" s="232">
         <v>70</v>
       </c>
-      <c r="H26" s="239"/>
+      <c r="B26" s="233"/>
+      <c r="C26" s="234"/>
+      <c r="D26" s="235"/>
+      <c r="E26" s="236"/>
+      <c r="F26" s="237"/>
+      <c r="G26" t="s" s="239">
+        <v>71</v>
+      </c>
+      <c r="H26" s="240"/>
     </row>
     <row r="27" ht="40.0" customHeight="true">
-      <c r="A27" t="s" s="240">
-        <v>71</v>
-      </c>
-      <c r="B27" s="241"/>
-      <c r="C27" t="s" s="243">
+      <c r="A27" t="s" s="241">
         <v>72</v>
       </c>
-      <c r="D27" s="244"/>
-      <c r="E27" s="245"/>
-      <c r="F27" s="246"/>
-      <c r="G27" t="s" s="248">
+      <c r="B27" s="242"/>
+      <c r="C27" t="s" s="244">
         <v>73</v>
       </c>
-      <c r="H27" s="249"/>
+      <c r="D27" s="245"/>
+      <c r="E27" s="246"/>
+      <c r="F27" s="247"/>
+      <c r="G27" t="s" s="249">
+        <v>74</v>
+      </c>
+      <c r="H27" s="250"/>
     </row>
     <row r="28" ht="40.0" customHeight="true">
-      <c r="A28" t="s" s="250">
-        <v>74</v>
-      </c>
-      <c r="B28" s="251"/>
-      <c r="C28" t="s" s="253">
+      <c r="A28" t="s" s="251">
         <v>75</v>
       </c>
-      <c r="D28" s="254"/>
-      <c r="E28" s="255"/>
-      <c r="F28" s="256"/>
-      <c r="G28" s="257"/>
-      <c r="H28" s="258"/>
+      <c r="B28" s="252"/>
+      <c r="C28" t="s" s="254">
+        <v>76</v>
+      </c>
+      <c r="D28" s="255"/>
+      <c r="E28" s="256"/>
+      <c r="F28" s="257"/>
+      <c r="G28" s="258"/>
+      <c r="H28" s="259"/>
     </row>
     <row r="29" ht="40.0" customHeight="true">
-      <c r="A29" t="s" s="259">
-        <v>76</v>
-      </c>
-      <c r="B29" s="260"/>
-      <c r="C29" s="261"/>
-      <c r="D29" s="262"/>
-      <c r="E29" t="s" s="264">
+      <c r="A29" t="s" s="260">
         <v>77</v>
       </c>
-      <c r="F29" s="265"/>
-      <c r="G29" t="s" s="267">
+      <c r="B29" s="261"/>
+      <c r="C29" s="262"/>
+      <c r="D29" s="263"/>
+      <c r="E29" t="s" s="265">
         <v>78</v>
       </c>
-      <c r="H29" s="268"/>
+      <c r="F29" s="266"/>
+      <c r="G29" t="s" s="268">
+        <v>79</v>
+      </c>
+      <c r="H29" s="269"/>
     </row>
     <row r="30" ht="40.0" customHeight="true">
-      <c r="A30" t="s" s="269">
-        <v>79</v>
-      </c>
-      <c r="B30" s="270"/>
-      <c r="C30" s="271"/>
-      <c r="D30" s="272"/>
-      <c r="E30" t="s" s="274">
+      <c r="A30" t="s" s="270">
         <v>80</v>
       </c>
-      <c r="F30" s="275"/>
-      <c r="G30" t="s" s="277">
+      <c r="B30" s="271"/>
+      <c r="C30" s="272"/>
+      <c r="D30" s="273"/>
+      <c r="E30" t="s" s="275">
         <v>81</v>
       </c>
+      <c r="F30" s="276"/>
+      <c r="G30" s="277"/>
       <c r="H30" s="278"/>
     </row>
     <row r="31" ht="40.0" customHeight="true">
@@ -2252,67 +2252,67 @@
         <v>85</v>
       </c>
       <c r="F32" s="294"/>
-      <c r="G32" s="295"/>
-      <c r="H32" s="296"/>
+      <c r="G32" t="s" s="296">
+        <v>86</v>
+      </c>
+      <c r="H32" s="297"/>
     </row>
     <row r="33" ht="40.0" customHeight="true">
-      <c r="A33" t="s" s="297">
-        <v>86</v>
-      </c>
-      <c r="B33" s="298"/>
-      <c r="C33" s="299"/>
-      <c r="D33" s="300"/>
-      <c r="E33" s="301"/>
-      <c r="F33" t="s" s="303">
+      <c r="A33" t="s" s="298">
         <v>87</v>
       </c>
-      <c r="G33" s="304"/>
-      <c r="H33" t="s" s="306">
+      <c r="B33" s="299"/>
+      <c r="C33" s="300"/>
+      <c r="D33" s="301"/>
+      <c r="E33" s="302"/>
+      <c r="F33" t="s" s="304">
         <v>88</v>
       </c>
+      <c r="G33" s="305"/>
+      <c r="H33" t="s" s="307">
+        <v>89</v>
+      </c>
     </row>
     <row r="34" ht="40.0" customHeight="true">
-      <c r="A34" t="s" s="307">
-        <v>89</v>
-      </c>
-      <c r="B34" s="308"/>
-      <c r="C34" t="s" s="310">
+      <c r="A34" t="s" s="308">
         <v>90</v>
       </c>
-      <c r="D34" s="311"/>
-      <c r="E34" s="312"/>
-      <c r="F34" s="313"/>
-      <c r="G34" s="314"/>
-      <c r="H34" s="315"/>
+      <c r="B34" s="309"/>
+      <c r="C34" t="s" s="311">
+        <v>91</v>
+      </c>
+      <c r="D34" s="312"/>
+      <c r="E34" s="313"/>
+      <c r="F34" s="314"/>
+      <c r="G34" s="315"/>
+      <c r="H34" s="316"/>
     </row>
     <row r="35" ht="40.0" customHeight="true">
-      <c r="A35" t="s" s="316">
-        <v>91</v>
-      </c>
-      <c r="B35" s="317"/>
-      <c r="C35" t="s" s="319">
+      <c r="A35" t="s" s="317">
         <v>92</v>
       </c>
-      <c r="D35" s="320"/>
-      <c r="E35" s="321"/>
-      <c r="F35" s="322"/>
-      <c r="G35" s="323"/>
-      <c r="H35" s="324"/>
+      <c r="B35" s="318"/>
+      <c r="C35" t="s" s="320">
+        <v>93</v>
+      </c>
+      <c r="D35" s="321"/>
+      <c r="E35" s="322"/>
+      <c r="F35" s="323"/>
+      <c r="G35" s="324"/>
+      <c r="H35" s="325"/>
     </row>
     <row r="36" ht="40.0" customHeight="true">
-      <c r="A36" t="s" s="325">
-        <v>93</v>
-      </c>
-      <c r="B36" s="326"/>
-      <c r="C36" t="s" s="328">
+      <c r="A36" t="s" s="326">
         <v>94</v>
       </c>
-      <c r="D36" s="329"/>
-      <c r="E36" s="330"/>
-      <c r="F36" s="331"/>
-      <c r="G36" t="s" s="333">
+      <c r="B36" s="327"/>
+      <c r="C36" t="s" s="329">
         <v>95</v>
       </c>
+      <c r="D36" s="330"/>
+      <c r="E36" s="331"/>
+      <c r="F36" s="332"/>
+      <c r="G36" s="333"/>
       <c r="H36" s="334"/>
     </row>
     <row r="37" ht="40.0" customHeight="true">

</xml_diff>

<commit_message>
updte der Doku und wunschtermine
</commit_message>
<xml_diff>
--- a/Turnierplanung.xlsx
+++ b/Turnierplanung.xlsx
@@ -38,32 +38,25 @@
     <t>U13</t>
   </si>
   <si>
-    <t>KW 36
-2026-09-05</t>
-  </si>
-  <si>
-    <t>Heidenheim - QB_U17_3 (QB)</t>
-  </si>
-  <si>
     <t>KW 37
 2026-09-12</t>
   </si>
   <si>
-    <t>Leverkusen - QB_SEN_1 (QB)</t>
+    <t>Heidenheim - QB_U17_3 (QB)</t>
   </si>
   <si>
     <t>KW 38
 2026-09-19</t>
   </si>
   <si>
-    <t>Leipzig - QB_U17_4 (QB)</t>
+    <t>Leverkusen - QB_SEN_1 (QB)</t>
   </si>
   <si>
     <t>KW 39
 2026-09-26</t>
   </si>
   <si>
-    <t>Solingen - QB_U17_5 (QB)</t>
+    <t>Leipzig - QB_U17_4 (QB)</t>
   </si>
   <si>
     <t>KW 40
@@ -77,7 +70,7 @@
 2026-10-10</t>
   </si>
   <si>
-    <t>Heidelberg - QB_U20_7 (QB)</t>
+    <t>Solingen - QB_U17_5 (QB)</t>
   </si>
   <si>
     <t>KW 42
@@ -228,7 +221,7 @@
     <t>FIE - FIE_Heidenheim (FIE)</t>
   </si>
   <si>
-    <t>Waldkirch - CHALLENGE_U15_10 (CHALLENGE)</t>
+    <t>Osnabrück - CHALLENGE_U15_11 (CHALLENGE)</t>
   </si>
   <si>
     <t>KW 6
@@ -252,7 +245,10 @@
 2027-02-27</t>
   </si>
   <si>
-    <t>Osnabrück - CHALLENGE_U15_11 (CHALLENGE)</t>
+    <t>Heidelberg - QB_U20_7 (QB)</t>
+  </si>
+  <si>
+    <t>Frankfurt - CHALLENGE_U15_9 (CHALLENGE)</t>
   </si>
   <si>
     <t>KW 10
@@ -263,7 +259,11 @@
 EFC - EFC_Differdange (EFC)</t>
   </si>
   <si>
-    <t>Frankfurt - CHALLENGE_U15_9 (CHALLENGE)</t>
+    <t>KW 11
+2027-03-20</t>
+  </si>
+  <si>
+    <t>Waldkirch - CHALLENGE_U15_10 (CHALLENGE)</t>
   </si>
   <si>
     <t>KW 12
@@ -814,10 +814,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -832,7 +832,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -868,13 +871,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -889,19 +892,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -922,19 +925,22 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -958,16 +964,10 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -985,16 +985,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1009,16 +1012,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1039,25 +1045,22 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1081,10 +1084,7 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1105,13 +1105,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1129,16 +1129,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1156,19 +1156,25 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1183,25 +1189,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1216,19 +1216,22 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1243,22 +1246,22 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1273,22 +1276,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1306,16 +1306,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1333,16 +1336,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1360,10 +1363,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1387,10 +1390,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1836,12 +1836,12 @@
         <v>14</v>
       </c>
       <c r="B5" s="30"/>
-      <c r="C5" s="31"/>
-      <c r="D5" s="32"/>
-      <c r="E5" s="33"/>
-      <c r="F5" t="s" s="35">
+      <c r="C5" t="s" s="32">
         <v>15</v>
       </c>
+      <c r="D5" s="33"/>
+      <c r="E5" s="34"/>
+      <c r="F5" s="35"/>
       <c r="G5" s="36"/>
       <c r="H5" s="37"/>
     </row>
@@ -1850,12 +1850,12 @@
         <v>16</v>
       </c>
       <c r="B6" s="39"/>
-      <c r="C6" t="s" s="41">
+      <c r="C6" s="40"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="42"/>
+      <c r="F6" t="s" s="44">
         <v>17</v>
       </c>
-      <c r="D6" s="42"/>
-      <c r="E6" s="43"/>
-      <c r="F6" s="44"/>
       <c r="G6" s="45"/>
       <c r="H6" s="46"/>
     </row>
@@ -1866,10 +1866,10 @@
       <c r="B7" s="48"/>
       <c r="C7" s="49"/>
       <c r="D7" s="50"/>
-      <c r="E7" t="s" s="52">
+      <c r="E7" s="51"/>
+      <c r="F7" t="s" s="53">
         <v>19</v>
       </c>
-      <c r="F7" s="53"/>
       <c r="G7" s="54"/>
       <c r="H7" s="55"/>
     </row>
@@ -1878,78 +1878,78 @@
         <v>20</v>
       </c>
       <c r="B8" s="57"/>
-      <c r="C8" s="58"/>
-      <c r="D8" s="59"/>
-      <c r="E8" s="60"/>
-      <c r="F8" t="s" s="62">
+      <c r="C8" t="s" s="59">
         <v>21</v>
       </c>
-      <c r="G8" s="63"/>
-      <c r="H8" s="64"/>
+      <c r="D8" s="60"/>
+      <c r="E8" s="61"/>
+      <c r="F8" t="s" s="63">
+        <v>22</v>
+      </c>
+      <c r="G8" s="64"/>
+      <c r="H8" s="65"/>
     </row>
     <row r="9" ht="40.0" customHeight="true">
-      <c r="A9" t="s" s="65">
-        <v>22</v>
-      </c>
-      <c r="B9" s="66"/>
-      <c r="C9" t="s" s="68">
+      <c r="A9" t="s" s="66">
         <v>23</v>
       </c>
-      <c r="D9" s="69"/>
-      <c r="E9" s="70"/>
-      <c r="F9" t="s" s="72">
+      <c r="B9" s="67"/>
+      <c r="C9" t="s" s="69">
         <v>24</v>
       </c>
-      <c r="G9" s="73"/>
-      <c r="H9" s="74"/>
+      <c r="D9" s="70"/>
+      <c r="E9" t="s" s="72">
+        <v>25</v>
+      </c>
+      <c r="F9" s="73"/>
+      <c r="G9" s="74"/>
+      <c r="H9" s="75"/>
     </row>
     <row r="10" ht="40.0" customHeight="true">
-      <c r="A10" t="s" s="75">
-        <v>25</v>
-      </c>
-      <c r="B10" s="76"/>
-      <c r="C10" t="s" s="78">
+      <c r="A10" t="s" s="76">
         <v>26</v>
       </c>
-      <c r="D10" s="79"/>
-      <c r="E10" t="s" s="81">
+      <c r="B10" t="s" s="78">
         <v>27</v>
       </c>
-      <c r="F10" s="82"/>
-      <c r="G10" s="83"/>
-      <c r="H10" s="84"/>
+      <c r="C10" s="79"/>
+      <c r="D10" s="80"/>
+      <c r="E10" t="s" s="82">
+        <v>28</v>
+      </c>
+      <c r="F10" s="83"/>
+      <c r="G10" s="84"/>
+      <c r="H10" s="85"/>
     </row>
     <row r="11" ht="40.0" customHeight="true">
-      <c r="A11" t="s" s="85">
-        <v>28</v>
-      </c>
-      <c r="B11" t="s" s="87">
+      <c r="A11" t="s" s="86">
         <v>29</v>
       </c>
+      <c r="B11" s="87"/>
       <c r="C11" s="88"/>
-      <c r="D11" s="89"/>
-      <c r="E11" t="s" s="91">
+      <c r="D11" t="s" s="90">
         <v>30</v>
       </c>
-      <c r="F11" s="92"/>
-      <c r="G11" s="93"/>
-      <c r="H11" s="94"/>
+      <c r="E11" t="s" s="92">
+        <v>31</v>
+      </c>
+      <c r="F11" t="s" s="94">
+        <v>32</v>
+      </c>
+      <c r="G11" s="95"/>
+      <c r="H11" s="96"/>
     </row>
     <row r="12" ht="40.0" customHeight="true">
-      <c r="A12" t="s" s="95">
-        <v>31</v>
-      </c>
-      <c r="B12" s="96"/>
-      <c r="C12" s="97"/>
-      <c r="D12" t="s" s="99">
-        <v>32</v>
-      </c>
-      <c r="E12" t="s" s="101">
+      <c r="A12" t="s" s="97">
         <v>33</v>
       </c>
-      <c r="F12" t="s" s="103">
+      <c r="B12" s="98"/>
+      <c r="C12" s="99"/>
+      <c r="D12" t="s" s="101">
         <v>34</v>
       </c>
+      <c r="E12" s="102"/>
+      <c r="F12" s="103"/>
       <c r="G12" s="104"/>
       <c r="H12" s="105"/>
     </row>
@@ -1959,60 +1959,60 @@
       </c>
       <c r="B13" s="107"/>
       <c r="C13" s="108"/>
-      <c r="D13" t="s" s="110">
+      <c r="D13" s="109"/>
+      <c r="E13" t="s" s="111">
         <v>36</v>
       </c>
-      <c r="E13" s="111"/>
-      <c r="F13" s="112"/>
-      <c r="G13" s="113"/>
-      <c r="H13" s="114"/>
+      <c r="F13" t="s" s="113">
+        <v>37</v>
+      </c>
+      <c r="G13" s="114"/>
+      <c r="H13" s="115"/>
     </row>
     <row r="14" ht="40.0" customHeight="true">
-      <c r="A14" t="s" s="115">
-        <v>37</v>
-      </c>
-      <c r="B14" s="116"/>
-      <c r="C14" s="117"/>
-      <c r="D14" s="118"/>
-      <c r="E14" t="s" s="120">
+      <c r="A14" t="s" s="116">
         <v>38</v>
       </c>
-      <c r="F14" t="s" s="122">
+      <c r="B14" s="117"/>
+      <c r="C14" t="s" s="119">
         <v>39</v>
       </c>
-      <c r="G14" s="123"/>
-      <c r="H14" s="124"/>
+      <c r="D14" t="s" s="121">
+        <v>40</v>
+      </c>
+      <c r="E14" s="122"/>
+      <c r="F14" t="s" s="124">
+        <v>41</v>
+      </c>
+      <c r="G14" s="125"/>
+      <c r="H14" s="126"/>
     </row>
     <row r="15" ht="40.0" customHeight="true">
-      <c r="A15" t="s" s="125">
-        <v>40</v>
-      </c>
-      <c r="B15" s="126"/>
-      <c r="C15" t="s" s="128">
-        <v>41</v>
-      </c>
-      <c r="D15" t="s" s="130">
+      <c r="A15" t="s" s="127">
         <v>42</v>
       </c>
-      <c r="E15" s="131"/>
-      <c r="F15" t="s" s="133">
+      <c r="B15" s="128"/>
+      <c r="C15" s="129"/>
+      <c r="D15" t="s" s="131">
         <v>43</v>
       </c>
-      <c r="G15" s="134"/>
-      <c r="H15" s="135"/>
+      <c r="E15" t="s" s="133">
+        <v>44</v>
+      </c>
+      <c r="F15" s="134"/>
+      <c r="G15" s="135"/>
+      <c r="H15" s="136"/>
     </row>
     <row r="16" ht="40.0" customHeight="true">
-      <c r="A16" t="s" s="136">
-        <v>44</v>
-      </c>
-      <c r="B16" s="137"/>
-      <c r="C16" s="138"/>
-      <c r="D16" t="s" s="140">
+      <c r="A16" t="s" s="137">
         <v>45</v>
       </c>
-      <c r="E16" t="s" s="142">
+      <c r="B16" s="138"/>
+      <c r="C16" s="139"/>
+      <c r="D16" t="s" s="141">
         <v>46</v>
       </c>
+      <c r="E16" s="142"/>
       <c r="F16" s="143"/>
       <c r="G16" s="144"/>
       <c r="H16" s="145"/>
@@ -2023,10 +2023,10 @@
       </c>
       <c r="B17" s="147"/>
       <c r="C17" s="148"/>
-      <c r="D17" t="s" s="150">
+      <c r="D17" s="149"/>
+      <c r="E17" t="s" s="151">
         <v>48</v>
       </c>
-      <c r="E17" s="151"/>
       <c r="F17" s="152"/>
       <c r="G17" s="153"/>
       <c r="H17" s="154"/>
@@ -2036,11 +2036,11 @@
         <v>49</v>
       </c>
       <c r="B18" s="156"/>
-      <c r="C18" s="157"/>
-      <c r="D18" s="158"/>
-      <c r="E18" t="s" s="160">
+      <c r="C18" t="s" s="158">
         <v>50</v>
       </c>
+      <c r="D18" s="159"/>
+      <c r="E18" s="160"/>
       <c r="F18" s="161"/>
       <c r="G18" s="162"/>
       <c r="H18" s="163"/>
@@ -2054,26 +2054,26 @@
         <v>52</v>
       </c>
       <c r="D19" s="168"/>
-      <c r="E19" s="169"/>
-      <c r="F19" s="170"/>
-      <c r="G19" s="171"/>
-      <c r="H19" s="172"/>
+      <c r="E19" t="s" s="170">
+        <v>53</v>
+      </c>
+      <c r="F19" t="s" s="172">
+        <v>54</v>
+      </c>
+      <c r="G19" s="173"/>
+      <c r="H19" s="174"/>
     </row>
     <row r="20" ht="40.0" customHeight="true">
-      <c r="A20" t="s" s="173">
-        <v>53</v>
-      </c>
-      <c r="B20" s="174"/>
-      <c r="C20" t="s" s="176">
-        <v>54</v>
-      </c>
-      <c r="D20" s="177"/>
-      <c r="E20" t="s" s="179">
+      <c r="A20" t="s" s="175">
         <v>55</v>
       </c>
-      <c r="F20" t="s" s="181">
+      <c r="B20" s="176"/>
+      <c r="C20" t="s" s="178">
         <v>56</v>
       </c>
+      <c r="D20" s="179"/>
+      <c r="E20" s="180"/>
+      <c r="F20" s="181"/>
       <c r="G20" s="182"/>
       <c r="H20" s="183"/>
     </row>
@@ -2082,45 +2082,45 @@
         <v>57</v>
       </c>
       <c r="B21" s="185"/>
-      <c r="C21" t="s" s="187">
+      <c r="C21" s="186"/>
+      <c r="D21" s="187"/>
+      <c r="E21" t="s" s="189">
         <v>58</v>
       </c>
-      <c r="D21" s="188"/>
-      <c r="E21" s="189"/>
-      <c r="F21" s="190"/>
-      <c r="G21" s="191"/>
-      <c r="H21" s="192"/>
+      <c r="F21" t="s" s="191">
+        <v>59</v>
+      </c>
+      <c r="G21" s="192"/>
+      <c r="H21" s="193"/>
     </row>
     <row r="22" ht="40.0" customHeight="true">
-      <c r="A22" t="s" s="193">
-        <v>59</v>
-      </c>
-      <c r="B22" s="194"/>
-      <c r="C22" s="195"/>
-      <c r="D22" s="196"/>
-      <c r="E22" t="s" s="198">
+      <c r="A22" t="s" s="194">
         <v>60</v>
       </c>
-      <c r="F22" t="s" s="200">
+      <c r="B22" s="195"/>
+      <c r="C22" t="s" s="197">
         <v>61</v>
       </c>
-      <c r="G22" s="201"/>
-      <c r="H22" s="202"/>
+      <c r="D22" s="198"/>
+      <c r="E22" s="199"/>
+      <c r="F22" s="200"/>
+      <c r="G22" t="s" s="202">
+        <v>62</v>
+      </c>
+      <c r="H22" s="203"/>
     </row>
     <row r="23" ht="40.0" customHeight="true">
-      <c r="A23" t="s" s="203">
-        <v>62</v>
-      </c>
-      <c r="B23" s="204"/>
-      <c r="C23" t="s" s="206">
+      <c r="A23" t="s" s="204">
         <v>63</v>
       </c>
+      <c r="B23" s="205"/>
+      <c r="C23" s="206"/>
       <c r="D23" s="207"/>
       <c r="E23" s="208"/>
-      <c r="F23" s="209"/>
-      <c r="G23" t="s" s="211">
+      <c r="F23" t="s" s="210">
         <v>64</v>
       </c>
+      <c r="G23" s="211"/>
       <c r="H23" s="212"/>
     </row>
     <row r="24" ht="40.0" customHeight="true">
@@ -2129,52 +2129,52 @@
       </c>
       <c r="B24" s="214"/>
       <c r="C24" s="215"/>
-      <c r="D24" s="216"/>
-      <c r="E24" s="217"/>
-      <c r="F24" t="s" s="219">
+      <c r="D24" t="s" s="217">
         <v>66</v>
       </c>
-      <c r="G24" s="220"/>
-      <c r="H24" s="221"/>
+      <c r="E24" t="s" s="219">
+        <v>67</v>
+      </c>
+      <c r="F24" s="220"/>
+      <c r="G24" s="221"/>
+      <c r="H24" s="222"/>
     </row>
     <row r="25" ht="40.0" customHeight="true">
-      <c r="A25" t="s" s="222">
-        <v>67</v>
-      </c>
-      <c r="B25" s="223"/>
-      <c r="C25" s="224"/>
-      <c r="D25" t="s" s="226">
+      <c r="A25" t="s" s="223">
         <v>68</v>
       </c>
+      <c r="B25" s="224"/>
+      <c r="C25" s="225"/>
+      <c r="D25" s="226"/>
       <c r="E25" t="s" s="228">
         <v>69</v>
       </c>
       <c r="F25" s="229"/>
-      <c r="G25" s="230"/>
-      <c r="H25" s="231"/>
+      <c r="G25" t="s" s="231">
+        <v>70</v>
+      </c>
+      <c r="H25" s="232"/>
     </row>
     <row r="26" ht="40.0" customHeight="true">
-      <c r="A26" t="s" s="232">
-        <v>70</v>
-      </c>
-      <c r="B26" s="233"/>
-      <c r="C26" s="234"/>
-      <c r="D26" s="235"/>
-      <c r="E26" s="236"/>
-      <c r="F26" s="237"/>
-      <c r="G26" t="s" s="239">
+      <c r="A26" t="s" s="233">
         <v>71</v>
       </c>
-      <c r="H26" s="240"/>
+      <c r="B26" s="234"/>
+      <c r="C26" t="s" s="236">
+        <v>72</v>
+      </c>
+      <c r="D26" s="237"/>
+      <c r="E26" s="238"/>
+      <c r="F26" s="239"/>
+      <c r="G26" s="240"/>
+      <c r="H26" s="241"/>
     </row>
     <row r="27" ht="40.0" customHeight="true">
-      <c r="A27" t="s" s="241">
-        <v>72</v>
-      </c>
-      <c r="B27" s="242"/>
-      <c r="C27" t="s" s="244">
+      <c r="A27" t="s" s="242">
         <v>73</v>
       </c>
+      <c r="B27" s="243"/>
+      <c r="C27" s="244"/>
       <c r="D27" s="245"/>
       <c r="E27" s="246"/>
       <c r="F27" s="247"/>

</xml_diff>

<commit_message>
Doku und small fixed
</commit_message>
<xml_diff>
--- a/Turnierplanung.xlsx
+++ b/Turnierplanung.xlsx
@@ -38,25 +38,32 @@
     <t>U13</t>
   </si>
   <si>
+    <t>KW 36
+2026-09-05</t>
+  </si>
+  <si>
+    <t>Heidenheim - QB_U17_3 (QB)</t>
+  </si>
+  <si>
     <t>KW 37
 2026-09-12</t>
   </si>
   <si>
-    <t>Heidenheim - QB_U17_3 (QB)</t>
+    <t>Leverkusen - QB_SEN_1 (QB)</t>
   </si>
   <si>
     <t>KW 38
 2026-09-19</t>
   </si>
   <si>
-    <t>Leverkusen - QB_SEN_1 (QB)</t>
+    <t>Leipzig - QB_U17_4 (QB)</t>
   </si>
   <si>
     <t>KW 39
 2026-09-26</t>
   </si>
   <si>
-    <t>Leipzig - QB_U17_4 (QB)</t>
+    <t>Solingen - QB_U17_5 (QB)</t>
   </si>
   <si>
     <t>KW 40
@@ -70,7 +77,7 @@
 2026-10-10</t>
   </si>
   <si>
-    <t>Solingen - QB_U17_5 (QB)</t>
+    <t>Heidelberg - QB_U20_7 (QB)</t>
   </si>
   <si>
     <t>KW 42
@@ -221,7 +228,7 @@
     <t>FIE - FIE_Heidenheim (FIE)</t>
   </si>
   <si>
-    <t>Osnabrück - CHALLENGE_U15_11 (CHALLENGE)</t>
+    <t>Waldkirch - CHALLENGE_U15_10 (CHALLENGE)</t>
   </si>
   <si>
     <t>KW 6
@@ -245,10 +252,7 @@
 2027-02-27</t>
   </si>
   <si>
-    <t>Heidelberg - QB_U20_7 (QB)</t>
-  </si>
-  <si>
-    <t>Frankfurt - CHALLENGE_U15_9 (CHALLENGE)</t>
+    <t>Osnabrück - CHALLENGE_U15_11 (CHALLENGE)</t>
   </si>
   <si>
     <t>KW 10
@@ -259,11 +263,7 @@
 EFC - EFC_Differdange (EFC)</t>
   </si>
   <si>
-    <t>KW 11
-2027-03-20</t>
-  </si>
-  <si>
-    <t>Waldkirch - CHALLENGE_U15_10 (CHALLENGE)</t>
+    <t>Frankfurt - CHALLENGE_U15_9 (CHALLENGE)</t>
   </si>
   <si>
     <t>KW 12
@@ -274,6 +274,9 @@
 EFC - EFC_Daugavpils (EFC)</t>
   </si>
   <si>
+    <t>Bonn - CHALLENGE_U15_8 (CHALLENGE)</t>
+  </si>
+  <si>
     <t>KW 13
 2027-04-03</t>
   </si>
@@ -303,9 +306,6 @@
   </si>
   <si>
     <t>EFC - EFC_EM_U20 (EFC)</t>
-  </si>
-  <si>
-    <t>Bonn - CHALLENGE_U15_8 (CHALLENGE)</t>
   </si>
   <si>
     <t>KW 17
@@ -814,10 +814,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -832,10 +832,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -871,13 +868,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -892,19 +889,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -925,22 +922,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -964,10 +958,16 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -985,19 +985,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1012,19 +1009,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1045,22 +1039,25 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1084,7 +1081,10 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1105,13 +1105,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1129,16 +1129,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1156,25 +1156,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1189,19 +1183,25 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1216,22 +1216,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1246,22 +1243,22 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1276,19 +1273,22 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1306,19 +1306,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1336,16 +1333,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1363,10 +1360,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1390,7 +1387,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1438,6 +1438,9 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
     <xf numFmtId="0" fontId="29" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
@@ -1538,9 +1541,6 @@
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1836,12 +1836,12 @@
         <v>14</v>
       </c>
       <c r="B5" s="30"/>
-      <c r="C5" t="s" s="32">
+      <c r="C5" s="31"/>
+      <c r="D5" s="32"/>
+      <c r="E5" s="33"/>
+      <c r="F5" t="s" s="35">
         <v>15</v>
       </c>
-      <c r="D5" s="33"/>
-      <c r="E5" s="34"/>
-      <c r="F5" s="35"/>
       <c r="G5" s="36"/>
       <c r="H5" s="37"/>
     </row>
@@ -1850,12 +1850,12 @@
         <v>16</v>
       </c>
       <c r="B6" s="39"/>
-      <c r="C6" s="40"/>
-      <c r="D6" s="41"/>
-      <c r="E6" s="42"/>
-      <c r="F6" t="s" s="44">
+      <c r="C6" t="s" s="41">
         <v>17</v>
       </c>
+      <c r="D6" s="42"/>
+      <c r="E6" s="43"/>
+      <c r="F6" s="44"/>
       <c r="G6" s="45"/>
       <c r="H6" s="46"/>
     </row>
@@ -1866,10 +1866,10 @@
       <c r="B7" s="48"/>
       <c r="C7" s="49"/>
       <c r="D7" s="50"/>
-      <c r="E7" s="51"/>
-      <c r="F7" t="s" s="53">
+      <c r="E7" t="s" s="52">
         <v>19</v>
       </c>
+      <c r="F7" s="53"/>
       <c r="G7" s="54"/>
       <c r="H7" s="55"/>
     </row>
@@ -1878,78 +1878,78 @@
         <v>20</v>
       </c>
       <c r="B8" s="57"/>
-      <c r="C8" t="s" s="59">
+      <c r="C8" s="58"/>
+      <c r="D8" s="59"/>
+      <c r="E8" s="60"/>
+      <c r="F8" t="s" s="62">
         <v>21</v>
       </c>
-      <c r="D8" s="60"/>
-      <c r="E8" s="61"/>
-      <c r="F8" t="s" s="63">
+      <c r="G8" s="63"/>
+      <c r="H8" s="64"/>
+    </row>
+    <row r="9" ht="40.0" customHeight="true">
+      <c r="A9" t="s" s="65">
         <v>22</v>
       </c>
-      <c r="G8" s="64"/>
-      <c r="H8" s="65"/>
-    </row>
-    <row r="9" ht="40.0" customHeight="true">
-      <c r="A9" t="s" s="66">
+      <c r="B9" s="66"/>
+      <c r="C9" t="s" s="68">
         <v>23</v>
       </c>
-      <c r="B9" s="67"/>
-      <c r="C9" t="s" s="69">
+      <c r="D9" s="69"/>
+      <c r="E9" s="70"/>
+      <c r="F9" t="s" s="72">
         <v>24</v>
       </c>
-      <c r="D9" s="70"/>
-      <c r="E9" t="s" s="72">
+      <c r="G9" s="73"/>
+      <c r="H9" s="74"/>
+    </row>
+    <row r="10" ht="40.0" customHeight="true">
+      <c r="A10" t="s" s="75">
         <v>25</v>
       </c>
-      <c r="F9" s="73"/>
-      <c r="G9" s="74"/>
-      <c r="H9" s="75"/>
-    </row>
-    <row r="10" ht="40.0" customHeight="true">
-      <c r="A10" t="s" s="76">
+      <c r="B10" s="76"/>
+      <c r="C10" t="s" s="78">
         <v>26</v>
       </c>
-      <c r="B10" t="s" s="78">
+      <c r="D10" s="79"/>
+      <c r="E10" t="s" s="81">
         <v>27</v>
       </c>
-      <c r="C10" s="79"/>
-      <c r="D10" s="80"/>
-      <c r="E10" t="s" s="82">
+      <c r="F10" s="82"/>
+      <c r="G10" s="83"/>
+      <c r="H10" s="84"/>
+    </row>
+    <row r="11" ht="40.0" customHeight="true">
+      <c r="A11" t="s" s="85">
         <v>28</v>
       </c>
-      <c r="F10" s="83"/>
-      <c r="G10" s="84"/>
-      <c r="H10" s="85"/>
-    </row>
-    <row r="11" ht="40.0" customHeight="true">
-      <c r="A11" t="s" s="86">
+      <c r="B11" t="s" s="87">
         <v>29</v>
       </c>
-      <c r="B11" s="87"/>
       <c r="C11" s="88"/>
-      <c r="D11" t="s" s="90">
+      <c r="D11" s="89"/>
+      <c r="E11" t="s" s="91">
         <v>30</v>
       </c>
-      <c r="E11" t="s" s="92">
+      <c r="F11" s="92"/>
+      <c r="G11" s="93"/>
+      <c r="H11" s="94"/>
+    </row>
+    <row r="12" ht="40.0" customHeight="true">
+      <c r="A12" t="s" s="95">
         <v>31</v>
       </c>
-      <c r="F11" t="s" s="94">
+      <c r="B12" s="96"/>
+      <c r="C12" s="97"/>
+      <c r="D12" t="s" s="99">
         <v>32</v>
       </c>
-      <c r="G11" s="95"/>
-      <c r="H11" s="96"/>
-    </row>
-    <row r="12" ht="40.0" customHeight="true">
-      <c r="A12" t="s" s="97">
+      <c r="E12" t="s" s="101">
         <v>33</v>
       </c>
-      <c r="B12" s="98"/>
-      <c r="C12" s="99"/>
-      <c r="D12" t="s" s="101">
+      <c r="F12" t="s" s="103">
         <v>34</v>
       </c>
-      <c r="E12" s="102"/>
-      <c r="F12" s="103"/>
       <c r="G12" s="104"/>
       <c r="H12" s="105"/>
     </row>
@@ -1959,60 +1959,60 @@
       </c>
       <c r="B13" s="107"/>
       <c r="C13" s="108"/>
-      <c r="D13" s="109"/>
-      <c r="E13" t="s" s="111">
+      <c r="D13" t="s" s="110">
         <v>36</v>
       </c>
-      <c r="F13" t="s" s="113">
+      <c r="E13" s="111"/>
+      <c r="F13" s="112"/>
+      <c r="G13" s="113"/>
+      <c r="H13" s="114"/>
+    </row>
+    <row r="14" ht="40.0" customHeight="true">
+      <c r="A14" t="s" s="115">
         <v>37</v>
       </c>
-      <c r="G13" s="114"/>
-      <c r="H13" s="115"/>
-    </row>
-    <row r="14" ht="40.0" customHeight="true">
-      <c r="A14" t="s" s="116">
+      <c r="B14" s="116"/>
+      <c r="C14" s="117"/>
+      <c r="D14" s="118"/>
+      <c r="E14" t="s" s="120">
         <v>38</v>
       </c>
-      <c r="B14" s="117"/>
-      <c r="C14" t="s" s="119">
+      <c r="F14" t="s" s="122">
         <v>39</v>
       </c>
-      <c r="D14" t="s" s="121">
+      <c r="G14" s="123"/>
+      <c r="H14" s="124"/>
+    </row>
+    <row r="15" ht="40.0" customHeight="true">
+      <c r="A15" t="s" s="125">
         <v>40</v>
       </c>
-      <c r="E14" s="122"/>
-      <c r="F14" t="s" s="124">
+      <c r="B15" s="126"/>
+      <c r="C15" t="s" s="128">
         <v>41</v>
       </c>
-      <c r="G14" s="125"/>
-      <c r="H14" s="126"/>
-    </row>
-    <row r="15" ht="40.0" customHeight="true">
-      <c r="A15" t="s" s="127">
+      <c r="D15" t="s" s="130">
         <v>42</v>
       </c>
-      <c r="B15" s="128"/>
-      <c r="C15" s="129"/>
-      <c r="D15" t="s" s="131">
+      <c r="E15" s="131"/>
+      <c r="F15" t="s" s="133">
         <v>43</v>
       </c>
-      <c r="E15" t="s" s="133">
+      <c r="G15" s="134"/>
+      <c r="H15" s="135"/>
+    </row>
+    <row r="16" ht="40.0" customHeight="true">
+      <c r="A16" t="s" s="136">
         <v>44</v>
       </c>
-      <c r="F15" s="134"/>
-      <c r="G15" s="135"/>
-      <c r="H15" s="136"/>
-    </row>
-    <row r="16" ht="40.0" customHeight="true">
-      <c r="A16" t="s" s="137">
+      <c r="B16" s="137"/>
+      <c r="C16" s="138"/>
+      <c r="D16" t="s" s="140">
         <v>45</v>
       </c>
-      <c r="B16" s="138"/>
-      <c r="C16" s="139"/>
-      <c r="D16" t="s" s="141">
+      <c r="E16" t="s" s="142">
         <v>46</v>
       </c>
-      <c r="E16" s="142"/>
       <c r="F16" s="143"/>
       <c r="G16" s="144"/>
       <c r="H16" s="145"/>
@@ -2023,10 +2023,10 @@
       </c>
       <c r="B17" s="147"/>
       <c r="C17" s="148"/>
-      <c r="D17" s="149"/>
-      <c r="E17" t="s" s="151">
+      <c r="D17" t="s" s="150">
         <v>48</v>
       </c>
+      <c r="E17" s="151"/>
       <c r="F17" s="152"/>
       <c r="G17" s="153"/>
       <c r="H17" s="154"/>
@@ -2036,11 +2036,11 @@
         <v>49</v>
       </c>
       <c r="B18" s="156"/>
-      <c r="C18" t="s" s="158">
+      <c r="C18" s="157"/>
+      <c r="D18" s="158"/>
+      <c r="E18" t="s" s="160">
         <v>50</v>
       </c>
-      <c r="D18" s="159"/>
-      <c r="E18" s="160"/>
       <c r="F18" s="161"/>
       <c r="G18" s="162"/>
       <c r="H18" s="163"/>
@@ -2054,26 +2054,26 @@
         <v>52</v>
       </c>
       <c r="D19" s="168"/>
-      <c r="E19" t="s" s="170">
+      <c r="E19" s="169"/>
+      <c r="F19" s="170"/>
+      <c r="G19" s="171"/>
+      <c r="H19" s="172"/>
+    </row>
+    <row r="20" ht="40.0" customHeight="true">
+      <c r="A20" t="s" s="173">
         <v>53</v>
       </c>
-      <c r="F19" t="s" s="172">
+      <c r="B20" s="174"/>
+      <c r="C20" t="s" s="176">
         <v>54</v>
       </c>
-      <c r="G19" s="173"/>
-      <c r="H19" s="174"/>
-    </row>
-    <row r="20" ht="40.0" customHeight="true">
-      <c r="A20" t="s" s="175">
+      <c r="D20" s="177"/>
+      <c r="E20" t="s" s="179">
         <v>55</v>
       </c>
-      <c r="B20" s="176"/>
-      <c r="C20" t="s" s="178">
+      <c r="F20" t="s" s="181">
         <v>56</v>
       </c>
-      <c r="D20" s="179"/>
-      <c r="E20" s="180"/>
-      <c r="F20" s="181"/>
       <c r="G20" s="182"/>
       <c r="H20" s="183"/>
     </row>
@@ -2082,45 +2082,45 @@
         <v>57</v>
       </c>
       <c r="B21" s="185"/>
-      <c r="C21" s="186"/>
-      <c r="D21" s="187"/>
-      <c r="E21" t="s" s="189">
+      <c r="C21" t="s" s="187">
         <v>58</v>
       </c>
-      <c r="F21" t="s" s="191">
+      <c r="D21" s="188"/>
+      <c r="E21" s="189"/>
+      <c r="F21" s="190"/>
+      <c r="G21" s="191"/>
+      <c r="H21" s="192"/>
+    </row>
+    <row r="22" ht="40.0" customHeight="true">
+      <c r="A22" t="s" s="193">
         <v>59</v>
       </c>
-      <c r="G21" s="192"/>
-      <c r="H21" s="193"/>
-    </row>
-    <row r="22" ht="40.0" customHeight="true">
-      <c r="A22" t="s" s="194">
+      <c r="B22" s="194"/>
+      <c r="C22" s="195"/>
+      <c r="D22" s="196"/>
+      <c r="E22" t="s" s="198">
         <v>60</v>
       </c>
-      <c r="B22" s="195"/>
-      <c r="C22" t="s" s="197">
+      <c r="F22" t="s" s="200">
         <v>61</v>
       </c>
-      <c r="D22" s="198"/>
-      <c r="E22" s="199"/>
-      <c r="F22" s="200"/>
-      <c r="G22" t="s" s="202">
+      <c r="G22" s="201"/>
+      <c r="H22" s="202"/>
+    </row>
+    <row r="23" ht="40.0" customHeight="true">
+      <c r="A23" t="s" s="203">
         <v>62</v>
       </c>
-      <c r="H22" s="203"/>
-    </row>
-    <row r="23" ht="40.0" customHeight="true">
-      <c r="A23" t="s" s="204">
+      <c r="B23" s="204"/>
+      <c r="C23" t="s" s="206">
         <v>63</v>
       </c>
-      <c r="B23" s="205"/>
-      <c r="C23" s="206"/>
       <c r="D23" s="207"/>
       <c r="E23" s="208"/>
-      <c r="F23" t="s" s="210">
+      <c r="F23" s="209"/>
+      <c r="G23" t="s" s="211">
         <v>64</v>
       </c>
-      <c r="G23" s="211"/>
       <c r="H23" s="212"/>
     </row>
     <row r="24" ht="40.0" customHeight="true">
@@ -2129,52 +2129,52 @@
       </c>
       <c r="B24" s="214"/>
       <c r="C24" s="215"/>
-      <c r="D24" t="s" s="217">
+      <c r="D24" s="216"/>
+      <c r="E24" s="217"/>
+      <c r="F24" t="s" s="219">
         <v>66</v>
       </c>
-      <c r="E24" t="s" s="219">
+      <c r="G24" s="220"/>
+      <c r="H24" s="221"/>
+    </row>
+    <row r="25" ht="40.0" customHeight="true">
+      <c r="A25" t="s" s="222">
         <v>67</v>
       </c>
-      <c r="F24" s="220"/>
-      <c r="G24" s="221"/>
-      <c r="H24" s="222"/>
-    </row>
-    <row r="25" ht="40.0" customHeight="true">
-      <c r="A25" t="s" s="223">
+      <c r="B25" s="223"/>
+      <c r="C25" s="224"/>
+      <c r="D25" t="s" s="226">
         <v>68</v>
       </c>
-      <c r="B25" s="224"/>
-      <c r="C25" s="225"/>
-      <c r="D25" s="226"/>
       <c r="E25" t="s" s="228">
         <v>69</v>
       </c>
       <c r="F25" s="229"/>
-      <c r="G25" t="s" s="231">
+      <c r="G25" s="230"/>
+      <c r="H25" s="231"/>
+    </row>
+    <row r="26" ht="40.0" customHeight="true">
+      <c r="A26" t="s" s="232">
         <v>70</v>
       </c>
-      <c r="H25" s="232"/>
-    </row>
-    <row r="26" ht="40.0" customHeight="true">
-      <c r="A26" t="s" s="233">
+      <c r="B26" s="233"/>
+      <c r="C26" s="234"/>
+      <c r="D26" s="235"/>
+      <c r="E26" s="236"/>
+      <c r="F26" s="237"/>
+      <c r="G26" t="s" s="239">
         <v>71</v>
       </c>
-      <c r="B26" s="234"/>
-      <c r="C26" t="s" s="236">
+      <c r="H26" s="240"/>
+    </row>
+    <row r="27" ht="40.0" customHeight="true">
+      <c r="A27" t="s" s="241">
         <v>72</v>
       </c>
-      <c r="D26" s="237"/>
-      <c r="E26" s="238"/>
-      <c r="F26" s="239"/>
-      <c r="G26" s="240"/>
-      <c r="H26" s="241"/>
-    </row>
-    <row r="27" ht="40.0" customHeight="true">
-      <c r="A27" t="s" s="242">
+      <c r="B27" s="242"/>
+      <c r="C27" t="s" s="244">
         <v>73</v>
       </c>
-      <c r="B27" s="243"/>
-      <c r="C27" s="244"/>
       <c r="D27" s="245"/>
       <c r="E27" s="246"/>
       <c r="F27" s="247"/>
@@ -2194,67 +2194,67 @@
       <c r="D28" s="255"/>
       <c r="E28" s="256"/>
       <c r="F28" s="257"/>
-      <c r="G28" s="258"/>
-      <c r="H28" s="259"/>
+      <c r="G28" t="s" s="259">
+        <v>77</v>
+      </c>
+      <c r="H28" s="260"/>
     </row>
     <row r="29" ht="40.0" customHeight="true">
-      <c r="A29" t="s" s="260">
-        <v>77</v>
-      </c>
-      <c r="B29" s="261"/>
-      <c r="C29" s="262"/>
-      <c r="D29" s="263"/>
-      <c r="E29" t="s" s="265">
+      <c r="A29" t="s" s="261">
         <v>78</v>
       </c>
-      <c r="F29" s="266"/>
-      <c r="G29" t="s" s="268">
+      <c r="B29" s="262"/>
+      <c r="C29" s="263"/>
+      <c r="D29" s="264"/>
+      <c r="E29" t="s" s="266">
         <v>79</v>
       </c>
-      <c r="H29" s="269"/>
+      <c r="F29" s="267"/>
+      <c r="G29" t="s" s="269">
+        <v>80</v>
+      </c>
+      <c r="H29" s="270"/>
     </row>
     <row r="30" ht="40.0" customHeight="true">
-      <c r="A30" t="s" s="270">
-        <v>80</v>
-      </c>
-      <c r="B30" s="271"/>
-      <c r="C30" s="272"/>
-      <c r="D30" s="273"/>
-      <c r="E30" t="s" s="275">
+      <c r="A30" t="s" s="271">
         <v>81</v>
       </c>
-      <c r="F30" s="276"/>
-      <c r="G30" s="277"/>
-      <c r="H30" s="278"/>
+      <c r="B30" s="272"/>
+      <c r="C30" s="273"/>
+      <c r="D30" s="274"/>
+      <c r="E30" t="s" s="276">
+        <v>82</v>
+      </c>
+      <c r="F30" s="277"/>
+      <c r="G30" s="278"/>
+      <c r="H30" s="279"/>
     </row>
     <row r="31" ht="40.0" customHeight="true">
-      <c r="A31" t="s" s="279">
-        <v>82</v>
-      </c>
-      <c r="B31" s="280"/>
-      <c r="C31" t="s" s="282">
+      <c r="A31" t="s" s="280">
         <v>83</v>
       </c>
-      <c r="D31" s="283"/>
-      <c r="E31" s="284"/>
-      <c r="F31" s="285"/>
-      <c r="G31" s="286"/>
-      <c r="H31" s="287"/>
+      <c r="B31" s="281"/>
+      <c r="C31" t="s" s="283">
+        <v>84</v>
+      </c>
+      <c r="D31" s="284"/>
+      <c r="E31" s="285"/>
+      <c r="F31" s="286"/>
+      <c r="G31" s="287"/>
+      <c r="H31" s="288"/>
     </row>
     <row r="32" ht="40.0" customHeight="true">
-      <c r="A32" t="s" s="288">
-        <v>84</v>
-      </c>
-      <c r="B32" s="289"/>
-      <c r="C32" s="290"/>
-      <c r="D32" s="291"/>
-      <c r="E32" t="s" s="293">
+      <c r="A32" t="s" s="289">
         <v>85</v>
       </c>
-      <c r="F32" s="294"/>
-      <c r="G32" t="s" s="296">
+      <c r="B32" s="290"/>
+      <c r="C32" s="291"/>
+      <c r="D32" s="292"/>
+      <c r="E32" t="s" s="294">
         <v>86</v>
       </c>
+      <c r="F32" s="295"/>
+      <c r="G32" s="296"/>
       <c r="H32" s="297"/>
     </row>
     <row r="33" ht="40.0" customHeight="true">

</xml_diff>

<commit_message>
Update der eVersionen von Java und Time
</commit_message>
<xml_diff>
--- a/Turnierplanung.xlsx
+++ b/Turnierplanung.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="103">
   <si>
     <t>Wochenende (KW)</t>
   </si>
@@ -77,7 +77,7 @@
 2026-10-10</t>
   </si>
   <si>
-    <t>Heidelberg - QB_U20_7 (QB)</t>
+    <t>Offenbach - QB_U20_6 (QB)</t>
   </si>
   <si>
     <t>KW 42
@@ -114,7 +114,7 @@
     <t>Erfurt - DM_VET_12 (DM)</t>
   </si>
   <si>
-    <t>Offenbach - QB_U20_6 (QB)</t>
+    <t>Heidelberg - QB_U20_7 (QB)</t>
   </si>
   <si>
     <t>KW 46
@@ -228,7 +228,7 @@
     <t>FIE - FIE_Heidenheim (FIE)</t>
   </si>
   <si>
-    <t>Waldkirch - CHALLENGE_U15_10 (CHALLENGE)</t>
+    <t>Frankfurt - CHALLENGE_U15_9 (CHALLENGE)</t>
   </si>
   <si>
     <t>KW 6
@@ -252,6 +252,13 @@
 2027-02-27</t>
   </si>
   <si>
+    <t>Waldkirch - CHALLENGE_U15_10 (CHALLENGE)</t>
+  </si>
+  <si>
+    <t>KW 9
+2027-03-06</t>
+  </si>
+  <si>
     <t>Osnabrück - CHALLENGE_U15_11 (CHALLENGE)</t>
   </si>
   <si>
@@ -261,9 +268,6 @@
   <si>
     <t>FIE - FIE_Budapest (FIE)
 EFC - EFC_Differdange (EFC)</t>
-  </si>
-  <si>
-    <t>Frankfurt - CHALLENGE_U15_9 (CHALLENGE)</t>
   </si>
   <si>
     <t>KW 12
@@ -366,7 +370,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="40">
+  <fonts count="41">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
@@ -379,6 +383,11 @@
       <sz val="11.0"/>
       <b val="true"/>
       <color indexed="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -659,7 +668,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="362">
+  <cellXfs count="370">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="true" applyFill="true" applyAlignment="true" applyBorder="true">
       <alignment horizontal="center" vertical="center"/>
@@ -1387,10 +1396,7 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1438,19 +1444,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
     <xf numFmtId="0" fontId="29" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1483,10 +1486,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1504,16 +1510,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1531,16 +1537,16 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1564,13 +1570,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1588,10 +1591,13 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1642,10 +1648,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1669,19 +1675,19 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1705,10 +1711,10 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
-      <alignment horizontal="left" vertical="top" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1718,6 +1724,33 @@
       <alignment horizontal="left" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="39" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
+      <alignment horizontal="center" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
+      <alignment horizontal="left" vertical="top" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="5" borderId="4" xfId="0" applyFont="true" applyAlignment="true" applyFill="true" applyBorder="true">
       <alignment horizontal="center" vertical="top" wrapText="true"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyAlignment="true" applyBorder="true" applyFill="true">
@@ -1750,7 +1783,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H40"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="25.0" customWidth="true"/>
@@ -2172,190 +2205,202 @@
         <v>72</v>
       </c>
       <c r="B27" s="242"/>
-      <c r="C27" t="s" s="244">
+      <c r="C27" s="243"/>
+      <c r="D27" s="244"/>
+      <c r="E27" s="245"/>
+      <c r="F27" s="246"/>
+      <c r="G27" t="s" s="248">
         <v>73</v>
       </c>
-      <c r="D27" s="245"/>
-      <c r="E27" s="246"/>
-      <c r="F27" s="247"/>
-      <c r="G27" t="s" s="249">
+      <c r="H27" s="249"/>
+    </row>
+    <row r="28" ht="40.0" customHeight="true">
+      <c r="A28" t="s" s="250">
         <v>74</v>
       </c>
-      <c r="H27" s="250"/>
-    </row>
-    <row r="28" ht="40.0" customHeight="true">
-      <c r="A28" t="s" s="251">
+      <c r="B28" s="251"/>
+      <c r="C28" t="s" s="253">
         <v>75</v>
       </c>
-      <c r="B28" s="252"/>
-      <c r="C28" t="s" s="254">
+      <c r="D28" s="254"/>
+      <c r="E28" s="255"/>
+      <c r="F28" s="256"/>
+      <c r="G28" s="257"/>
+      <c r="H28" s="258"/>
+    </row>
+    <row r="29" ht="40.0" customHeight="true">
+      <c r="A29" t="s" s="259">
         <v>76</v>
       </c>
-      <c r="D28" s="255"/>
-      <c r="E28" s="256"/>
-      <c r="F28" s="257"/>
-      <c r="G28" t="s" s="259">
+      <c r="B29" s="260"/>
+      <c r="C29" t="s" s="262">
         <v>77</v>
       </c>
-      <c r="H28" s="260"/>
-    </row>
-    <row r="29" ht="40.0" customHeight="true">
-      <c r="A29" t="s" s="261">
+      <c r="D29" s="263"/>
+      <c r="E29" s="264"/>
+      <c r="F29" s="265"/>
+      <c r="G29" t="s" s="267">
         <v>78</v>
       </c>
-      <c r="B29" s="262"/>
-      <c r="C29" s="263"/>
-      <c r="D29" s="264"/>
-      <c r="E29" t="s" s="266">
+      <c r="H29" s="268"/>
+    </row>
+    <row r="30" ht="40.0" customHeight="true">
+      <c r="A30" t="s" s="269">
         <v>79</v>
       </c>
-      <c r="F29" s="267"/>
-      <c r="G29" t="s" s="269">
+      <c r="B30" s="270"/>
+      <c r="C30" s="271"/>
+      <c r="D30" s="272"/>
+      <c r="E30" t="s" s="274">
         <v>80</v>
       </c>
-      <c r="H29" s="270"/>
-    </row>
-    <row r="30" ht="40.0" customHeight="true">
-      <c r="A30" t="s" s="271">
+      <c r="F30" s="275"/>
+      <c r="G30" t="s" s="277">
         <v>81</v>
       </c>
-      <c r="B30" s="272"/>
-      <c r="C30" s="273"/>
-      <c r="D30" s="274"/>
-      <c r="E30" t="s" s="276">
+      <c r="H30" s="278"/>
+    </row>
+    <row r="31" ht="40.0" customHeight="true">
+      <c r="A31" t="s" s="279">
         <v>82</v>
       </c>
-      <c r="F30" s="277"/>
-      <c r="G30" s="278"/>
-      <c r="H30" s="279"/>
-    </row>
-    <row r="31" ht="40.0" customHeight="true">
-      <c r="A31" t="s" s="280">
+      <c r="B31" s="280"/>
+      <c r="C31" s="281"/>
+      <c r="D31" s="282"/>
+      <c r="E31" t="s" s="284">
         <v>83</v>
       </c>
-      <c r="B31" s="281"/>
-      <c r="C31" t="s" s="283">
+      <c r="F31" s="285"/>
+      <c r="G31" s="286"/>
+      <c r="H31" s="287"/>
+    </row>
+    <row r="32" ht="40.0" customHeight="true">
+      <c r="A32" t="s" s="288">
         <v>84</v>
       </c>
-      <c r="D31" s="284"/>
-      <c r="E31" s="285"/>
-      <c r="F31" s="286"/>
-      <c r="G31" s="287"/>
-      <c r="H31" s="288"/>
-    </row>
-    <row r="32" ht="40.0" customHeight="true">
-      <c r="A32" t="s" s="289">
+      <c r="B32" s="289"/>
+      <c r="C32" t="s" s="291">
         <v>85</v>
       </c>
-      <c r="B32" s="290"/>
-      <c r="C32" s="291"/>
       <c r="D32" s="292"/>
-      <c r="E32" t="s" s="294">
+      <c r="E32" s="293"/>
+      <c r="F32" s="294"/>
+      <c r="G32" s="295"/>
+      <c r="H32" s="296"/>
+    </row>
+    <row r="33" ht="40.0" customHeight="true">
+      <c r="A33" t="s" s="297">
         <v>86</v>
       </c>
-      <c r="F32" s="295"/>
-      <c r="G32" s="296"/>
-      <c r="H32" s="297"/>
-    </row>
-    <row r="33" ht="40.0" customHeight="true">
-      <c r="A33" t="s" s="298">
+      <c r="B33" s="298"/>
+      <c r="C33" s="299"/>
+      <c r="D33" s="300"/>
+      <c r="E33" t="s" s="302">
         <v>87</v>
       </c>
-      <c r="B33" s="299"/>
-      <c r="C33" s="300"/>
-      <c r="D33" s="301"/>
-      <c r="E33" s="302"/>
-      <c r="F33" t="s" s="304">
+      <c r="F33" s="303"/>
+      <c r="G33" s="304"/>
+      <c r="H33" s="305"/>
+    </row>
+    <row r="34" ht="40.0" customHeight="true">
+      <c r="A34" t="s" s="306">
         <v>88</v>
       </c>
-      <c r="G33" s="305"/>
-      <c r="H33" t="s" s="307">
+      <c r="B34" s="307"/>
+      <c r="C34" s="308"/>
+      <c r="D34" s="309"/>
+      <c r="E34" s="310"/>
+      <c r="F34" t="s" s="312">
         <v>89</v>
       </c>
-    </row>
-    <row r="34" ht="40.0" customHeight="true">
-      <c r="A34" t="s" s="308">
+      <c r="G34" s="313"/>
+      <c r="H34" t="s" s="315">
         <v>90</v>
       </c>
-      <c r="B34" s="309"/>
-      <c r="C34" t="s" s="311">
+    </row>
+    <row r="35" ht="40.0" customHeight="true">
+      <c r="A35" t="s" s="316">
         <v>91</v>
       </c>
-      <c r="D34" s="312"/>
-      <c r="E34" s="313"/>
-      <c r="F34" s="314"/>
-      <c r="G34" s="315"/>
-      <c r="H34" s="316"/>
-    </row>
-    <row r="35" ht="40.0" customHeight="true">
-      <c r="A35" t="s" s="317">
+      <c r="B35" s="317"/>
+      <c r="C35" t="s" s="319">
         <v>92</v>
       </c>
-      <c r="B35" s="318"/>
-      <c r="C35" t="s" s="320">
+      <c r="D35" s="320"/>
+      <c r="E35" s="321"/>
+      <c r="F35" s="322"/>
+      <c r="G35" s="323"/>
+      <c r="H35" s="324"/>
+    </row>
+    <row r="36" ht="40.0" customHeight="true">
+      <c r="A36" t="s" s="325">
         <v>93</v>
       </c>
-      <c r="D35" s="321"/>
-      <c r="E35" s="322"/>
-      <c r="F35" s="323"/>
-      <c r="G35" s="324"/>
-      <c r="H35" s="325"/>
-    </row>
-    <row r="36" ht="40.0" customHeight="true">
-      <c r="A36" t="s" s="326">
+      <c r="B36" s="326"/>
+      <c r="C36" t="s" s="328">
         <v>94</v>
       </c>
-      <c r="B36" s="327"/>
-      <c r="C36" t="s" s="329">
+      <c r="D36" s="329"/>
+      <c r="E36" s="330"/>
+      <c r="F36" s="331"/>
+      <c r="G36" s="332"/>
+      <c r="H36" s="333"/>
+    </row>
+    <row r="37" ht="40.0" customHeight="true">
+      <c r="A37" t="s" s="334">
         <v>95</v>
       </c>
-      <c r="D36" s="330"/>
-      <c r="E36" s="331"/>
-      <c r="F36" s="332"/>
-      <c r="G36" s="333"/>
-      <c r="H36" s="334"/>
-    </row>
-    <row r="37" ht="40.0" customHeight="true">
-      <c r="A37" t="s" s="335">
+      <c r="B37" s="335"/>
+      <c r="C37" t="s" s="337">
         <v>96</v>
       </c>
-      <c r="B37" s="336"/>
-      <c r="C37" s="337"/>
       <c r="D37" s="338"/>
       <c r="E37" s="339"/>
-      <c r="F37" t="s" s="341">
+      <c r="F37" s="340"/>
+      <c r="G37" s="341"/>
+      <c r="H37" s="342"/>
+    </row>
+    <row r="38" ht="40.0" customHeight="true">
+      <c r="A38" t="s" s="343">
         <v>97</v>
       </c>
-      <c r="G37" s="342"/>
-      <c r="H37" s="343"/>
-    </row>
-    <row r="38" ht="40.0" customHeight="true">
-      <c r="A38" t="s" s="344">
+      <c r="B38" s="344"/>
+      <c r="C38" s="345"/>
+      <c r="D38" s="346"/>
+      <c r="E38" s="347"/>
+      <c r="F38" t="s" s="349">
         <v>98</v>
       </c>
-      <c r="B38" s="345"/>
-      <c r="C38" t="s" s="347">
+      <c r="G38" s="350"/>
+      <c r="H38" s="351"/>
+    </row>
+    <row r="39" ht="40.0" customHeight="true">
+      <c r="A39" t="s" s="352">
         <v>99</v>
       </c>
-      <c r="D38" s="348"/>
-      <c r="E38" s="349"/>
-      <c r="F38" s="350"/>
-      <c r="G38" s="351"/>
-      <c r="H38" s="352"/>
-    </row>
-    <row r="39" ht="40.0" customHeight="true">
-      <c r="A39" t="s" s="353">
+      <c r="B39" s="353"/>
+      <c r="C39" t="s" s="355">
         <v>100</v>
       </c>
-      <c r="B39" s="354"/>
-      <c r="C39" t="s" s="356">
+      <c r="D39" s="356"/>
+      <c r="E39" s="357"/>
+      <c r="F39" s="358"/>
+      <c r="G39" s="359"/>
+      <c r="H39" s="360"/>
+    </row>
+    <row r="40" ht="40.0" customHeight="true">
+      <c r="A40" t="s" s="361">
         <v>101</v>
       </c>
-      <c r="D39" s="357"/>
-      <c r="E39" s="358"/>
-      <c r="F39" s="359"/>
-      <c r="G39" s="360"/>
-      <c r="H39" s="361"/>
+      <c r="B40" s="362"/>
+      <c r="C40" t="s" s="364">
+        <v>102</v>
+      </c>
+      <c r="D40" s="365"/>
+      <c r="E40" s="366"/>
+      <c r="F40" s="367"/>
+      <c r="G40" s="368"/>
+      <c r="H40" s="369"/>
     </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>

</xml_diff>